<commit_message>
Clarify XM38 A/B/C emergency blade applies to Toyota/Lexus shell
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KaJs6Wdeh5fe4LTTDbYhia
</commit_message>
<xml_diff>
--- a/Xhorse_키날_비상키_목록.xlsx
+++ b/Xhorse_키날_비상키_목록.xlsx
@@ -5743,7 +5743,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>XM38 (공통)</t>
+          <t>XSTO01EN (XM38 토요타·렉서스 쉘)</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -5754,7 +5754,7 @@
       <c r="C56" s="2" t="n"/>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>XM38 쉘용 비상키 (A/B/C 타입)</t>
+          <t>XM38 토요타·렉서스형 쉘 전용 비상키 (A/B/C 타입, 판매처 사진 기준)</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -5872,7 +5872,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -5983,29 +5983,41 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>판매처 설명: 키날 미포함, "universal flip remote key blades" 구매 안내. Honrow에서 XM38 쉘용 비상키(A/B/C 타입) 별도 판매</t>
+          <t>판매처 설명: 키날 미포함, "universal flip remote key blades" 구매 안내</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>XSTO01EN (토요타·렉서스)</t>
+          <t>Honrow A/B/C 비상키</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>쉘 모양별로 토요타·렉서스 TOY48 스마트키 비상키가 지정됨</t>
+          <t>판매처 사진상 XM38 토요타·렉서스형 쉘(XSTO01EN)용. XM38 범용 쉘용 아님</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
+          <t>XSTO01EN (토요타·렉서스)</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>쉘 모양별로 토요타·렉서스 TOY48 스마트키 비상키가 지정됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
           <t>MLB 기판 (아우디·포르쉐)</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>아우디·포르쉐 HU162 스마트키 비상키가 지정됨</t>
         </is>

</xml_diff>

<commit_message>
Rename generation labels, add newly found chip info, single-line rows
Chip labels now name the model a new version replaces instead of
'2nd generation'. Adds XEDS21EN XT57B, XSMQB4EN chip list, XZ vehicle
coverage, XSDM04EN/XSTO01EN blade info, and turns off cell wrapping.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KaJs6Wdeh5fe4LTTDbYhia
</commit_message>
<xml_diff>
--- a/Xhorse_키날_비상키_목록.xlsx
+++ b/Xhorse_키날_비상키_목록.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'공용 키날 (키웨이별)'!$A$1:$K$93</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'공용 키날 (전체 상품)'!$A$1:$L$442</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'키날 세트·롤핀·부속'!$A$1:$H$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'XS 비상키 (전체 모델)'!$A$1:$K$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'XS 비상키 (전체 모델)'!$A$1:$K$66</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -95,20 +95,20 @@
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top"/>
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -24524,7 +24524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K65"/>
+  <dimension ref="A1:K66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -24932,25 +24932,25 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>전용 스마트키 비상키</t>
+          <t>공용 스마트키 키날 (Keyshop Online 안내)</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>XM38 스마트키용 비상키 (insert)</t>
+          <t>KEYDIY TOY40 / TOY48 S-S (#165)</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Universal Smart Key Insert for Xhorse Universal Smart Key (XM38)</t>
+          <t>Keydiy Xhorse Universal Smart Remote Key Blade TOY2 / TOY40 / TOY48 S-S Toyota Lexus (#165)</t>
         </is>
       </c>
       <c r="H8" s="3" t="n">
-        <v>3.99</v>
+        <v>1</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Royal Key Supply</t>
+          <t>Keyshop Online</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -24960,19 +24960,19 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Royal Key Supply 설명: "Universal smart key insert for Xhorse (XSTO01EN) XM38"</t>
+          <t>Keyshop Online XSTO01EN 설명: "comes without an emergency key … any universal blade will fit. If you want to use this remote for Toyota, please buy this emergency blade: … TOY40 / TOY48 S/S (#165)"</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>XSBM90GL</t>
+          <t>XSTO01EN</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>BMW</t>
+          <t>Toyota</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -24987,33 +24987,47 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>키날 포함 (BW9MH)</t>
+          <t>전용 스마트키 비상키</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>포함</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="n"/>
-      <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="2" t="inlineStr"/>
+          <t>XM38 스마트키용 비상키 (insert)</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Universal Smart Key Insert for Xhorse Universal Smart Key (XM38)</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Royal Key Supply</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>ABKEYS: 같은 제품 XSBMM0GL "Key Blade: Included"</t>
+          <t>Royal Key Supply 설명: "Universal smart key insert for Xhorse (XSTO01EN) XM38"</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>XSDFX1EN</t>
+          <t>XSBM90GL</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Knife</t>
+          <t>BMW</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -25023,17 +25037,17 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>공용 폴딩 키날 (차에 맞는 키웨이 선택)</t>
+          <t>키날 포함 (BW9MH)</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>공용 키날 시트 참고</t>
+          <t>포함</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -25042,19 +25056,19 @@
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>가격표 공용 키날 O</t>
+          <t>ABKEYS: 같은 제품 XSBMM0GL "Key Blade: Included"</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>XSDM04EN</t>
+          <t>XSDFX1EN</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>MQB</t>
+          <t>Knife</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -25090,12 +25104,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>XSKF01EN</t>
+          <t>XSDM04EN</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>BMW</t>
+          <t>MQB</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -25110,47 +25124,33 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>공용 폴딩 키날 (차에 맞는 키웨이 선택)</t>
+          <t>공용 폴딩 키날 (HU66)</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>키웨이 HU92</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>KeyDiy Xhorse Remote Key Blade For Bmw HU92</t>
-        </is>
-      </c>
-      <c r="H12" s="3" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS</t>
-        </is>
-      </c>
-      <c r="J12" s="4" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+          <t>키웨이 HU66 (폴딩 키날, 미포함)</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>ABKEYS 스마트키 상세의 "Key Blade: Optional" 지정 상품</t>
+          <t>xhorseshop.eu: "Blade: Flip HU66 profile blade (Not included)" → 공용 키날 시트의 HU66</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>XSKFF1EN</t>
+          <t>XSKF01EN</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Knife</t>
+          <t>BMW</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -25170,16 +25170,16 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>키웨이 HU66 (Long)</t>
+          <t>키웨이 HU92</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Volkswagen Flip Remote Long Key Blade, HU66</t>
+          <t>KeyDiy Xhorse Remote Key Blade For Bmw HU92</t>
         </is>
       </c>
       <c r="H13" s="3" t="n">
-        <v>1.15</v>
+        <v>0.65</v>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
@@ -25200,12 +25200,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>XSMQB1EN</t>
+          <t>XSKFF1EN</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>MQB</t>
+          <t>Knife</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -25255,7 +25255,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>XSMQB4EN</t>
+          <t>XSMQB1EN</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -25280,28 +25280,42 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>공용 키날 시트 참고</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr"/>
-      <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="inlineStr"/>
-      <c r="J15" s="2" t="inlineStr"/>
+          <t>키웨이 HU66 (Long)</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Volkswagen Flip Remote Long Key Blade, HU66</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>ABKEYS</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>xhorseshop.eu: "MQB type XSMQB4EN Flip type 3 buttons smart key"</t>
+          <t>ABKEYS 스마트키 상세의 "Key Blade: Optional" 지정 상품</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>XSSC01EN</t>
+          <t>XSMQB4EN</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Supercar</t>
+          <t>MQB</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -25316,7 +25330,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>공용 폴딩 키날 사용 (판매처 설명: "universal flip remote key blades")</t>
+          <t>공용 폴딩 키날 (차에 맞는 키웨이 선택)</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -25328,12 +25342,16 @@
       <c r="H16" s="2" t="n"/>
       <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="inlineStr"/>
-      <c r="K16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>xhorseshop.eu: "MQB type XSMQB4EN Flip type 3 buttons smart key"</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>XSSC04EN</t>
+          <t>XSSC01EN</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -25370,7 +25388,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>XSSC05EN</t>
+          <t>XSSC04EN</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -25407,7 +25425,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>XSSC21EN</t>
+          <t>XSSC05EN</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -25427,7 +25445,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>공용 폴딩 키날 (차에 맞는 키웨이 선택)</t>
+          <t>공용 폴딩 키날 사용 (판매처 설명: "universal flip remote key blades")</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -25439,16 +25457,12 @@
       <c r="H19" s="2" t="n"/>
       <c r="I19" s="2" t="inlineStr"/>
       <c r="J19" s="2" t="inlineStr"/>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>가격표 공용 키날 O</t>
-        </is>
-      </c>
+      <c r="K19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>XSSC25EN</t>
+          <t>XSSC21EN</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -25489,12 +25503,12 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>XSBEZ2EN</t>
+          <t>XSSC25EN</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Benz</t>
+          <t>Supercar</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -25504,17 +25518,17 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>판매처 정보 없음 (확인 필요)</t>
+          <t>공용 폴딩 키날 (차에 맞는 키웨이 선택)</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>판매처 미기재</t>
+          <t>공용 키날 시트 참고</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr"/>
@@ -25523,19 +25537,19 @@
       <c r="J21" s="2" t="inlineStr"/>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>판매처에서 비상키 정보를 찾지 못했어요 (벤츠 스타일 XM38 신제품, 확인 필요). [근거] OBDII365·VVDIshop·xhorseshop.eu 설명에 키날 언급 없음</t>
+          <t>가격표 공용 키날 O</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>XSCH01EN</t>
+          <t>XSBEZ2EN</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Chrysler</t>
+          <t>Benz</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -25545,52 +25559,38 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>공용 폴딩 키날 (차에 맞는 키웨이 선택)</t>
+          <t>판매처 정보 없음 (확인 필요)</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>키웨이 CY22</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>KeyDiy Xhorse Remote Key Blade For Jeep CY22</t>
-        </is>
-      </c>
-      <c r="H22" s="3" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS</t>
-        </is>
-      </c>
-      <c r="J22" s="4" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+          <t>판매처 미기재</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="n"/>
+      <c r="I22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr"/>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>ABKEYS 스마트키 상세의 "Key Blade: Optional" 지정 상품</t>
+          <t>판매처에서 비상키 정보를 찾지 못했어요 (벤츠 스타일 XM38 신제품, 확인 필요). [근거] OBDII365·VVDIshop·xhorseshop.eu 설명에 키날 언급 없음</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>XSCL01EN</t>
+          <t>XSCH01EN</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Chevrolet</t>
+          <t>Chrysler</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -25610,19 +25610,37 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>key4: universal flip remote key blades 구매 안내</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr"/>
-      <c r="H23" s="2" t="n"/>
-      <c r="I23" s="2" t="inlineStr"/>
-      <c r="J23" s="2" t="inlineStr"/>
-      <c r="K23" s="2" t="inlineStr"/>
+          <t>키웨이 CY22</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>KeyDiy Xhorse Remote Key Blade For Jeep CY22</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>ABKEYS</t>
+        </is>
+      </c>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>ABKEYS 스마트키 상세의 "Key Blade: Optional" 지정 상품</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>XSCLN1EN</t>
+          <t>XSCL01EN</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -25647,28 +25665,24 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>공용 키날 시트 참고</t>
+          <t>key4: universal flip remote key blades 구매 안내</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr"/>
       <c r="H24" s="2" t="n"/>
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="inlineStr"/>
-      <c r="K24" s="2" t="inlineStr">
-        <is>
-          <t>가격표 공용 키날 O</t>
-        </is>
-      </c>
+      <c r="K24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>XSCS00EN</t>
+          <t>XSCLN1EN</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Hyundai</t>
+          <t>Chevrolet</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -25688,42 +25702,28 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>키웨이 HU66 (Long)</t>
-        </is>
-      </c>
-      <c r="G25" s="2" t="inlineStr">
-        <is>
-          <t>Volkswagen Flip Remote Long Key Blade, HU66</t>
-        </is>
-      </c>
-      <c r="H25" s="3" t="n">
-        <v>1.15</v>
-      </c>
-      <c r="I25" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS</t>
-        </is>
-      </c>
-      <c r="J25" s="4" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+          <t>공용 키날 시트 참고</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="n"/>
+      <c r="I25" s="2" t="inlineStr"/>
+      <c r="J25" s="2" t="inlineStr"/>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>ABKEYS 스마트키 상세의 "Key Blade: Optional" 지정 상품</t>
+          <t>가격표 공용 키날 O</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>XSDFX2EN</t>
+          <t>XSCS00EN</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Knife</t>
+          <t>Hyundai</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -25743,24 +25743,42 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>나이프(폴딩) 스타일, 키날 미포함 (UHS·Locksmith Keyless)</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="inlineStr"/>
-      <c r="H26" s="2" t="n"/>
-      <c r="I26" s="2" t="inlineStr"/>
-      <c r="J26" s="2" t="inlineStr"/>
-      <c r="K26" s="2" t="inlineStr"/>
+          <t>키웨이 HU66 (Long)</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Volkswagen Flip Remote Long Key Blade, HU66</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>ABKEYS</t>
+        </is>
+      </c>
+      <c r="J26" s="4" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>ABKEYS 스마트키 상세의 "Key Blade: Optional" 지정 상품</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>XSFO02EN</t>
+          <t>XSDFX2EN</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Ford</t>
+          <t>Knife</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -25775,12 +25793,12 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>공용 폴딩 키날 사용 (판매처 설명: "universal flip remote key blades")</t>
+          <t>공용 폴딩 키날 (차에 맞는 키웨이 선택)</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>공용 키날 시트 참고</t>
+          <t>나이프(폴딩) 스타일, 키날 미포함 (UHS·Locksmith Keyless)</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr"/>
@@ -25792,12 +25810,12 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>XSGA80EN</t>
+          <t>XSFO02EN</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>VW</t>
+          <t>Ford</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -25829,12 +25847,12 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>XSKA85EN</t>
+          <t>XSGA80EN</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Kia EV</t>
+          <t>VW</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -25844,33 +25862,29 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>판매처 정보 없음 (확인 필요)</t>
+          <t>공용 폴딩 키날 사용 (판매처 설명: "universal flip remote key blades")</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>판매처 미기재</t>
+          <t>공용 키날 시트 참고</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr"/>
       <c r="H29" s="2" t="n"/>
       <c r="I29" s="2" t="inlineStr"/>
       <c r="J29" s="2" t="inlineStr"/>
-      <c r="K29" s="2" t="inlineStr">
-        <is>
-          <t>판매처에서 비상키 정보를 찾지 못했어요 (기아 EV 스타일 XM38 신제품, 확인 필요). [근거] OBDII365·VVDIshop·xhorseshop.eu 설명에 키날 언급 없음</t>
-        </is>
-      </c>
+      <c r="K29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>XSKA86EN</t>
+          <t>XSKA85EN</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -25911,12 +25925,12 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>XSKC04EN</t>
+          <t>XSKA86EN</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>King Card</t>
+          <t>Kia EV</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -25931,24 +25945,28 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>키날 없음 (카드형)</t>
+          <t>판매처 정보 없음 (확인 필요)</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>해당 없음</t>
+          <t>판매처 미기재</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr"/>
       <c r="H31" s="2" t="n"/>
       <c r="I31" s="2" t="inlineStr"/>
       <c r="J31" s="2" t="inlineStr"/>
-      <c r="K31" s="2" t="inlineStr"/>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>판매처에서 비상키 정보를 찾지 못했어요 (기아 EV 스타일 XM38 신제품, 확인 필요). [근거] OBDII365·VVDIshop·xhorseshop.eu 설명에 키날 언급 없음</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>XSKC05EN</t>
+          <t>XSKC04EN</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -25985,12 +26003,12 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>XSKF20EN</t>
+          <t>XSKC05EN</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>BMW</t>
+          <t>King Card</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -26000,47 +26018,29 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>공용 폴딩 키날 (차에 맞는 키웨이 선택)</t>
+          <t>키날 없음 (카드형)</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>키웨이 HU66 (Long)</t>
-        </is>
-      </c>
-      <c r="G33" s="2" t="inlineStr">
-        <is>
-          <t>Volkswagen Flip Remote Long Key Blade, HU66</t>
-        </is>
-      </c>
-      <c r="H33" s="3" t="n">
-        <v>1.15</v>
-      </c>
-      <c r="I33" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS</t>
-        </is>
-      </c>
-      <c r="J33" s="4" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
-      <c r="K33" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS 스마트키 상세의 "Key Blade: Optional" 지정 상품</t>
-        </is>
-      </c>
+          <t>해당 없음</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr"/>
+      <c r="H33" s="2" t="n"/>
+      <c r="I33" s="2" t="inlineStr"/>
+      <c r="J33" s="2" t="inlineStr"/>
+      <c r="K33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>XSKF21EN</t>
+          <t>XSKF20EN</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -26095,12 +26095,12 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>XSKF30EN</t>
+          <t>XSKF21EN</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Knife</t>
+          <t>BMW</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -26150,7 +26150,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>XSKF31EN</t>
+          <t>XSKF30EN</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -26175,23 +26175,37 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>공용 키날 시트 참고</t>
-        </is>
-      </c>
-      <c r="G36" s="2" t="inlineStr"/>
-      <c r="H36" s="2" t="n"/>
-      <c r="I36" s="2" t="inlineStr"/>
-      <c r="J36" s="2" t="inlineStr"/>
+          <t>키웨이 HU66 (Long)</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Volkswagen Flip Remote Long Key Blade, HU66</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>ABKEYS</t>
+        </is>
+      </c>
+      <c r="J36" s="4" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>가격표 공용 키날 O</t>
+          <t>ABKEYS 스마트키 상세의 "Key Blade: Optional" 지정 상품</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>XSKFF0EN</t>
+          <t>XSKF31EN</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -26216,24 +26230,28 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>3버튼 버전 XSKFF1EN과 같은 방식 (Best Key Supply: 키날 별도 장착)</t>
+          <t>공용 키날 시트 참고</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr"/>
       <c r="H37" s="2" t="n"/>
       <c r="I37" s="2" t="inlineStr"/>
       <c r="J37" s="2" t="inlineStr"/>
-      <c r="K37" s="2" t="inlineStr"/>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>가격표 공용 키날 O</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>XSMS01EN</t>
+          <t>XSKFF0EN</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Maserati</t>
+          <t>Knife</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -26243,38 +26261,34 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>판매처 정보 없음 (확인 필요)</t>
+          <t>공용 폴딩 키날 (차에 맞는 키웨이 선택)</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>판매처 미기재</t>
+          <t>3버튼 버전 XSKFF1EN과 같은 방식 (Best Key Supply: 키날 별도 장착)</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr"/>
       <c r="H38" s="2" t="n"/>
       <c r="I38" s="2" t="inlineStr"/>
       <c r="J38" s="2" t="inlineStr"/>
-      <c r="K38" s="2" t="inlineStr">
-        <is>
-          <t>판매처에서 비상키 정보를 찾지 못했어요 (마세라티 스타일 XM38 신제품, 확인 필요). [근거] OBDII365·VVDIshop·xhorseshop.eu 설명에 키날 언급 없음</t>
-        </is>
-      </c>
+      <c r="K38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>XSNIS2EN</t>
+          <t>XSMS01EN</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Nissan</t>
+          <t>Maserati</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -26289,47 +26303,33 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>전용 스마트키 비상키</t>
+          <t>판매처 정보 없음 (확인 필요)</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>키웨이 NSN14</t>
-        </is>
-      </c>
-      <c r="G39" s="2" t="inlineStr">
-        <is>
-          <t>Nissan 2007-2025 Smart Key Blade H0564-EG010, NSN14</t>
-        </is>
-      </c>
-      <c r="H39" s="3" t="n">
-        <v>1.95</v>
-      </c>
-      <c r="I39" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS</t>
-        </is>
-      </c>
-      <c r="J39" s="4" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+          <t>판매처 미기재</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr"/>
+      <c r="H39" s="2" t="n"/>
+      <c r="I39" s="2" t="inlineStr"/>
+      <c r="J39" s="2" t="inlineStr"/>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>ABKEYS 스마트키 상세의 "Key Blade: Optional" 지정 상품</t>
+          <t>판매처에서 비상키 정보를 찾지 못했어요 (마세라티 스타일 XM38 신제품, 확인 필요). [근거] OBDII365·VVDIshop·xhorseshop.eu 설명에 키날 언급 없음</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>XSPS01EN</t>
+          <t>XSNIS2EN</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Porsche</t>
+          <t>Nissan</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -26339,34 +26339,52 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>공용 폴딩 키날 사용 (판매처 설명: "universal flip remote key blades")</t>
+          <t>전용 스마트키 비상키</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>공용 키날 시트 참고</t>
-        </is>
-      </c>
-      <c r="G40" s="2" t="inlineStr"/>
-      <c r="H40" s="2" t="n"/>
-      <c r="I40" s="2" t="inlineStr"/>
-      <c r="J40" s="2" t="inlineStr"/>
-      <c r="K40" s="2" t="inlineStr"/>
+          <t>키웨이 NSN14</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Nissan 2007-2025 Smart Key Blade H0564-EG010, NSN14</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>ABKEYS</t>
+        </is>
+      </c>
+      <c r="J40" s="4" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>ABKEYS 스마트키 상세의 "Key Blade: Optional" 지정 상품</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>XSSBR0EN</t>
+          <t>XSPS01EN</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Subaru</t>
+          <t>Porsche</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -26398,12 +26416,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>XSTO03EN</t>
+          <t>XSSBR0EN</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Toyota</t>
+          <t>Subaru</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -26413,17 +26431,17 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>확인 필요 (판매처 간 상충)</t>
+          <t>공용 폴딩 키날 사용 (판매처 설명: "universal flip remote key blades")</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>key4는 공용 폴딩 키날 안내 / 같은 토요타형 XSTO01EN은 TOY48 전용 비상키</t>
+          <t>공용 키날 시트 참고</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr"/>
@@ -26435,12 +26453,12 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>XSCD01EN</t>
+          <t>XSTO03EN</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Cadillac</t>
+          <t>Toyota</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -26450,17 +26468,17 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>공용 폴딩 키날 사용 (판매처 설명: "universal flip remote key blades")</t>
+          <t>확인 필요 (판매처 간 상충)</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>공용 키날 시트 참고</t>
+          <t>key4는 공용 폴딩 키날 안내 / 같은 토요타형 XSTO01EN은 TOY48 전용 비상키</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr"/>
@@ -26472,12 +26490,12 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>XSJP01EN</t>
+          <t>XSCD01EN</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Jeep</t>
+          <t>Cadillac</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -26487,17 +26505,17 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>키날 포함 (CY22)</t>
+          <t>공용 폴딩 키날 사용 (판매처 설명: "universal flip remote key blades")</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>포함</t>
+          <t>공용 키날 시트 참고</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr"/>
@@ -26509,12 +26527,12 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>XSLR01EN</t>
+          <t>XSJP01EN</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Rover</t>
+          <t>Jeep</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -26529,42 +26547,24 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>전용 스마트키 비상키</t>
+          <t>키날 포함 (CY22)</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>키웨이 HU101</t>
-        </is>
-      </c>
-      <c r="G45" s="2" t="inlineStr">
-        <is>
-          <t>Range Rover, Land Rover 2010+ Smart Key Blade, HU101</t>
-        </is>
-      </c>
-      <c r="H45" s="3" t="n">
-        <v>2.65</v>
-      </c>
-      <c r="I45" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS</t>
-        </is>
-      </c>
-      <c r="J45" s="4" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
-      <c r="K45" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS 스마트키 상세의 "Key Blade: Optional" 지정 상품</t>
-        </is>
-      </c>
+          <t>포함</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr"/>
+      <c r="H45" s="2" t="n"/>
+      <c r="I45" s="2" t="inlineStr"/>
+      <c r="J45" s="2" t="inlineStr"/>
+      <c r="K45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>XSLR03EN</t>
+          <t>XSLR01EN</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -26584,34 +26584,52 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>확인 필요</t>
+          <t>전용 스마트키 비상키</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>다른 판매처도 정보 없음. 같은 랜드로버형 XSLR01EN은 HU101 전용 비상키</t>
-        </is>
-      </c>
-      <c r="G46" s="2" t="inlineStr"/>
-      <c r="H46" s="2" t="n"/>
-      <c r="I46" s="2" t="inlineStr"/>
-      <c r="J46" s="2" t="inlineStr"/>
-      <c r="K46" s="2" t="inlineStr"/>
+          <t>키웨이 HU101</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Range Rover, Land Rover 2010+ Smart Key Blade, HU101</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>ABKEYS</t>
+        </is>
+      </c>
+      <c r="J46" s="4" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>ABKEYS 스마트키 상세의 "Key Blade: Optional" 지정 상품</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>XSBTK0EN</t>
+          <t>XSLR03EN</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Bluetooth</t>
+          <t>Rover</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>블루투스 디지털 키</t>
+          <t>스마트키</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -26621,12 +26639,12 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>해당 없음</t>
+          <t>확인 필요</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>해당 없음</t>
+          <t>다른 판매처도 정보 없음. 같은 랜드로버형 XSLR01EN은 HU101 전용 비상키</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr"/>
@@ -26638,7 +26656,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>XSBTKOGL</t>
+          <t>XSBTK0EN</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -26670,26 +26688,22 @@
       <c r="H48" s="2" t="n"/>
       <c r="I48" s="2" t="inlineStr"/>
       <c r="J48" s="2" t="inlineStr"/>
-      <c r="K48" s="2" t="inlineStr">
-        <is>
-          <t>휴대폰 디지털키 (키날 자리 없음)</t>
-        </is>
-      </c>
+      <c r="K48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>XSWK02EN</t>
+          <t>XSBTKOGL</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Watch (SW-007)</t>
+          <t>Bluetooth</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>스마트워치형 키</t>
+          <t>블루투스 디지털 키</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -26711,12 +26725,16 @@
       <c r="H49" s="2" t="n"/>
       <c r="I49" s="2" t="inlineStr"/>
       <c r="J49" s="2" t="inlineStr"/>
-      <c r="K49" s="2" t="inlineStr"/>
+      <c r="K49" s="2" t="inlineStr">
+        <is>
+          <t>휴대폰 디지털키 (키날 자리 없음)</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>XSWK05EN</t>
+          <t>XSWK02EN</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -26753,17 +26771,17 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>XSTO00EN</t>
+          <t>XSWK05EN</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Toyota</t>
+          <t>Watch (SW-007)</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>스마트키 기판 (XS)</t>
+          <t>스마트워치형 키</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -26773,33 +26791,29 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>기판만 판매. 토요타 스마트키 쉘용 비상키 필요</t>
+          <t>해당 없음</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>판매처 지정 없음 (토요타 스마트키는 보통 TOY48)</t>
+          <t>해당 없음</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr"/>
       <c r="H51" s="2" t="n"/>
       <c r="I51" s="2" t="inlineStr"/>
       <c r="J51" s="2" t="inlineStr"/>
-      <c r="K51" s="2" t="inlineStr">
-        <is>
-          <t>UHS: "Smart Key PCB … TOY.T"</t>
-        </is>
-      </c>
+      <c r="K51" s="2" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>XSMA41EN</t>
+          <t>XSTO00EN</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Audi</t>
+          <t>Toyota</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -26814,42 +26828,28 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>전용 스마트키 비상키</t>
+          <t>기판만 판매. 토요타 스마트키 쉘용 비상키 필요</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>키웨이 HU162</t>
-        </is>
-      </c>
-      <c r="G52" s="2" t="inlineStr">
-        <is>
-          <t>Audi 2018-2024 Smart Key Blade, HU162</t>
-        </is>
-      </c>
-      <c r="H52" s="3" t="n">
-        <v>5.75</v>
-      </c>
-      <c r="I52" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS</t>
-        </is>
-      </c>
-      <c r="J52" s="4" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
+          <t>판매처 지정 없음 (토요타 스마트키는 보통 TOY48)</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr"/>
+      <c r="H52" s="2" t="n"/>
+      <c r="I52" s="2" t="inlineStr"/>
+      <c r="J52" s="2" t="inlineStr"/>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>ABKEYS 스마트키 상세의 "Key Blade: Optional" 지정 상품</t>
+          <t>UHS: "Smart Key PCB … TOY.T"</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>XSMA4YEN</t>
+          <t>XSMA41EN</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -26904,7 +26904,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>XSMA81EN</t>
+          <t>XSMA4YEN</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -26924,21 +26924,21 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>전용 스마트키 비상키 (추정)</t>
+          <t>전용 스마트키 비상키</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>HU162 아우디 스마트키 비상키</t>
+          <t>키웨이 HU162</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Audi 2022-2025 Smart Key Blade, HU162</t>
+          <t>Audi 2018-2024 Smart Key Blade, HU162</t>
         </is>
       </c>
       <c r="H54" s="3" t="n">
-        <v>8.99</v>
+        <v>5.75</v>
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
@@ -26952,14 +26952,14 @@
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>같은 아우디 A8 MLB 기판 XSMA8YEN에 ABKEYS가 지정한 비상키</t>
+          <t>ABKEYS 스마트키 상세의 "Key Blade: Optional" 지정 상품</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>XSMA8YEN</t>
+          <t>XSMA81EN</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -26979,12 +26979,12 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>전용 스마트키 비상키</t>
+          <t>전용 스마트키 비상키 (추정)</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>키웨이 HU162</t>
+          <t>HU162 아우디 스마트키 비상키</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -27007,19 +27007,19 @@
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>ABKEYS 스마트키 상세의 "Key Blade: Optional" 지정 상품</t>
+          <t>같은 아우디 A8 MLB 기판 XSMA8YEN에 ABKEYS가 지정한 비상키</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>XSMPS1EN</t>
+          <t>XSMA8YEN</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Porsche</t>
+          <t>Audi</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -27039,16 +27039,16 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>HU162 포르쉐 스마트키 비상키</t>
+          <t>키웨이 HU162</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Porsche 2018-2025 Smart Key Blade, HU162</t>
+          <t>Audi 2022-2025 Smart Key Blade, HU162</t>
         </is>
       </c>
       <c r="H56" s="3" t="n">
-        <v>3.25</v>
+        <v>8.99</v>
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
@@ -27062,14 +27062,14 @@
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>Keyshop Online "Test Key: HU162T", 같은 포르쉐 MLB 기판 XSMPSYEN에 ABKEYS가 지정한 비상키</t>
+          <t>ABKEYS 스마트키 상세의 "Key Blade: Optional" 지정 상품</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>XSMPSYEN</t>
+          <t>XSMPS1EN</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -27094,7 +27094,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>키웨이 HU162</t>
+          <t>HU162 포르쉐 스마트키 비상키</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -27117,19 +27117,19 @@
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
-          <t>ABKEYS 스마트키 상세의 "Key Blade: Optional" 지정 상품</t>
+          <t>Keyshop Online "Test Key: HU162T", 같은 포르쉐 MLB 기판 XSMPSYEN에 ABKEYS가 지정한 비상키</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>XSMTUYEN</t>
+          <t>XSMPSYEN</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Touareg</t>
+          <t>Porsche</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -27144,33 +27144,47 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>기판만 판매. 넣을 쉘에 맞는 비상키 필요</t>
+          <t>전용 스마트키 비상키</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>판매처 미기재</t>
-        </is>
-      </c>
-      <c r="G58" s="2" t="inlineStr"/>
-      <c r="H58" s="2" t="n"/>
-      <c r="I58" s="2" t="inlineStr"/>
-      <c r="J58" s="2" t="inlineStr"/>
+          <t>키웨이 HU162</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>Porsche 2018-2025 Smart Key Blade, HU162</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>ABKEYS</t>
+        </is>
+      </c>
+      <c r="J58" s="4" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>폭스바겐 투아렉 MLB 스마트키 기판만 파는 제품이에요. 비상키는 기판을 넣을 투아렉 쉘에 맞는 것을 써야 해요. [근거] OBDII365: "Toureg Style MLB Key PCB"</t>
+          <t>ABKEYS 스마트키 상세의 "Key Blade: Optional" 지정 상품</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>XSADJ1EN</t>
+          <t>XSMTUYEN</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Audi</t>
+          <t>Touareg</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -27185,24 +27199,28 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>기판만 판매. 아우디 순정형 쉘용 비상키 필요</t>
+          <t>기판만 판매. 넣을 쉘에 맞는 비상키 필요</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>UHS: Board only, Emergency Blade not included</t>
+          <t>판매처 미기재</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr"/>
       <c r="H59" s="2" t="n"/>
       <c r="I59" s="2" t="inlineStr"/>
       <c r="J59" s="2" t="inlineStr"/>
-      <c r="K59" s="2" t="inlineStr"/>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>폭스바겐 투아렉 MLB 스마트키 기판만 파는 제품이에요. 비상키는 기판을 넣을 투아렉 쉘에 맞는 것을 써야 해요. [근거] OBDII365: "Toureg Style MLB Key PCB"</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>XSADJ1GL</t>
+          <t>XSADJ1EN</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -27227,28 +27245,24 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>XSADJ1EN과 같음</t>
+          <t>UHS: Board only, Emergency Blade not included</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr"/>
       <c r="H60" s="2" t="n"/>
       <c r="I60" s="2" t="inlineStr"/>
       <c r="J60" s="2" t="inlineStr"/>
-      <c r="K60" s="2" t="inlineStr">
-        <is>
-          <t>UHS: XSADJ1EN "Board only", "Emergency Blade (not included)"</t>
-        </is>
-      </c>
+      <c r="K60" s="2" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>XSBMB1EN</t>
+          <t>XSADJ1GL</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Bread</t>
+          <t>Audi</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -27263,29 +27277,33 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>기판만 판매. 사용하는 쉘에 맞는 비상키 필요</t>
+          <t>기판만 판매. 아우디 순정형 쉘용 비상키 필요</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>판매처 미기재</t>
+          <t>XSADJ1EN과 같음</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr"/>
       <c r="H61" s="2" t="n"/>
       <c r="I61" s="2" t="inlineStr"/>
       <c r="J61" s="2" t="inlineStr"/>
-      <c r="K61" s="2" t="inlineStr"/>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>UHS: XSADJ1EN "Board only", "Emergency Blade (not included)"</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>XSBMU1EN</t>
+          <t>XSBMB1EN</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>Bread</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -27317,12 +27335,12 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>XSBZ01EN</t>
+          <t>XSBMU1EN</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Benz</t>
+          <t>U</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -27337,7 +27355,7 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>기판만 판매. 넣을 쉘에 맞는 비상키 필요</t>
+          <t>기판만 판매. 사용하는 쉘에 맞는 비상키 필요</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
@@ -27349,21 +27367,17 @@
       <c r="H63" s="2" t="n"/>
       <c r="I63" s="2" t="inlineStr"/>
       <c r="J63" s="2" t="inlineStr"/>
-      <c r="K63" s="2" t="inlineStr">
-        <is>
-          <t>벤츠 적외선(FBS3) 스마트키 기판만 파는 제품이에요. 비상키는 벤츠 쉘에 맞는 것을 써야 해요. [근거] key4: "Proximity Smart Key PCB for Mercedes IR Fobik Style FBS3"</t>
-        </is>
-      </c>
+      <c r="K63" s="2" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>XSTO20EN</t>
+          <t>XSBZ01EN</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Toyota</t>
+          <t>Benz</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -27378,12 +27392,12 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>비상키 포함</t>
+          <t>판매처마다 다름 (확인 필요)</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>포함</t>
+          <t>판매처 미기재</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr"/>
@@ -27392,19 +27406,19 @@
       <c r="J64" s="2" t="inlineStr"/>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>Keyshop Online: "Includes emergency key: Yes"</t>
+          <t>Keyshop Online "Includes emergency key: Yes" / key4·UHS는 "PCB" (기판만)</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>XSBMK1EN</t>
+          <t>XSTO20EN</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>BMW</t>
+          <t>Toyota</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -27419,12 +27433,12 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>기판만 판매. 넣을 쉘에 맞는 비상키 필요</t>
+          <t>비상키 포함</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>판매처 미기재</t>
+          <t>포함</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr"/>
@@ -27433,12 +27447,53 @@
       <c r="J65" s="2" t="inlineStr"/>
       <c r="K65" s="2" t="inlineStr">
         <is>
+          <t>Keyshop Online: "Includes emergency key: Yes"</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>XSBMK1EN</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>BMW</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>스마트키 기판 (XS)</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>기판만 판매. 넣을 쉘에 맞는 비상키 필요</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>판매처 미기재</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr"/>
+      <c r="H66" s="2" t="n"/>
+      <c r="I66" s="2" t="inlineStr"/>
+      <c r="J66" s="2" t="inlineStr"/>
+      <c r="K66" s="2" t="inlineStr">
+        <is>
           <t>BMW 스마트키용 기판만 파는 제품이에요(쉘·키날 없음). 비상키는 기판을 넣을 BMW 쉘에 맞는 것을 써야 해요. [근거] OBDII365: "Knife Style PCB for BMW G/F Chassis"</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K65"/>
+  <autoFilter ref="A1:K66"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J4" r:id="rId2"/>
@@ -27446,22 +27501,23 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J6" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J7" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J13" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J14" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J33" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J26" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J34" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J35" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J39" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J45" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J52" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J36" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J40" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J46" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J53" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J54" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J55" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J56" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J57" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J58" r:id="rId23"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Clean up price list: universal-blade compatibility, short chip names, buy links
공용 키날 호환 now means compatibility with KEYDIY/Xhorse universal blades
(O / X / 해당 없음 / 확인 필요), independent of whether a blade is
included. X rows name the blade to buy with a link in 비고; chip and
transponder columns hold only the chip info, with remarks moved to 비고.
Re-checked with Xhorse accessory photos (XSTO03EN, XSJP01EN -> O).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KaJs6Wdeh5fe4LTTDbYhia
</commit_message>
<xml_diff>
--- a/Xhorse_키날_비상키_목록.xlsx
+++ b/Xhorse_키날_비상키_목록.xlsx
@@ -24652,7 +24652,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -24707,7 +24707,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -24762,7 +24762,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -24817,7 +24817,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -24872,7 +24872,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -24927,7 +24927,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -24982,7 +24982,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -25344,7 +25344,7 @@
       <c r="J16" s="2" t="inlineStr"/>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>xhorseshop.eu: "MQB type XSMQB4EN Flip type 3 buttons smart key"</t>
+          <t>가격표 공용 키날 O</t>
         </is>
       </c>
     </row>
@@ -25559,7 +25559,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>확인 필요</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -25899,7 +25899,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>확인 필요</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -25940,7 +25940,7 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>확인 필요</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -25981,7 +25981,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>해당 없음</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -26018,7 +26018,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>해당 없음</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -26298,7 +26298,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>확인 필요</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -26468,24 +26468,28 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>확인 필요 (판매처 간 상충)</t>
+          <t>공용 폴딩 키날 (차에 맞는 키웨이 선택)</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>key4는 공용 폴딩 키날 안내 / 같은 토요타형 XSTO01EN은 TOY48 전용 비상키</t>
+          <t>공용 키날 시트 참고</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr"/>
       <c r="H43" s="2" t="n"/>
       <c r="I43" s="2" t="inlineStr"/>
       <c r="J43" s="2" t="inlineStr"/>
-      <c r="K43" s="2" t="inlineStr"/>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>Xhorse 구성품 사진에 공용 폴딩 키날 모양 "Key Blade – 별도 구매", key4도 공용 키날 구매 안내</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -26542,24 +26546,28 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>키날 포함 (CY22)</t>
+          <t>공용 폴딩 키날 (차에 맞는 키웨이 선택)</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>포함</t>
+          <t>공용 키날 시트 참고 (예: 지프 CY22·Y159)</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr"/>
       <c r="H45" s="2" t="n"/>
       <c r="I45" s="2" t="inlineStr"/>
       <c r="J45" s="2" t="inlineStr"/>
-      <c r="K45" s="2" t="inlineStr"/>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>Xhorse 구성품 사진에 공용 폴딩 키날 모양 "Key Blade – 별도 구매" (ABKEYS의 "Key Blade: Included" 표기와 다름)</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -26716,7 +26724,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>해당 없음</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -26753,7 +26761,7 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>해당 없음</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -26794,7 +26802,7 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>해당 없음</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -26831,7 +26839,7 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>해당 없음</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -26868,7 +26876,7 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>해당 없음</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
@@ -27258,7 +27266,7 @@
       <c r="J60" s="2" t="inlineStr"/>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>폭스바겐 투아렉 MLB 스마트키 기판만 파는 제품이에요. 비상키는 기판을 넣을 투아렉 쉘에 맞는 것을 써야 해요. [근거] OBDII365: "Toureg Style MLB Key PCB"</t>
+          <t>기판만 파는 투아렉 MLB 기판이라 공용 키날과 호환 안 돼요. 투아렉 스마트키 비상키(HU162)를 쓰는 것으로 보여요(판매처 지정은 없음): Volkswagen Touareg 2019-2024 Smart Key Blade, HU162 ($7.99) https://abkeys.com/products/volkswagen-touareq-smart-key-blade-hu162-4602 / XZ처럼 기판만 파는 XS 제품군이에요 (XZ와 달리 "특정 브랜드 전용" 표기는 없음)</t>
         </is>
       </c>
     </row>
@@ -27280,7 +27288,7 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>해당 없음</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
@@ -27317,7 +27325,7 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>해당 없음</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -27358,7 +27366,7 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>해당 없음</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
@@ -27395,7 +27403,7 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>해당 없음</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -27432,7 +27440,7 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>해당 없음</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -27473,7 +27481,7 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>해당 없음</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -27514,7 +27522,7 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>해당 없음</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
@@ -27533,7 +27541,7 @@
       <c r="J67" s="2" t="inlineStr"/>
       <c r="K67" s="2" t="inlineStr">
         <is>
-          <t>BMW 스마트키용 기판만 파는 제품이에요(쉘·키날 없음). 비상키는 기판을 넣을 BMW 쉘에 맞는 것을 써야 해요. [근거] OBDII365: "Knife Style PCB for BMW G/F Chassis"</t>
+          <t>기판만 파는 제품이라 키날은 넣을 쉘에 따라 달라요. 판매처가 지정한 비상키는 없어요. / XZ처럼 기판만 파는 XS 제품군이에요 (XZ와 달리 "특정 브랜드 전용" 표기는 없음)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rename XS emergency sheet to dedicated blades and keep only non-universal models
Lists the 14 XS models whose blade is not a KEYDIY/Xhorse universal
blade (X / 확인 필요 in the price list) with the matching emergency key,
price and link.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KaJs6Wdeh5fe4LTTDbYhia
</commit_message>
<xml_diff>
--- a/Xhorse_키날_비상키_목록.xlsx
+++ b/Xhorse_키날_비상키_목록.xlsx
@@ -10,14 +10,14 @@
     <sheet name="공용 키날 (키웨이별)" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="공용 키날 (전체 상품)" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="키날 세트·롤핀·부속" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="XS 비상키 (전체 모델)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="XS 비상키 (전용키날)" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="참고" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'공용 키날 (키웨이별)'!$A$1:$K$93</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'공용 키날 (전체 상품)'!$A$1:$L$442</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'키날 세트·롤핀·부속'!$A$1:$H$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'XS 비상키 (전체 모델)'!$A$1:$K$67</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'XS 비상키 (전용키날)'!$A$1:$J$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -24524,20 +24524,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K67"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="50" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
-    <col width="60" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="90" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -24558,54 +24557,49 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>공용 키날 사용</t>
+          <t>공용 키날 호환</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>비상키 방식</t>
+          <t>맞는 비상키 (키웨이)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>맞는 비상키 / 키날</t>
+          <t>비상키 상품명</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>비상키 상품명</t>
+          <t>1개 가격 (USD)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>비상키 1개 가격 (USD)</t>
+          <t>판매처</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>판매처</t>
+          <t>비상키 페이지</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>비상키 페이지</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>근거</t>
+          <t>근거 / 비고</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>XSBMM0GL</t>
+          <t>XSBM90GL</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Bmw</t>
+          <t>BMW</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -24620,29 +24614,42 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>키날 포함 (BW9MH)</t>
+          <t>BMW 오토바이 BW9MH (키날 포함)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>포함</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr"/>
+          <t>Bmw Motorcycle Chip Less Key, BW9MH</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>6.75</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>ABKEYS</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>XSBMM0GL과 같은 제품. 키날 포함. 교체용 키날만 파는 상품은 없어서 같은 키웨이의 칩 없는 키를 적음</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>XSTO01EN</t>
+          <t>XSBMM0GL</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Toyota</t>
+          <t>Bmw</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -24652,387 +24659,352 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>전용 스마트키 비상키</t>
+          <t>BMW 오토바이 BW9MH (키날 포함)</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>키웨이 TOY48</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Lexus 2013-2024 Smart Key Blade 69515-30380, TOY48</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="n">
-        <v>1.95</v>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
+          <t>Bmw Motorcycle Chip Less Key, BW9MH</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>6.75</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>ABKEYS</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS 스마트키 상세의 "Key Blade: Optional" 지정 상품</t>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>키날이 포함돼 나와요(ABKEYS "Key Blade: Included"). 교체용 키날만 파는 상품은 없어서 같은 키웨이의 칩 없는 키를 적음</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>XSTO01EN</t>
+          <t>XSMA41EN</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Toyota</t>
+          <t>Audi</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>스마트키</t>
+          <t>스마트키 기판 (XS)</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>전용 스마트키 비상키</t>
+          <t>아우디 스마트키 비상키 HU162</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>키웨이 TOY48</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Toyota 2012-2020 Smart Key Blade 69515-33100 69515-06030, TOY48</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="n">
-        <v>1.99</v>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
+          <t>Audi 2018-2024 Smart Key Blade, HU162</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>ABKEYS</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS 스마트키 상세의 "Key Blade: Optional" 지정 상품</t>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>ABKEYS가 XSMA41EN 상세에 지정한 비상키</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>XSTO01EN</t>
+          <t>XSMA4YEN</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Toyota</t>
+          <t>Audi</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>스마트키</t>
+          <t>스마트키 기판 (XS)</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>전용 스마트키 비상키</t>
+          <t>아우디 스마트키 비상키 HU162</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>키웨이 TOY48</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>Toyota 2013-2025 Smart Key Blade 69515-33120, TOY48</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="n">
-        <v>2.65</v>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
+          <t>Audi 2018-2024 Smart Key Blade, HU162</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>ABKEYS</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS 스마트키 상세의 "Key Blade: Optional" 지정 상품</t>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>ABKEYS가 XSMA4YEN 상세에 지정한 비상키 (ABK-2435)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>XSTO01EN</t>
+          <t>XSMA81EN</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Toyota</t>
+          <t>Audi</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>스마트키</t>
+          <t>스마트키 기판 (XS)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>전용 스마트키 비상키</t>
+          <t>아우디 A8 스마트키 비상키 HU162</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>키웨이 TOY48</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Toyota 2017-2026 Smart Key Blade 69515-47030 69515-06050, TOY48</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="n">
-        <v>2.25</v>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
+          <t>Audi 2022-2025 Smart Key Blade, HU162</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>ABKEYS</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS 스마트키 상세의 "Key Blade: Optional" 지정 상품</t>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>같은 A8 MLB 기판 XSMA8YEN에 ABKEYS가 지정한 비상키 (XSMA81EN 직접 지정은 없음)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>XSTO01EN</t>
+          <t>XSMA8YEN</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Toyota</t>
+          <t>Audi</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>스마트키</t>
+          <t>스마트키 기판 (XS)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>XM38 토요타·렉서스형 쉘 전용 비상키 (A/B/C 타입, 판매처 사진 기준)</t>
+          <t>아우디 A8 스마트키 비상키 HU162</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>A/B/C 타입 비상키</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Xhorse VVDI Emergency key blade for XM38 Smart key shell</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>Honrow</t>
-        </is>
-      </c>
-      <c r="J7" s="4" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>판매처 사진상 XM38 토요타·렉서스형 쉘용</t>
+          <t>Audi 2022-2025 Smart Key Blade, HU162</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>ABKEYS</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>ABKEYS가 XSMA8YEN 상세에 지정한 비상키 (ABK-3354)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>XSTO01EN</t>
+          <t>XSMPS1EN</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Toyota</t>
+          <t>Porsche</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>스마트키</t>
+          <t>스마트키 기판 (XS)</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>공용 스마트키 키날 (Keyshop Online 안내)</t>
+          <t>포르쉐 스마트키 비상키 HU162</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>KEYDIY TOY40 / TOY48 S-S (#165)</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>Keydiy Xhorse Universal Smart Remote Key Blade TOY2 / TOY40 / TOY48 S-S Toyota Lexus (#165)</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>Keyshop Online</t>
-        </is>
-      </c>
-      <c r="J8" s="4" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>Keyshop Online XSTO01EN 설명: "comes without an emergency key … any universal blade will fit. If you want to use this remote for Toyota, please buy this emergency blade: … TOY40 / TOY48 S/S (#165)"</t>
+          <t>Porsche 2018-2025 Smart Key Blade, HU162</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>ABKEYS</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Keyshop Online "Test Key: HU162T", 같은 포르쉐 MLB 기판 XSMPSYEN에 ABKEYS가 지정한 비상키</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>XSTO01EN</t>
+          <t>XSMPSYEN</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Toyota</t>
+          <t>Porsche</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>스마트키</t>
+          <t>스마트키 기판 (XS)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>전용 스마트키 비상키</t>
+          <t>포르쉐 스마트키 비상키 HU162</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>XM38 스마트키용 비상키 (insert)</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>Universal Smart Key Insert for Xhorse Universal Smart Key (XM38)</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="n">
-        <v>3.99</v>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>Royal Key Supply</t>
-        </is>
-      </c>
-      <c r="J9" s="4" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>Royal Key Supply 설명: "Universal smart key insert for Xhorse (XSTO01EN) XM38"</t>
+          <t>Porsche 2018-2025 Smart Key Blade, HU162</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>ABKEYS</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>ABKEYS가 XSMPSYEN 상세에 지정한 비상키 (ABK-3082)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>XSBM90GL</t>
+          <t>XSMTUYEN</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>BMW</t>
+          <t>Touareg</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>스마트키</t>
+          <t>스마트키 기판 (XS)</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -25042,33 +25014,42 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>키날 포함 (BW9MH)</t>
+          <t>폭스바겐 투아렉 스마트키 비상키 HU162 (추정)</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>포함</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="n"/>
-      <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" s="2" t="inlineStr"/>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS: 같은 제품 XSBMM0GL "Key Blade: Included"</t>
+          <t>Volkswagen Touareg 2019-2024 Smart Key Blade, HU162</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>7.99</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>ABKEYS</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>투아렉 MLB 기판이라 투아렉 순정 비상키(HU162)로 보임. 판매처 지정은 없음</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>XSDFX1EN</t>
+          <t>XSNIS2EN</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Knife</t>
+          <t>Nissan</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -25078,38 +25059,47 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>공용 폴딩 키날 (차에 맞는 키웨이 선택)</t>
+          <t>닛산 스마트키 비상키 NSN14</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>공용 키날 시트 참고</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="n"/>
-      <c r="I11" s="2" t="inlineStr"/>
-      <c r="J11" s="2" t="inlineStr"/>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>가격표 공용 키날 O</t>
+          <t>Nissan 2007-2025 Smart Key Blade H0564-EG010, NSN14</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>ABKEYS</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>ABKEYS가 XSNIS2EN 상세에 지정한 비상키</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>XSDM04EN</t>
+          <t>XSBEZ2EN</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>MQB</t>
+          <t>Benz</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -25119,38 +25109,33 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>확인 필요</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>공용 폴딩 키날 (HU66)</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>키웨이 HU66 (폴딩 키날, 미포함)</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="n"/>
+          <t>미공개</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="n"/>
+      <c r="H12" s="2" t="inlineStr"/>
       <c r="I12" s="2" t="inlineStr"/>
-      <c r="J12" s="2" t="inlineStr"/>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>xhorseshop.eu: "Blade: Flip HU66 profile blade (Not included)" → 공용 키날 시트의 HU66</t>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Xhorse 구성품 사진에 전용 비상키 머리 부품("Key Blade – 별도 구매")만 나오고 키날 이름·호환 키날은 Xhorse·판매처 모두 미공개. "모델명 + blade" 검색, 판매처 상품 페이지, Xhorse 대리점 XM 키 카테고리에서도 키날 상품을 찾지 못함</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>XSKF01EN</t>
+          <t>XSKA85EN</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>BMW</t>
+          <t>Kia EV</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -25160,52 +25145,33 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>확인 필요</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>공용 폴딩 키날 (차에 맞는 키웨이 선택)</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>키웨이 HU92</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>KeyDiy Xhorse Remote Key Blade For Bmw HU92</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS</t>
-        </is>
-      </c>
-      <c r="J13" s="4" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS 스마트키 상세의 "Key Blade: Optional" 지정 상품</t>
+          <t>미공개</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr"/>
+      <c r="G13" s="2" t="n"/>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Xhorse 구성품 사진에 전용 비상키 머리 부품("Key Blade – 별도 구매")만 나오고 키날 이름·호환 키날은 Xhorse·판매처 모두 미공개. "모델명 + blade" 검색, 판매처 상품 페이지, Xhorse 대리점 XM 키 카테고리에서도 키날 상품을 찾지 못함</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>XSKFF1EN</t>
+          <t>XSKA86EN</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Knife</t>
+          <t>Kia EV</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -25215,52 +25181,33 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>확인 필요</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>공용 폴딩 키날 (차에 맞는 키웨이 선택)</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>키웨이 HU66 (Long)</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>Volkswagen Flip Remote Long Key Blade, HU66</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="n">
-        <v>1.15</v>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS</t>
-        </is>
-      </c>
-      <c r="J14" s="4" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS 스마트키 상세의 "Key Blade: Optional" 지정 상품</t>
+          <t>미공개</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="n"/>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Xhorse 구성품 사진에 전용 비상키 머리 부품("Key Blade – 별도 구매")만 나오고 키날 이름·호환 키날은 Xhorse·판매처 모두 미공개. "모델명 + blade" 검색, 판매처 상품 페이지, Xhorse 대리점 XM 키 카테고리에서도 키날 상품을 찾지 못함</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>XSMQB1EN</t>
+          <t>XSMS01EN</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>MQB</t>
+          <t>Maserati</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -25270,2307 +25217,37 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>확인 필요</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>공용 폴딩 키날 (차에 맞는 키웨이 선택)</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>키웨이 HU66 (Long)</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>Volkswagen Flip Remote Long Key Blade, HU66</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="n">
-        <v>1.15</v>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS</t>
-        </is>
-      </c>
-      <c r="J15" s="4" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS 스마트키 상세의 "Key Blade: Optional" 지정 상품</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>XSMQB4EN</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>MQB</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>스마트키</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>공용 폴딩 키날 (차에 맞는 키웨이 선택)</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>공용 키날 시트 참고</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr"/>
-      <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="inlineStr"/>
-      <c r="J16" s="2" t="inlineStr"/>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>가격표 공용 키날 O</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>XSSC01EN</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Supercar</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>스마트키</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>공용 폴딩 키날 사용 (판매처 설명: "universal flip remote key blades")</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>공용 키날 시트 참고</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr"/>
-      <c r="H17" s="2" t="n"/>
-      <c r="I17" s="2" t="inlineStr"/>
-      <c r="J17" s="2" t="inlineStr"/>
-      <c r="K17" s="2" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>XSSC04EN</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Supercar</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>스마트키</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>공용 폴딩 키날 사용 (판매처 설명: "universal flip remote key blades")</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>공용 키날 시트 참고</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr"/>
-      <c r="H18" s="2" t="n"/>
-      <c r="I18" s="2" t="inlineStr"/>
-      <c r="J18" s="2" t="inlineStr"/>
-      <c r="K18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>XSSC05EN</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Supercar</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>스마트키</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>공용 폴딩 키날 사용 (판매처 설명: "universal flip remote key blades")</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>공용 키날 시트 참고</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr"/>
-      <c r="H19" s="2" t="n"/>
-      <c r="I19" s="2" t="inlineStr"/>
-      <c r="J19" s="2" t="inlineStr"/>
-      <c r="K19" s="2" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>XSSC21EN</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Supercar</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>스마트키</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>공용 폴딩 키날 (차에 맞는 키웨이 선택)</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>공용 키날 시트 참고</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr"/>
-      <c r="H20" s="2" t="n"/>
-      <c r="I20" s="2" t="inlineStr"/>
-      <c r="J20" s="2" t="inlineStr"/>
-      <c r="K20" s="2" t="inlineStr">
-        <is>
-          <t>가격표 공용 키날 O</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>XSSC25EN</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Supercar</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>스마트키</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>공용 폴딩 키날 (차에 맞는 키웨이 선택)</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>공용 키날 시트 참고</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr"/>
-      <c r="H21" s="2" t="n"/>
-      <c r="I21" s="2" t="inlineStr"/>
-      <c r="J21" s="2" t="inlineStr"/>
-      <c r="K21" s="2" t="inlineStr">
-        <is>
-          <t>가격표 공용 키날 O</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>XSBEZ2EN</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Benz</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>스마트키</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>확인 필요</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>키날 별도 구매 (종류 미기재, 확인 필요)</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>판매처 미기재</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr"/>
-      <c r="H22" s="2" t="n"/>
-      <c r="I22" s="2" t="inlineStr"/>
-      <c r="J22" s="2" t="inlineStr"/>
-      <c r="K22" s="2" t="inlineStr">
-        <is>
-          <t>Xhorse 구성품 사진 "Key Blade – 별도 구매"(비상키 머리 부품), Best Key Supply "Blade: Not Included"</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>XSCH01EN</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Chrysler</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>스마트키</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>공용 폴딩 키날 (차에 맞는 키웨이 선택)</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>키웨이 CY22</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>KeyDiy Xhorse Remote Key Blade For Jeep CY22</t>
-        </is>
-      </c>
-      <c r="H23" s="3" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="I23" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS</t>
-        </is>
-      </c>
-      <c r="J23" s="4" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
-      <c r="K23" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS 스마트키 상세의 "Key Blade: Optional" 지정 상품</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>XSCL01EN</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Chevrolet</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>스마트키</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>공용 폴딩 키날 (차에 맞는 키웨이 선택)</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>key4: universal flip remote key blades 구매 안내</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr"/>
-      <c r="H24" s="2" t="n"/>
-      <c r="I24" s="2" t="inlineStr"/>
-      <c r="J24" s="2" t="inlineStr"/>
-      <c r="K24" s="2" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>XSCLN1EN</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Chevrolet</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>스마트키</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>공용 폴딩 키날 (차에 맞는 키웨이 선택)</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>공용 키날 시트 참고</t>
-        </is>
-      </c>
-      <c r="G25" s="2" t="inlineStr"/>
-      <c r="H25" s="2" t="n"/>
-      <c r="I25" s="2" t="inlineStr"/>
-      <c r="J25" s="2" t="inlineStr"/>
-      <c r="K25" s="2" t="inlineStr">
-        <is>
-          <t>가격표 공용 키날 O</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>XSCS00EN</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Hyundai</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>스마트키</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>공용 폴딩 키날 (차에 맞는 키웨이 선택)</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>키웨이 HU66 (Long)</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>Volkswagen Flip Remote Long Key Blade, HU66</t>
-        </is>
-      </c>
-      <c r="H26" s="3" t="n">
-        <v>1.15</v>
-      </c>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS</t>
-        </is>
-      </c>
-      <c r="J26" s="4" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
-      <c r="K26" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS 스마트키 상세의 "Key Blade: Optional" 지정 상품</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>XSDFX2EN</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Knife</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>스마트키</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>공용 폴딩 키날 (차에 맞는 키웨이 선택)</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>나이프(폴딩) 스타일, 키날 미포함 (UHS·Locksmith Keyless)</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="inlineStr"/>
-      <c r="H27" s="2" t="n"/>
-      <c r="I27" s="2" t="inlineStr"/>
-      <c r="J27" s="2" t="inlineStr"/>
-      <c r="K27" s="2" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>XSFO02EN</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>Ford</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>스마트키</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>공용 폴딩 키날 사용 (판매처 설명: "universal flip remote key blades")</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>공용 키날 시트 참고</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr"/>
-      <c r="H28" s="2" t="n"/>
-      <c r="I28" s="2" t="inlineStr"/>
-      <c r="J28" s="2" t="inlineStr"/>
-      <c r="K28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>XSGA80EN</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>VW</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>스마트키</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>공용 폴딩 키날 사용 (판매처 설명: "universal flip remote key blades")</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>공용 키날 시트 참고</t>
-        </is>
-      </c>
-      <c r="G29" s="2" t="inlineStr"/>
-      <c r="H29" s="2" t="n"/>
-      <c r="I29" s="2" t="inlineStr"/>
-      <c r="J29" s="2" t="inlineStr"/>
-      <c r="K29" s="2" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>XSKA85EN</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>Kia EV</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>스마트키</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>확인 필요</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>키날 별도 구매 (종류 미기재, 확인 필요)</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>판매처 미기재</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr"/>
-      <c r="H30" s="2" t="n"/>
-      <c r="I30" s="2" t="inlineStr"/>
-      <c r="J30" s="2" t="inlineStr"/>
-      <c r="K30" s="2" t="inlineStr">
-        <is>
-          <t>Xhorse 구성품 사진 "Key Blade – 별도 구매"(비상키 머리 부품), Best Key Supply "Blade: Not Included"</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>XSKA86EN</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>Kia EV</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>스마트키</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>확인 필요</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>키날 별도 구매 (종류 미기재, 확인 필요)</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>판매처 미기재</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="inlineStr"/>
-      <c r="H31" s="2" t="n"/>
-      <c r="I31" s="2" t="inlineStr"/>
-      <c r="J31" s="2" t="inlineStr"/>
-      <c r="K31" s="2" t="inlineStr">
-        <is>
-          <t>Xhorse 구성품 사진 "Key Blade – 별도 구매"(비상키 머리 부품), Best Key Supply "Blade: Not Included"</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>XSKC04EN</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>King Card</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>카드형 스마트키</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>해당 없음</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>키날 없음 (카드형)</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>해당 없음</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr"/>
-      <c r="H32" s="2" t="n"/>
-      <c r="I32" s="2" t="inlineStr"/>
-      <c r="J32" s="2" t="inlineStr"/>
-      <c r="K32" s="2" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>XSKC05EN</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>King Card</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>카드형 스마트키</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>해당 없음</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>키날 없음 (카드형)</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>해당 없음</t>
-        </is>
-      </c>
-      <c r="G33" s="2" t="inlineStr"/>
-      <c r="H33" s="2" t="n"/>
-      <c r="I33" s="2" t="inlineStr"/>
-      <c r="J33" s="2" t="inlineStr"/>
-      <c r="K33" s="2" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>XSKF20EN</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>BMW</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>스마트키</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>공용 폴딩 키날 (차에 맞는 키웨이 선택)</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>키웨이 HU66 (Long)</t>
-        </is>
-      </c>
-      <c r="G34" s="2" t="inlineStr">
-        <is>
-          <t>Volkswagen Flip Remote Long Key Blade, HU66</t>
-        </is>
-      </c>
-      <c r="H34" s="3" t="n">
-        <v>1.15</v>
-      </c>
-      <c r="I34" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS</t>
-        </is>
-      </c>
-      <c r="J34" s="4" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
-      <c r="K34" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS 스마트키 상세의 "Key Blade: Optional" 지정 상품</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>XSKF21EN</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>BMW</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>스마트키</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>공용 폴딩 키날 (차에 맞는 키웨이 선택)</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t>키웨이 HU66 (Long)</t>
-        </is>
-      </c>
-      <c r="G35" s="2" t="inlineStr">
-        <is>
-          <t>Volkswagen Flip Remote Long Key Blade, HU66</t>
-        </is>
-      </c>
-      <c r="H35" s="3" t="n">
-        <v>1.15</v>
-      </c>
-      <c r="I35" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS</t>
-        </is>
-      </c>
-      <c r="J35" s="4" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
-      <c r="K35" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS 스마트키 상세의 "Key Blade: Optional" 지정 상품</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>XSKF30EN</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>Knife</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>스마트키</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>공용 폴딩 키날 (차에 맞는 키웨이 선택)</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t>키웨이 HU66 (Long)</t>
-        </is>
-      </c>
-      <c r="G36" s="2" t="inlineStr">
-        <is>
-          <t>Volkswagen Flip Remote Long Key Blade, HU66</t>
-        </is>
-      </c>
-      <c r="H36" s="3" t="n">
-        <v>1.15</v>
-      </c>
-      <c r="I36" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS</t>
-        </is>
-      </c>
-      <c r="J36" s="4" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
-      <c r="K36" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS 스마트키 상세의 "Key Blade: Optional" 지정 상품</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>XSKF31EN</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>Knife</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>스마트키</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>공용 폴딩 키날 (차에 맞는 키웨이 선택)</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t>공용 키날 시트 참고</t>
-        </is>
-      </c>
-      <c r="G37" s="2" t="inlineStr"/>
-      <c r="H37" s="2" t="n"/>
-      <c r="I37" s="2" t="inlineStr"/>
-      <c r="J37" s="2" t="inlineStr"/>
-      <c r="K37" s="2" t="inlineStr">
-        <is>
-          <t>가격표 공용 키날 O</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>XSKFF0EN</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>Knife</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>스마트키</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>공용 폴딩 키날 (차에 맞는 키웨이 선택)</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>3버튼 버전 XSKFF1EN과 같은 방식 (Best Key Supply: 키날 별도 장착)</t>
-        </is>
-      </c>
-      <c r="G38" s="2" t="inlineStr"/>
-      <c r="H38" s="2" t="n"/>
-      <c r="I38" s="2" t="inlineStr"/>
-      <c r="J38" s="2" t="inlineStr"/>
-      <c r="K38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>XSMS01EN</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>Maserati</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>스마트키</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>확인 필요</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>키날 별도 구매 (종류 미기재, 확인 필요)</t>
-        </is>
-      </c>
-      <c r="F39" s="2" t="inlineStr">
-        <is>
-          <t>판매처 미기재</t>
-        </is>
-      </c>
-      <c r="G39" s="2" t="inlineStr"/>
-      <c r="H39" s="2" t="n"/>
-      <c r="I39" s="2" t="inlineStr"/>
-      <c r="J39" s="2" t="inlineStr"/>
-      <c r="K39" s="2" t="inlineStr">
-        <is>
-          <t>Xhorse 구성품 사진 "Key Blade – 별도 구매"(비상키 머리 부품)</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>XSNIS2EN</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>Nissan</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>스마트키</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>전용 스마트키 비상키</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="inlineStr">
-        <is>
-          <t>키웨이 NSN14</t>
-        </is>
-      </c>
-      <c r="G40" s="2" t="inlineStr">
-        <is>
-          <t>Nissan 2007-2025 Smart Key Blade H0564-EG010, NSN14</t>
-        </is>
-      </c>
-      <c r="H40" s="3" t="n">
-        <v>1.95</v>
-      </c>
-      <c r="I40" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS</t>
-        </is>
-      </c>
-      <c r="J40" s="4" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
-      <c r="K40" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS 스마트키 상세의 "Key Blade: Optional" 지정 상품</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>XSPS01EN</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>Porsche</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>스마트키</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>공용 폴딩 키날 사용 (판매처 설명: "universal flip remote key blades")</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>공용 키날 시트 참고</t>
-        </is>
-      </c>
-      <c r="G41" s="2" t="inlineStr"/>
-      <c r="H41" s="2" t="n"/>
-      <c r="I41" s="2" t="inlineStr"/>
-      <c r="J41" s="2" t="inlineStr"/>
-      <c r="K41" s="2" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>XSSBR0EN</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Subaru</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>스마트키</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>공용 폴딩 키날 사용 (판매처 설명: "universal flip remote key blades")</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>공용 키날 시트 참고</t>
-        </is>
-      </c>
-      <c r="G42" s="2" t="inlineStr"/>
-      <c r="H42" s="2" t="n"/>
-      <c r="I42" s="2" t="inlineStr"/>
-      <c r="J42" s="2" t="inlineStr"/>
-      <c r="K42" s="2" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>XSTO03EN</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>Toyota</t>
-        </is>
-      </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>스마트키</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr">
-        <is>
-          <t>공용 폴딩 키날 (차에 맞는 키웨이 선택)</t>
-        </is>
-      </c>
-      <c r="F43" s="2" t="inlineStr">
-        <is>
-          <t>공용 키날 시트 참고</t>
-        </is>
-      </c>
-      <c r="G43" s="2" t="inlineStr"/>
-      <c r="H43" s="2" t="n"/>
-      <c r="I43" s="2" t="inlineStr"/>
-      <c r="J43" s="2" t="inlineStr"/>
-      <c r="K43" s="2" t="inlineStr">
-        <is>
-          <t>Xhorse 구성품 사진에 공용 폴딩 키날 모양 "Key Blade – 별도 구매", key4도 공용 키날 구매 안내</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>XSCD01EN</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>Cadillac</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>스마트키</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>공용 폴딩 키날 사용 (판매처 설명: "universal flip remote key blades")</t>
-        </is>
-      </c>
-      <c r="F44" s="2" t="inlineStr">
-        <is>
-          <t>공용 키날 시트 참고</t>
-        </is>
-      </c>
-      <c r="G44" s="2" t="inlineStr"/>
-      <c r="H44" s="2" t="n"/>
-      <c r="I44" s="2" t="inlineStr"/>
-      <c r="J44" s="2" t="inlineStr"/>
-      <c r="K44" s="2" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>XSJP01EN</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>Jeep</t>
-        </is>
-      </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>스마트키</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>공용 폴딩 키날 (차에 맞는 키웨이 선택)</t>
-        </is>
-      </c>
-      <c r="F45" s="2" t="inlineStr">
-        <is>
-          <t>공용 키날 시트 참고 (예: 지프 CY22·Y159)</t>
-        </is>
-      </c>
-      <c r="G45" s="2" t="inlineStr"/>
-      <c r="H45" s="2" t="n"/>
-      <c r="I45" s="2" t="inlineStr"/>
-      <c r="J45" s="2" t="inlineStr"/>
-      <c r="K45" s="2" t="inlineStr">
-        <is>
-          <t>Xhorse 구성품 사진에 공용 폴딩 키날 모양 "Key Blade – 별도 구매" (ABKEYS의 "Key Blade: Included" 표기와 다름)</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>XSLR01EN</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>Rover</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>스마트키</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>공용 폴딩 키날 (Xhorse 사진 기준)</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>공용 키날 시트 참고</t>
-        </is>
-      </c>
-      <c r="G46" s="2" t="inlineStr"/>
-      <c r="H46" s="2" t="n"/>
-      <c r="I46" s="2" t="inlineStr"/>
-      <c r="J46" s="2" t="inlineStr"/>
-      <c r="K46" s="2" t="inlineStr">
-        <is>
-          <t>Xhorse 구성품 사진에 공용 폴딩 키날 모양 "Key Blade – 별도 구매". ABKEYS는 아래 HU101 랜드로버 스마트키 비상키를 지정</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>XSLR01EN</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>Rover</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>스마트키</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>전용 스마트키 비상키</t>
-        </is>
-      </c>
-      <c r="F47" s="2" t="inlineStr">
-        <is>
-          <t>키웨이 HU101</t>
-        </is>
-      </c>
-      <c r="G47" s="2" t="inlineStr">
-        <is>
-          <t>Range Rover, Land Rover 2010+ Smart Key Blade, HU101</t>
-        </is>
-      </c>
-      <c r="H47" s="3" t="n">
-        <v>2.65</v>
-      </c>
-      <c r="I47" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS</t>
-        </is>
-      </c>
-      <c r="J47" s="4" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
-      <c r="K47" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS 스마트키 상세의 "Key Blade: Optional" 지정 상품</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>XSLR03EN</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>Rover</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>스마트키</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>공용 폴딩 키날 (차에 맞는 키웨이 선택)</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="inlineStr">
-        <is>
-          <t>공용 키날 시트 참고</t>
-        </is>
-      </c>
-      <c r="G48" s="2" t="inlineStr"/>
-      <c r="H48" s="2" t="n"/>
-      <c r="I48" s="2" t="inlineStr"/>
-      <c r="J48" s="2" t="inlineStr"/>
-      <c r="K48" s="2" t="inlineStr">
-        <is>
-          <t>같은 랜드로버 모양 XSLR01EN의 Xhorse 구성품 사진에 공용 폴딩 키날 모양 "Key Blade – 별도 구매" (XSLR03EN은 Best Key Supply "Blade: Not Included")</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>XSBTK0EN</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="inlineStr">
-        <is>
-          <t>Bluetooth</t>
-        </is>
-      </c>
-      <c r="C49" s="2" t="inlineStr">
-        <is>
-          <t>블루투스 디지털 키</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="inlineStr">
-        <is>
-          <t>해당 없음</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="inlineStr">
-        <is>
-          <t>해당 없음</t>
-        </is>
-      </c>
-      <c r="F49" s="2" t="inlineStr">
-        <is>
-          <t>해당 없음</t>
-        </is>
-      </c>
-      <c r="G49" s="2" t="inlineStr"/>
-      <c r="H49" s="2" t="n"/>
-      <c r="I49" s="2" t="inlineStr"/>
-      <c r="J49" s="2" t="inlineStr"/>
-      <c r="K49" s="2" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>XSBTKOGL</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>Bluetooth</t>
-        </is>
-      </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>블루투스 디지털 키</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>해당 없음</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>해당 없음</t>
-        </is>
-      </c>
-      <c r="F50" s="2" t="inlineStr">
-        <is>
-          <t>해당 없음</t>
-        </is>
-      </c>
-      <c r="G50" s="2" t="inlineStr"/>
-      <c r="H50" s="2" t="n"/>
-      <c r="I50" s="2" t="inlineStr"/>
-      <c r="J50" s="2" t="inlineStr"/>
-      <c r="K50" s="2" t="inlineStr">
-        <is>
-          <t>휴대폰 디지털키 (키날 자리 없음)</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr">
-        <is>
-          <t>XSWK02EN</t>
-        </is>
-      </c>
-      <c r="B51" s="2" t="inlineStr">
-        <is>
-          <t>Watch (SW-007)</t>
-        </is>
-      </c>
-      <c r="C51" s="2" t="inlineStr">
-        <is>
-          <t>스마트워치형 키</t>
-        </is>
-      </c>
-      <c r="D51" s="2" t="inlineStr">
-        <is>
-          <t>해당 없음</t>
-        </is>
-      </c>
-      <c r="E51" s="2" t="inlineStr">
-        <is>
-          <t>해당 없음</t>
-        </is>
-      </c>
-      <c r="F51" s="2" t="inlineStr">
-        <is>
-          <t>해당 없음</t>
-        </is>
-      </c>
-      <c r="G51" s="2" t="inlineStr"/>
-      <c r="H51" s="2" t="n"/>
-      <c r="I51" s="2" t="inlineStr"/>
-      <c r="J51" s="2" t="inlineStr"/>
-      <c r="K51" s="2" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>XSWK05EN</t>
-        </is>
-      </c>
-      <c r="B52" s="2" t="inlineStr">
-        <is>
-          <t>Watch (SW-007)</t>
-        </is>
-      </c>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
-          <t>스마트워치형 키</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="inlineStr">
-        <is>
-          <t>해당 없음</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="inlineStr">
-        <is>
-          <t>해당 없음</t>
-        </is>
-      </c>
-      <c r="F52" s="2" t="inlineStr">
-        <is>
-          <t>해당 없음</t>
-        </is>
-      </c>
-      <c r="G52" s="2" t="inlineStr"/>
-      <c r="H52" s="2" t="n"/>
-      <c r="I52" s="2" t="inlineStr"/>
-      <c r="J52" s="2" t="inlineStr"/>
-      <c r="K52" s="2" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="2" t="inlineStr">
-        <is>
-          <t>XSTO00EN</t>
-        </is>
-      </c>
-      <c r="B53" s="2" t="inlineStr">
-        <is>
-          <t>Toyota</t>
-        </is>
-      </c>
-      <c r="C53" s="2" t="inlineStr">
-        <is>
-          <t>스마트키 기판 (XS)</t>
-        </is>
-      </c>
-      <c r="D53" s="2" t="inlineStr">
-        <is>
-          <t>해당 없음</t>
-        </is>
-      </c>
-      <c r="E53" s="2" t="inlineStr">
-        <is>
-          <t>기판만 판매. 토요타 스마트키 쉘용 비상키 필요</t>
-        </is>
-      </c>
-      <c r="F53" s="2" t="inlineStr">
-        <is>
-          <t>판매처 지정 없음 (토요타 스마트키는 보통 TOY48)</t>
-        </is>
-      </c>
-      <c r="G53" s="2" t="inlineStr"/>
-      <c r="H53" s="2" t="n"/>
-      <c r="I53" s="2" t="inlineStr"/>
-      <c r="J53" s="2" t="inlineStr"/>
-      <c r="K53" s="2" t="inlineStr">
-        <is>
-          <t>UHS: "Smart Key PCB … TOY.T"</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>XSMA41EN</t>
-        </is>
-      </c>
-      <c r="B54" s="2" t="inlineStr">
-        <is>
-          <t>Audi</t>
-        </is>
-      </c>
-      <c r="C54" s="2" t="inlineStr">
-        <is>
-          <t>스마트키 기판 (XS)</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>전용 스마트키 비상키</t>
-        </is>
-      </c>
-      <c r="F54" s="2" t="inlineStr">
-        <is>
-          <t>키웨이 HU162</t>
-        </is>
-      </c>
-      <c r="G54" s="2" t="inlineStr">
-        <is>
-          <t>Audi 2018-2024 Smart Key Blade, HU162</t>
-        </is>
-      </c>
-      <c r="H54" s="3" t="n">
-        <v>5.75</v>
-      </c>
-      <c r="I54" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS</t>
-        </is>
-      </c>
-      <c r="J54" s="4" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
-      <c r="K54" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS 스마트키 상세의 "Key Blade: Optional" 지정 상품</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t>XSMA4YEN</t>
-        </is>
-      </c>
-      <c r="B55" s="2" t="inlineStr">
-        <is>
-          <t>Audi</t>
-        </is>
-      </c>
-      <c r="C55" s="2" t="inlineStr">
-        <is>
-          <t>스마트키 기판 (XS)</t>
-        </is>
-      </c>
-      <c r="D55" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E55" s="2" t="inlineStr">
-        <is>
-          <t>전용 스마트키 비상키</t>
-        </is>
-      </c>
-      <c r="F55" s="2" t="inlineStr">
-        <is>
-          <t>키웨이 HU162</t>
-        </is>
-      </c>
-      <c r="G55" s="2" t="inlineStr">
-        <is>
-          <t>Audi 2018-2024 Smart Key Blade, HU162</t>
-        </is>
-      </c>
-      <c r="H55" s="3" t="n">
-        <v>5.75</v>
-      </c>
-      <c r="I55" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS</t>
-        </is>
-      </c>
-      <c r="J55" s="4" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
-      <c r="K55" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS 스마트키 상세의 "Key Blade: Optional" 지정 상품</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t>XSMA81EN</t>
-        </is>
-      </c>
-      <c r="B56" s="2" t="inlineStr">
-        <is>
-          <t>Audi</t>
-        </is>
-      </c>
-      <c r="C56" s="2" t="inlineStr">
-        <is>
-          <t>스마트키 기판 (XS)</t>
-        </is>
-      </c>
-      <c r="D56" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="inlineStr">
-        <is>
-          <t>전용 스마트키 비상키 (추정)</t>
-        </is>
-      </c>
-      <c r="F56" s="2" t="inlineStr">
-        <is>
-          <t>HU162 아우디 스마트키 비상키</t>
-        </is>
-      </c>
-      <c r="G56" s="2" t="inlineStr">
-        <is>
-          <t>Audi 2022-2025 Smart Key Blade, HU162</t>
-        </is>
-      </c>
-      <c r="H56" s="3" t="n">
-        <v>8.99</v>
-      </c>
-      <c r="I56" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS</t>
-        </is>
-      </c>
-      <c r="J56" s="4" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
-      <c r="K56" s="2" t="inlineStr">
-        <is>
-          <t>같은 아우디 A8 MLB 기판 XSMA8YEN에 ABKEYS가 지정한 비상키</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="2" t="inlineStr">
-        <is>
-          <t>XSMA8YEN</t>
-        </is>
-      </c>
-      <c r="B57" s="2" t="inlineStr">
-        <is>
-          <t>Audi</t>
-        </is>
-      </c>
-      <c r="C57" s="2" t="inlineStr">
-        <is>
-          <t>스마트키 기판 (XS)</t>
-        </is>
-      </c>
-      <c r="D57" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E57" s="2" t="inlineStr">
-        <is>
-          <t>전용 스마트키 비상키</t>
-        </is>
-      </c>
-      <c r="F57" s="2" t="inlineStr">
-        <is>
-          <t>키웨이 HU162</t>
-        </is>
-      </c>
-      <c r="G57" s="2" t="inlineStr">
-        <is>
-          <t>Audi 2022-2025 Smart Key Blade, HU162</t>
-        </is>
-      </c>
-      <c r="H57" s="3" t="n">
-        <v>8.99</v>
-      </c>
-      <c r="I57" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS</t>
-        </is>
-      </c>
-      <c r="J57" s="4" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
-      <c r="K57" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS 스마트키 상세의 "Key Blade: Optional" 지정 상품</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="2" t="inlineStr">
-        <is>
-          <t>XSMPS1EN</t>
-        </is>
-      </c>
-      <c r="B58" s="2" t="inlineStr">
-        <is>
-          <t>Porsche</t>
-        </is>
-      </c>
-      <c r="C58" s="2" t="inlineStr">
-        <is>
-          <t>스마트키 기판 (XS)</t>
-        </is>
-      </c>
-      <c r="D58" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E58" s="2" t="inlineStr">
-        <is>
-          <t>전용 스마트키 비상키</t>
-        </is>
-      </c>
-      <c r="F58" s="2" t="inlineStr">
-        <is>
-          <t>HU162 포르쉐 스마트키 비상키</t>
-        </is>
-      </c>
-      <c r="G58" s="2" t="inlineStr">
-        <is>
-          <t>Porsche 2018-2025 Smart Key Blade, HU162</t>
-        </is>
-      </c>
-      <c r="H58" s="3" t="n">
-        <v>3.25</v>
-      </c>
-      <c r="I58" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS</t>
-        </is>
-      </c>
-      <c r="J58" s="4" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
-      <c r="K58" s="2" t="inlineStr">
-        <is>
-          <t>Keyshop Online "Test Key: HU162T", 같은 포르쉐 MLB 기판 XSMPSYEN에 ABKEYS가 지정한 비상키</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="2" t="inlineStr">
-        <is>
-          <t>XSMPSYEN</t>
-        </is>
-      </c>
-      <c r="B59" s="2" t="inlineStr">
-        <is>
-          <t>Porsche</t>
-        </is>
-      </c>
-      <c r="C59" s="2" t="inlineStr">
-        <is>
-          <t>스마트키 기판 (XS)</t>
-        </is>
-      </c>
-      <c r="D59" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E59" s="2" t="inlineStr">
-        <is>
-          <t>전용 스마트키 비상키</t>
-        </is>
-      </c>
-      <c r="F59" s="2" t="inlineStr">
-        <is>
-          <t>키웨이 HU162</t>
-        </is>
-      </c>
-      <c r="G59" s="2" t="inlineStr">
-        <is>
-          <t>Porsche 2018-2025 Smart Key Blade, HU162</t>
-        </is>
-      </c>
-      <c r="H59" s="3" t="n">
-        <v>3.25</v>
-      </c>
-      <c r="I59" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS</t>
-        </is>
-      </c>
-      <c r="J59" s="4" t="inlineStr">
-        <is>
-          <t>링크</t>
-        </is>
-      </c>
-      <c r="K59" s="2" t="inlineStr">
-        <is>
-          <t>ABKEYS 스마트키 상세의 "Key Blade: Optional" 지정 상품</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="2" t="inlineStr">
-        <is>
-          <t>XSMTUYEN</t>
-        </is>
-      </c>
-      <c r="B60" s="2" t="inlineStr">
-        <is>
-          <t>Touareg</t>
-        </is>
-      </c>
-      <c r="C60" s="2" t="inlineStr">
-        <is>
-          <t>스마트키 기판 (XS)</t>
-        </is>
-      </c>
-      <c r="D60" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E60" s="2" t="inlineStr">
-        <is>
-          <t>기판만 판매. 넣을 쉘에 맞는 비상키 필요</t>
-        </is>
-      </c>
-      <c r="F60" s="2" t="inlineStr">
-        <is>
-          <t>판매처 미기재</t>
-        </is>
-      </c>
-      <c r="G60" s="2" t="inlineStr"/>
-      <c r="H60" s="2" t="n"/>
-      <c r="I60" s="2" t="inlineStr"/>
-      <c r="J60" s="2" t="inlineStr"/>
-      <c r="K60" s="2" t="inlineStr">
-        <is>
-          <t>기판만 파는 투아렉 MLB 기판이라 공용 키날과 호환 안 돼요. 투아렉 스마트키 비상키(HU162)를 쓰는 것으로 보여요(판매처 지정은 없음): Volkswagen Touareg 2019-2024 Smart Key Blade, HU162 ($7.99) https://abkeys.com/products/volkswagen-touareq-smart-key-blade-hu162-4602 / XZ처럼 기판만 파는 XS 제품군이에요 (XZ와 달리 "특정 브랜드 전용" 표기는 없음)</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="2" t="inlineStr">
-        <is>
-          <t>XSADJ1EN</t>
-        </is>
-      </c>
-      <c r="B61" s="2" t="inlineStr">
-        <is>
-          <t>Audi</t>
-        </is>
-      </c>
-      <c r="C61" s="2" t="inlineStr">
-        <is>
-          <t>스마트키 기판 (XS)</t>
-        </is>
-      </c>
-      <c r="D61" s="2" t="inlineStr">
-        <is>
-          <t>해당 없음</t>
-        </is>
-      </c>
-      <c r="E61" s="2" t="inlineStr">
-        <is>
-          <t>기판만 판매. 아우디 순정형 쉘용 비상키 필요</t>
-        </is>
-      </c>
-      <c r="F61" s="2" t="inlineStr">
-        <is>
-          <t>UHS: Board only, Emergency Blade not included</t>
-        </is>
-      </c>
-      <c r="G61" s="2" t="inlineStr"/>
-      <c r="H61" s="2" t="n"/>
-      <c r="I61" s="2" t="inlineStr"/>
-      <c r="J61" s="2" t="inlineStr"/>
-      <c r="K61" s="2" t="inlineStr"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="2" t="inlineStr">
-        <is>
-          <t>XSADJ1GL</t>
-        </is>
-      </c>
-      <c r="B62" s="2" t="inlineStr">
-        <is>
-          <t>Audi</t>
-        </is>
-      </c>
-      <c r="C62" s="2" t="inlineStr">
-        <is>
-          <t>스마트키 기판 (XS)</t>
-        </is>
-      </c>
-      <c r="D62" s="2" t="inlineStr">
-        <is>
-          <t>해당 없음</t>
-        </is>
-      </c>
-      <c r="E62" s="2" t="inlineStr">
-        <is>
-          <t>기판만 판매. 아우디 순정형 쉘용 비상키 필요</t>
-        </is>
-      </c>
-      <c r="F62" s="2" t="inlineStr">
-        <is>
-          <t>XSADJ1EN과 같음</t>
-        </is>
-      </c>
-      <c r="G62" s="2" t="inlineStr"/>
-      <c r="H62" s="2" t="n"/>
-      <c r="I62" s="2" t="inlineStr"/>
-      <c r="J62" s="2" t="inlineStr"/>
-      <c r="K62" s="2" t="inlineStr">
-        <is>
-          <t>UHS: XSADJ1EN "Board only", "Emergency Blade (not included)"</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="2" t="inlineStr">
-        <is>
-          <t>XSBMB1EN</t>
-        </is>
-      </c>
-      <c r="B63" s="2" t="inlineStr">
-        <is>
-          <t>Bread</t>
-        </is>
-      </c>
-      <c r="C63" s="2" t="inlineStr">
-        <is>
-          <t>스마트키 기판 (XS)</t>
-        </is>
-      </c>
-      <c r="D63" s="2" t="inlineStr">
-        <is>
-          <t>해당 없음</t>
-        </is>
-      </c>
-      <c r="E63" s="2" t="inlineStr">
-        <is>
-          <t>기판만 판매. 사용하는 쉘에 맞는 비상키 필요</t>
-        </is>
-      </c>
-      <c r="F63" s="2" t="inlineStr">
-        <is>
-          <t>판매처 미기재</t>
-        </is>
-      </c>
-      <c r="G63" s="2" t="inlineStr"/>
-      <c r="H63" s="2" t="n"/>
-      <c r="I63" s="2" t="inlineStr"/>
-      <c r="J63" s="2" t="inlineStr"/>
-      <c r="K63" s="2" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="2" t="inlineStr">
-        <is>
-          <t>XSBMU1EN</t>
-        </is>
-      </c>
-      <c r="B64" s="2" t="inlineStr">
-        <is>
-          <t>U</t>
-        </is>
-      </c>
-      <c r="C64" s="2" t="inlineStr">
-        <is>
-          <t>스마트키 기판 (XS)</t>
-        </is>
-      </c>
-      <c r="D64" s="2" t="inlineStr">
-        <is>
-          <t>해당 없음</t>
-        </is>
-      </c>
-      <c r="E64" s="2" t="inlineStr">
-        <is>
-          <t>기판만 판매. 사용하는 쉘에 맞는 비상키 필요</t>
-        </is>
-      </c>
-      <c r="F64" s="2" t="inlineStr">
-        <is>
-          <t>판매처 미기재</t>
-        </is>
-      </c>
-      <c r="G64" s="2" t="inlineStr"/>
-      <c r="H64" s="2" t="n"/>
-      <c r="I64" s="2" t="inlineStr"/>
-      <c r="J64" s="2" t="inlineStr"/>
-      <c r="K64" s="2" t="inlineStr"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="2" t="inlineStr">
-        <is>
-          <t>XSBZ01EN</t>
-        </is>
-      </c>
-      <c r="B65" s="2" t="inlineStr">
-        <is>
-          <t>Benz</t>
-        </is>
-      </c>
-      <c r="C65" s="2" t="inlineStr">
-        <is>
-          <t>스마트키 기판 (XS)</t>
-        </is>
-      </c>
-      <c r="D65" s="2" t="inlineStr">
-        <is>
-          <t>해당 없음</t>
-        </is>
-      </c>
-      <c r="E65" s="2" t="inlineStr">
-        <is>
-          <t>판매처마다 다름 (확인 필요)</t>
-        </is>
-      </c>
-      <c r="F65" s="2" t="inlineStr">
-        <is>
-          <t>판매처 미기재</t>
-        </is>
-      </c>
-      <c r="G65" s="2" t="inlineStr"/>
-      <c r="H65" s="2" t="n"/>
-      <c r="I65" s="2" t="inlineStr"/>
-      <c r="J65" s="2" t="inlineStr"/>
-      <c r="K65" s="2" t="inlineStr">
-        <is>
-          <t>Keyshop Online "Includes emergency key: Yes" / key4·UHS는 "PCB" (기판만)</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="2" t="inlineStr">
-        <is>
-          <t>XSTO20EN</t>
-        </is>
-      </c>
-      <c r="B66" s="2" t="inlineStr">
-        <is>
-          <t>Toyota</t>
-        </is>
-      </c>
-      <c r="C66" s="2" t="inlineStr">
-        <is>
-          <t>스마트키 기판 (XS)</t>
-        </is>
-      </c>
-      <c r="D66" s="2" t="inlineStr">
-        <is>
-          <t>해당 없음</t>
-        </is>
-      </c>
-      <c r="E66" s="2" t="inlineStr">
-        <is>
-          <t>비상키 포함</t>
-        </is>
-      </c>
-      <c r="F66" s="2" t="inlineStr">
-        <is>
-          <t>포함</t>
-        </is>
-      </c>
-      <c r="G66" s="2" t="inlineStr"/>
-      <c r="H66" s="2" t="n"/>
-      <c r="I66" s="2" t="inlineStr"/>
-      <c r="J66" s="2" t="inlineStr"/>
-      <c r="K66" s="2" t="inlineStr">
-        <is>
-          <t>Keyshop Online: "Includes emergency key: Yes"</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="2" t="inlineStr">
-        <is>
-          <t>XSBMK1EN</t>
-        </is>
-      </c>
-      <c r="B67" s="2" t="inlineStr">
-        <is>
-          <t>BMW</t>
-        </is>
-      </c>
-      <c r="C67" s="2" t="inlineStr">
-        <is>
-          <t>스마트키 기판 (XS)</t>
-        </is>
-      </c>
-      <c r="D67" s="2" t="inlineStr">
-        <is>
-          <t>해당 없음</t>
-        </is>
-      </c>
-      <c r="E67" s="2" t="inlineStr">
-        <is>
-          <t>기판만 판매. 넣을 쉘에 맞는 비상키 필요</t>
-        </is>
-      </c>
-      <c r="F67" s="2" t="inlineStr">
-        <is>
-          <t>판매처 미기재</t>
-        </is>
-      </c>
-      <c r="G67" s="2" t="inlineStr"/>
-      <c r="H67" s="2" t="n"/>
-      <c r="I67" s="2" t="inlineStr"/>
-      <c r="J67" s="2" t="inlineStr"/>
-      <c r="K67" s="2" t="inlineStr">
-        <is>
-          <t>기판만 파는 제품이라 키날은 넣을 쉘에 따라 달라요. 판매처가 지정한 비상키는 없어요. / XZ처럼 기판만 파는 XS 제품군이에요 (XZ와 달리 "특정 브랜드 전용" 표기는 없음)</t>
+          <t>미공개</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="n"/>
+      <c r="H15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Xhorse 구성품 사진에 전용 비상키 머리 부품("Key Blade – 별도 구매")만 나오고 키날 이름·호환 키날은 Xhorse·판매처 모두 미공개. "모델명 + blade" 검색, 판매처 상품 페이지, Xhorse 대리점 XM 키 카테고리에서도 키날 상품을 찾지 못함</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K67"/>
+  <autoFilter ref="A1:J15"/>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J4" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J5" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J6" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J7" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J13" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J14" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J26" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J34" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J35" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J36" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J40" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J47" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J54" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J55" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J56" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J57" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J58" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J59" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -27688,12 +25365,12 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>XS 비상키 (전체 모델)</t>
+          <t>XS 비상키 (전용키날)</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>가격표의 XS 59개 모델 전부. 판매처가 지정한 비상키가 있으면 상품·가격·링크를 연결 (ABKEYS "Key Blade: Optional" 지정, Royal Key Supply XM38 insert, Honrow A/B/C). 지정이 없는 모델은 방식과 근거만 적음</t>
+          <t>XS 스마트키 중 공용 키날(KEYDIY/Xhorse 공용 키날)이 맞지 않는 모델 14개만 정리. 모델마다 맞는 비상키(키웨이), 상품, 가격, 링크. 판정 기준은 Xhorse_모델별_가격표.xlsx의 "공용 키날 호환"과 같음 (X, 확인 필요). 공용 키날이 맞는 XS 모델은 "공용 키날" 시트에서 차 키웨이에 맞는 키날을 고르면 됨</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct Y-number note: KD blades are normally stamped with digits only
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KaJs6Wdeh5fe4LTTDbYhia
</commit_message>
<xml_diff>
--- a/Xhorse_키날_비상키_목록.xlsx
+++ b/Xhorse_키날_비상키_목록.xlsx
@@ -1017,7 +1017,7 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Silca 정식 표기 KIA9TE. UHS의 "#Y75"는 Y-번호. gskeyae는 #156을 "KK12 HU134"로 표기. 순정 리모컨에는 안 맞음</t>
+          <t>Silca 정식 표기 KIA9TE. UHS의 "#Y75"는 Y-번호. gskeyae는 #156을 "KK12 HU134"로 표기. 키날 각인은 156 또는 75(Y-75의 숫자)로 옴. 순정 리모컨에는 안 맞음</t>
         </is>
       </c>
     </row>
@@ -12961,7 +12961,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>KD 키날 몸통에 찍혀 나오는 두 번째 번호 (UHS 상품 사진: TOY47 키날에 "Y22" 각인, UHS 설명 "Number on Blade: Y66"). Keyshop 50종 목록은 한 상품코드에 "#129 Y-16"처럼 둘 다 적고, Keystation은 "HYN17 #129 #Y16", Acme Locksmith는 "HY18 (Y-16#)"로 같은 키날에 씀. 같은 키날이라도 찍힌 번호가 다를 수 있음 (UHS: MIT8 키날은 Y21·29·08이 찍혀 오거나 번호가 없을 수 있음). KEYDIY·Xhorse 공식 설명은 찾지 못해 어느 회사가 매긴 번호인지는 미확인</t>
+          <t>판매처가 #번호와 함께 쓰는 두 번째 번호. 한 상품에 둘을 같이 적은 곳: Keyshop 50종 목록("HYN17 - #129 Y-16", 상품코드 하나), Keystation("HYN17 #129 #Y16"), Acme Locksmith("HY18 (Y-16#)"). KD 키날에는 보통 숫자만 찍혀 있음(사용자 확인. 사진으로 본 각인: KK12 "156" 또는 "75", HY18R "130"). Y가 찍힌 사진은 TOY47 "Y22" 1건뿐. KK12처럼 숫자 각인이 #번호(156)일 때도, Y-번호의 숫자(75)일 때도 있음. 어느 회사가 매긴 번호인지는 공식 자료로 확인 못 함</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
NE73 KEYDIY 칸에 Y-30 추정값 기록
판매처 표기가 Y-30 5곳 대 #53/Y-14 5곳으로 갈렸지만, NE72와 NE73을
따로 파는 판매처(Reid's, Access Fobs)는 모두 NE73 = Y-30이고
#53(Y-14)은 판매처 7곳 기준 NE72 키날이라 Y-30으로 추정해 기록.
비고 맨 앞에 [추정]을 달고 확인 상태는 일부 확인으로 둠.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KaJs6Wdeh5fe4LTTDbYhia
</commit_message>
<xml_diff>
--- a/Xhorse_키날_비상키_목록.xlsx
+++ b/Xhorse_키날_비상키_목록.xlsx
@@ -45,7 +45,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -67,11 +67,6 @@
         <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F8CBAD"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -90,7 +85,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -105,9 +100,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -3535,7 +3527,11 @@
           <t>없음</t>
         </is>
       </c>
-      <c r="B76" s="2" t="inlineStr"/>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>Y-30</t>
+        </is>
+      </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
           <t>NE73</t>
@@ -3551,15 +3547,19 @@
           <t>푸조·시트로엥·르노</t>
         </is>
       </c>
-      <c r="F76" s="6" t="inlineStr">
-        <is>
-          <t>확인 필요</t>
-        </is>
-      </c>
-      <c r="G76" s="3" t="inlineStr"/>
+      <c r="F76" s="5" t="inlineStr">
+        <is>
+          <t>일부 확인</t>
+        </is>
+      </c>
+      <c r="G76" s="3" t="inlineStr">
+        <is>
+          <t>Y-30 5곳</t>
+        </is>
+      </c>
       <c r="H76" s="3" t="inlineStr">
         <is>
-          <t>[판매처끼리 엇갈림, 추가 검색 후에도 비슷함] Y-30으로 적은 곳 5곳(Access Fobs "NE73 NE-38 Y30#"·Reid's "Silca NE73 JMA NE-38 NE#Y-30"·A-D-E "#Y-30 NE73"·Keyshop "NE73 #53 Y-30"·NW Keys "NE73/NE72 Y30") 대 #53 또는 Y-14로 적은 곳 5곳(eBay "Type 53 NE73"·MK3/VVDI "NE72/NE73 53"·Keystation "NE73 Y-14"·Keylocksupplies "Y-14# Renault NE73"·KEYECU "Y14 NE73 NE72") → KEYDIY 칸 비움. Silca·JMA 참조를 함께 적은 판매처(Access Fobs·Reid's)는 Y-30</t>
+          <t>[추정: Y-30 (사용자 결정으로 기록). 판매처 표기가 5곳 대 5곳으로 갈려 실물 각인 확인 전까지는 추정] 근거: ① JMA 공식 등가표에서 Silca NE72 = JMA NE-36, Silca NE73 = JMA NE-38로 서로 다른 키 ② NE72 = #53(Y-14)은 판매처 7곳(위 줄) ③ NE72와 NE73을 따로 파는 판매처는 모두 NE73 = Y-30: Reid's(Silca NE72·JMA NE-36 = NE#Y-14, Silca NE73·JMA NE-38 = NE#Y-30), Access Fobs(NE72 "53/Y14", NE73 "Y30#") ④ A-D-E는 "Y-30이 Y-14보다 짧음", Autowave는 NE72용을 "Long Blade"로 따로 팖 → 긴 것 Y-14 = NE72, 짧은 것 Y-30 = NE73 ⑤ Y-30을 적은 판매처는 Keystation 한 곳 빼고 모두 NE73에 붙임. 반대 근거(#53 또는 Y-14): eBay "Type 53 NE73"·MK3/VVDI "NE72/NE73 53"·Keystation "NE72 Y-30 / NE73 Y-14"(NE72 짝이 판매처 7곳과 반대)·Keylocksupplies "Y-14# Renault NE73"·KEYECU "Y14 NE73 NE72" — 대부분 두 이름을 한 상품에 같이 붙인 표기라 NE73 번호를 정해 주지 못함. Keyshop 50종 목록의 "NE73 #53 Y-30"은 같은 목록에 틀린 #번호가 여럿 있어(DWO5R #13·VA2 LONG #13·MIT08 #15) #53은 믿기 어려움 → Y-30의 #번호는 비움. 실물 확인: 기존 키와 키날 길이 비교(Y-30이 짧음) 또는 키날 각인</t>
         </is>
       </c>
     </row>
@@ -4102,7 +4102,7 @@
           <t>TOYO-18P = ERREBI MZ22P113, TY43P80, ILCO LXP90P, SILCA MAZ23LP, TOY40P / 차종: LEXUS (TOYOTA) ® | 250 ES | 1989- | LEXUS (TOYOTA) ® | 300 E</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/toyo-18p/11379/</t>
         </is>
@@ -4129,7 +4129,7 @@
           <t>TP00HY-18P = ERREBI T00HYN13P, T00HYN13P, EZ KK10P, HY20PT, KK20, SILCA HYN20BTE</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/tp00hy-18p/11541/</t>
         </is>
@@ -4156,7 +4156,7 @@
           <t>TP00KI-7P = ERREBI T00KIA7P, EZ KK7, SILCA TOY49TE</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/tp00ki-7p/11560/</t>
         </is>
@@ -4183,7 +4183,7 @@
           <t>TP00KI-9P = ERREBI T00KIA10P, ILCO KK9-PT, SILCA KIA7BTE</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/tp00ki-9p/11562/</t>
         </is>
@@ -4210,7 +4210,7 @@
           <t>Silca KIA7 = JMA HY-18, 상품 코드 HYN#77</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2175&amp;controller=product</t>
         </is>
@@ -4237,7 +4237,7 @@
           <t>KEYDIY - LXP90 / TOY40 - Flip Key Blade - #13 - For Xhorse / Keydiy Universal Remote Flip Keys</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>https://www.uhs-hardware.com/products/keydiy-lxp90-toy40-flip-key-blade-13-for-xhorse-keydiy-universal-remote-flip-keys</t>
         </is>
@@ -4264,7 +4264,7 @@
           <t>TOY40/48 - #13 - UB10004 (Lexus / Toyota), TOY49 - #77 - UB10021 (Hyundai / Kia / Toyota / PSA)</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -4291,7 +4291,7 @@
           <t>Hyundai/Kia, Toyota HY22, TOY48 (Short) - 77# - Key Blade for Xhorse &amp; KeyDIY Universal Remotes (Pack of 10)</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>https://autorescuetools.com/products/77-hy22-toy48-shorty-hyundai-kia-toyota-key-blade-for-xhorse-keydiy-universal-remotes-pack-of-10x</t>
         </is>
@@ -4318,7 +4318,7 @@
           <t>Hyundai/Kia Keydiy KIA7 Flip Keyblade - Blade77</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>https://remkeys.com/product/hyundai-kia-keydiy-kia7-flip-keyblade-blade77-hykb12-remkeys/</t>
         </is>
@@ -4345,7 +4345,7 @@
           <t>TOYO-30P1 = ERREBI TY47P80, SILCA TOY48P / 차종: LEXUS (TOYOTA) ® | VARIOUS MODELS | - | SCION ® | VARIOUS MO</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/toyo-30p1/11414/</t>
         </is>
@@ -4372,7 +4372,7 @@
           <t>KEYDIY - TOY48 - Flip Key Blade - #77 - For Xhorse / Keydiy Universal Remote Flip Keys</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>https://www.uhs-hardware.com/products/keydiy-toy48-flip-key-blade-77-for-xhorse-keydiy-universal-remote-flip-keys</t>
         </is>
@@ -4399,7 +4399,7 @@
           <t>Hyundai/Kia, Toyota HY22, TOY48 (Short) - 77# - Key Blade for Xhorse &amp; KeyDIY Universal Remotes (Pack of 10)</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>https://autorescuetools.com/products/77-hy22-toy48-shorty-hyundai-kia-toyota-key-blade-for-xhorse-keydiy-universal-remotes-pack-of-10x</t>
         </is>
@@ -4426,7 +4426,7 @@
           <t>Cross Reference: TOYO-36, TOY48</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>https://www.key4.com/universal-key-blades-autel-ikey-remotes-toy48-toyo36</t>
         </is>
@@ -4476,7 +4476,7 @@
           <t>Ilco 제품 TOY48-GTK, TOY48-GTS, EB3-F-TOY48 (Ilco도 TOY48 이름 사용)</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
+      <c r="E17" s="6" t="inlineStr">
         <is>
           <t>https://www.key4.com/uploads/files/products/metal_keys/AC-ILC-KEYDIR13/Key_Blank_Directory_-_Edition_13.pdf</t>
         </is>
@@ -4503,7 +4503,7 @@
           <t>Blade for KEYDIY and Xhorse Remote - HY22 / TOY48</t>
         </is>
       </c>
-      <c r="E18" s="7" t="inlineStr">
+      <c r="E18" s="6" t="inlineStr">
         <is>
           <t>https://accessfobs.co.uk/products/copy-of-blade-for-keydiy-and-xhorse-remote-lexus-toyota-type-toy48</t>
         </is>
@@ -4553,7 +4553,7 @@
           <t>HY-13D = EZ HY15, ILCO X280</t>
         </is>
       </c>
-      <c r="E20" s="7" t="inlineStr">
+      <c r="E20" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/hy-13d/5824/</t>
         </is>
@@ -4580,7 +4580,7 @@
           <t>HY-11DP1 = ERREBI KIA4RP173, SILCA HYN14RDP / 차종: HYUNDAI (CANADA) ® | SANTAFE | 2007-2010 | HYUNDAI ® | CRETA</t>
         </is>
       </c>
-      <c r="E21" s="7" t="inlineStr">
+      <c r="E21" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/hy-11dp1/5814/</t>
         </is>
@@ -4607,7 +4607,7 @@
           <t>KEYDIY - HY15 - Flip Key Blade - #33 - For Xhorse / Keydiy Universal Remote Flip Keys</t>
         </is>
       </c>
-      <c r="E22" s="7" t="inlineStr">
+      <c r="E22" s="6" t="inlineStr">
         <is>
           <t>https://www.uhs-hardware.com/products/keydiy-hy15-flip-key-blade-33-for-xhorse-keydiy-universal-remote-flip-keys</t>
         </is>
@@ -4634,7 +4634,7 @@
           <t>HYN14R - #33 - UB10012 (Hyundai / Kia)</t>
         </is>
       </c>
-      <c r="E23" s="7" t="inlineStr">
+      <c r="E23" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -4661,7 +4661,7 @@
           <t>Silca HYN14R = JMA HY-11D, 상품 코드 HYN#33</t>
         </is>
       </c>
-      <c r="E24" s="7" t="inlineStr">
+      <c r="E24" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2143&amp;controller=product</t>
         </is>
@@ -4688,7 +4688,7 @@
           <t>Cross Reference: HY15, HY-13D, HYN14R</t>
         </is>
       </c>
-      <c r="E25" s="7" t="inlineStr">
+      <c r="E25" s="6" t="inlineStr">
         <is>
           <t>https://www.key4.com/hyundai-kia-flip-key-blade-hy15</t>
         </is>
@@ -4738,7 +4738,7 @@
           <t>HY-11 = EZ HY17, ILCO X282</t>
         </is>
       </c>
-      <c r="E27" s="7" t="inlineStr">
+      <c r="E27" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/hy-11/5812/</t>
         </is>
@@ -4765,7 +4765,7 @@
           <t>HY-11P3 = ERREBI KIA4P129, EZ HY17P, SILCA HYN14CP / 차종: HYUNDAI (USA) ® | VARIOUS MODELS | 2012- | HYUNDAI ® | VARIO</t>
         </is>
       </c>
-      <c r="E28" s="7" t="inlineStr">
+      <c r="E28" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/hy-11p3/5817/</t>
         </is>
@@ -4792,7 +4792,7 @@
           <t>KEYDIY - HYN14 - Flip Key Blade - #50 - For Xhorse / Keydiy Universal Remote Flip Keys</t>
         </is>
       </c>
-      <c r="E29" s="7" t="inlineStr">
+      <c r="E29" s="6" t="inlineStr">
         <is>
           <t>https://www.uhs-hardware.com/products/keydiy-hyn14-flip-key-blade-50-for-xhorse-keydiy-universal-remote-flip-keys</t>
         </is>
@@ -4819,7 +4819,7 @@
           <t>HYN14 - #50 - UB10015 (Hyundai / Kia)</t>
         </is>
       </c>
-      <c r="E30" s="7" t="inlineStr">
+      <c r="E30" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -4846,7 +4846,7 @@
           <t>Silca HYN14 = JMA HY-11, 상품 코드 HYN#50</t>
         </is>
       </c>
-      <c r="E31" s="7" t="inlineStr">
+      <c r="E31" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2144&amp;controller=product</t>
         </is>
@@ -4873,7 +4873,7 @@
           <t>10x New Uncut Universal Flip Remote Key Blade For Hyundai HY17 HYN14 HY-11</t>
         </is>
       </c>
-      <c r="E32" s="7" t="inlineStr">
+      <c r="E32" s="6" t="inlineStr">
         <is>
           <t>https://www.ebay.com/itm/313166504588</t>
         </is>
@@ -4900,7 +4900,7 @@
           <t>Ilco 디렉터리 13판 119·120쪽 HYUNDAI: HYN14-GTS (EZ HY16), HYN14FB (–), HYN14MH (–) — 반대 근거</t>
         </is>
       </c>
-      <c r="E33" s="7" t="inlineStr">
+      <c r="E33" s="6" t="inlineStr">
         <is>
           <t>https://www.key4.com/uploads/files/products/metal_keys/AC-ILC-KEYDIR13/Key_Blank_Directory_-_Edition_13.pdf</t>
         </is>
@@ -4927,7 +4927,7 @@
           <t>KIA RONDO 2007-2010: HY17-P / HYUNDAI ELANTRA 2006-2010: HY17-P</t>
         </is>
       </c>
-      <c r="E34" s="7" t="inlineStr">
+      <c r="E34" s="6" t="inlineStr">
         <is>
           <t>https://www.keycraze.com/ilco/2023-auto-truck-key-blank-reference.pdf</t>
         </is>
@@ -4954,7 +4954,7 @@
           <t>Hyundai Various Models Automotive X282 HY17 HY11 HY14U HYN14FH Key Blank (Silca HYN14FH = 이 줄)</t>
         </is>
       </c>
-      <c r="E35" s="7" t="inlineStr">
+      <c r="E35" s="6" t="inlineStr">
         <is>
           <t>https://www.ebay.com/itm/255108867180</t>
         </is>
@@ -4981,7 +4981,7 @@
           <t>HYN14/HY16 2-in-1 for Hyundai HY16 and Silca HYN14 by Original Lishi (공구 이름 = 두 블랭크용)</t>
         </is>
       </c>
-      <c r="E36" s="7" t="inlineStr">
+      <c r="E36" s="6" t="inlineStr">
         <is>
           <t>https://www.lockpicks.com/products/hyn14-hy16-2-in-1-for-hyundai-hy16-and-silca-hyn14-by-original-lishi</t>
         </is>
@@ -5031,7 +5031,7 @@
           <t>HY-12 = EZ HY16, ILCO X281</t>
         </is>
       </c>
-      <c r="E38" s="7" t="inlineStr">
+      <c r="E38" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/hy-12/5821/</t>
         </is>
@@ -5058,7 +5058,7 @@
           <t>HY-14 = EZ HY16</t>
         </is>
       </c>
-      <c r="E39" s="7" t="inlineStr">
+      <c r="E39" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/hy-14/5826/</t>
         </is>
@@ -5085,7 +5085,7 @@
           <t>KEYDIY - HY16 - Flip Key Blade - #36 - For Xhorse / Keydiy Universal Remote Flip Keys</t>
         </is>
       </c>
-      <c r="E40" s="7" t="inlineStr">
+      <c r="E40" s="6" t="inlineStr">
         <is>
           <t>https://www.uhs-hardware.com/products/keydiy-hy16-flip-key-blade-36-for-xhorse-keydiy-universal-remote-flip-keys</t>
         </is>
@@ -5112,7 +5112,7 @@
           <t>HY16 - #36 - UB10013 (Hyundai / Kia)</t>
         </is>
       </c>
-      <c r="E41" s="7" t="inlineStr">
+      <c r="E41" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -5139,7 +5139,7 @@
           <t>HY-12P3 = ERREBI HYN15P129, EZ HY16P / 차종: KIA ® | VARIOUS MODELS | -</t>
         </is>
       </c>
-      <c r="E42" s="7" t="inlineStr">
+      <c r="E42" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/hy-12p3/5822/</t>
         </is>
@@ -5166,7 +5166,7 @@
           <t>HYN15 - #34 - UB10069 (Hyundai / Kia)</t>
         </is>
       </c>
-      <c r="E43" s="7" t="inlineStr">
+      <c r="E43" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -5193,7 +5193,7 @@
           <t>Key4 HYN15 키날 사진, 각인 34</t>
         </is>
       </c>
-      <c r="E44" s="7" t="inlineStr">
+      <c r="E44" s="6" t="inlineStr">
         <is>
           <t>https://www.key4.com/uploads/files/products/key_blades/KB-KDY-HYN15/KB-KDY-HYN15_photo.jpg</t>
         </is>
@@ -5220,7 +5220,7 @@
           <t>Keydiy Xhorse Universal Flip Remote key Blade HY17 / HYN15 Hyundai Kia (#34)</t>
         </is>
       </c>
-      <c r="E45" s="7" t="inlineStr">
+      <c r="E45" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/keydiy-xhorse-universal-flip-remote-key-blade-hy17-hyn15-hyundai-kia-34</t>
         </is>
@@ -5247,7 +5247,7 @@
           <t>HY17/HYN15 2-in-1 (Service Key: Ilco HY17, Silca HYN15)</t>
         </is>
       </c>
-      <c r="E46" s="7" t="inlineStr">
+      <c r="E46" s="6" t="inlineStr">
         <is>
           <t>https://www.originallishi.com/2-in-1tools/hy17-hyn15-2-in-1/</t>
         </is>
@@ -5274,7 +5274,7 @@
           <t>Mr Li's Original HYN15 (HY17) 2in1 Pick &amp; Decoder for KIA</t>
         </is>
       </c>
-      <c r="E47" s="7" t="inlineStr">
+      <c r="E47" s="6" t="inlineStr">
         <is>
           <t>https://www.keyprint.co.uk/hyn15-kia-2in1-pick-and-decoder</t>
         </is>
@@ -5301,7 +5301,7 @@
           <t>ORIGINAL LISHI - HY17 HYN15 Hyundai / 2-in-1 Pick &amp; Decoder</t>
         </is>
       </c>
-      <c r="E48" s="7" t="inlineStr">
+      <c r="E48" s="6" t="inlineStr">
         <is>
           <t>https://www.uhs-hardware.com/products/original-lishi-hyundai-hy17-hyn15-2-in-1-pick-decoder-ag</t>
         </is>
@@ -5328,7 +5328,7 @@
           <t>LISHI HY17 / HYN15 / Hyundai / 2-in-1 Pick &amp; Decoder AG</t>
         </is>
       </c>
-      <c r="E49" s="7" t="inlineStr">
+      <c r="E49" s="6" t="inlineStr">
         <is>
           <t>https://www.mykeysupply.com/product/lishi-hy17-hyn15-hyundai-2-in-1-pick-decoder-ag/</t>
         </is>
@@ -5355,7 +5355,7 @@
           <t>KIA RIO 2006-2009: HY16-P / RIO (CANADA) 2006-2009: HYN15MH, HYN15-GTS</t>
         </is>
       </c>
-      <c r="E50" s="7" t="inlineStr">
+      <c r="E50" s="6" t="inlineStr">
         <is>
           <t>https://www.keycraze.com/ilco/2023-auto-truck-key-blank-reference.pdf</t>
         </is>
@@ -5382,7 +5382,7 @@
           <t>Silca HYN15CP key blank for KIA / Hyundai — Kia Rio 2006-2009</t>
         </is>
       </c>
-      <c r="E51" s="7" t="inlineStr">
+      <c r="E51" s="6" t="inlineStr">
         <is>
           <t>https://www.zieh-fix.com/en/key-blanks/silca-hyn15cp-key-blank-for-kia-hyundai.html</t>
         </is>
@@ -5409,7 +5409,7 @@
           <t>HYN15 MH Blade for Kia — KIA RIO 2006-2009</t>
         </is>
       </c>
-      <c r="E52" s="7" t="inlineStr">
+      <c r="E52" s="6" t="inlineStr">
         <is>
           <t>https://www.keyprint.co.uk/hyn15-mh-blade-for-kia2037</t>
         </is>
@@ -5436,7 +5436,7 @@
           <t>SILCA HYN15FH Flip Key Blade To Suit KIA (Rio 2006-2009)</t>
         </is>
       </c>
-      <c r="E53" s="7" t="inlineStr">
+      <c r="E53" s="6" t="inlineStr">
         <is>
           <t>https://www.aldridgesecurity.co.uk/silca-2619-silca-hyn15fh-flip-key-blade-to-suit-kia.html</t>
         </is>
@@ -5463,7 +5463,7 @@
           <t>Hyundai Aftermarket ILCO HY16-P Key Blank Fits Accent 2006-2011 &amp; Kia Rio 06-09</t>
         </is>
       </c>
-      <c r="E54" s="7" t="inlineStr">
+      <c r="E54" s="6" t="inlineStr">
         <is>
           <t>https://www.ebay.com/itm/Hyundai-Aftermarket-ILCO-HY16-P-Key-Blank-Fits-Accent-2006-2011-Kia-Rio-06-09-/321130159420</t>
         </is>
@@ -5490,7 +5490,7 @@
           <t>Flip Remote Key Blade For Hyundai HYN15 (엘란트라·세라토·i30)</t>
         </is>
       </c>
-      <c r="E55" s="7" t="inlineStr">
+      <c r="E55" s="6" t="inlineStr">
         <is>
           <t>https://www.key4.com/hyundai-flip-key-blade-hyn15</t>
         </is>
@@ -5540,7 +5540,7 @@
           <t>HY-19DP3 = EZ HY18P</t>
         </is>
       </c>
-      <c r="E57" s="7" t="inlineStr">
+      <c r="E57" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/hy-19dp3/5832/</t>
         </is>
@@ -5567,7 +5567,7 @@
           <t>TP00HY-19DP1 = ERREBI T00KIA8P, ILCO HYN17, SILCA HYN17BTE</t>
         </is>
       </c>
-      <c r="E58" s="7" t="inlineStr">
+      <c r="E58" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/tp00hy-19dp1/11543/</t>
         </is>
@@ -5594,7 +5594,7 @@
           <t>KEYDIY - HY18 - Flip Key Blade - #129 - For Xhorse / Keydiy Universal Remote Flip Keys</t>
         </is>
       </c>
-      <c r="E59" s="7" t="inlineStr">
+      <c r="E59" s="6" t="inlineStr">
         <is>
           <t>https://www.uhs-hardware.com/products/keydiy-hy18-flip-key-blade-129-for-xhorse-keydiy-universal-remote-flip-keys</t>
         </is>
@@ -5621,7 +5621,7 @@
           <t>HYN17 - #129 Y-16 - UB10031 (Hyundai / Kia)</t>
         </is>
       </c>
-      <c r="E60" s="7" t="inlineStr">
+      <c r="E60" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -5648,7 +5648,7 @@
           <t>Silca HYN17(상품명 "HY17") = JMA HY-19D, 상품 코드 HYN#129</t>
         </is>
       </c>
-      <c r="E61" s="7" t="inlineStr">
+      <c r="E61" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2177&amp;controller=product</t>
         </is>
@@ -5675,7 +5675,7 @@
           <t>Keydiy / Xhorse HYN17 #129 #Y16 - HYN20 - Kia16 Picanto Flip Key Blade (검색 결과)</t>
         </is>
       </c>
-      <c r="E62" s="7" t="inlineStr">
+      <c r="E62" s="6" t="inlineStr">
         <is>
           <t>https://keystation.co.uk/kia-hyn17-picanto-flip-key-blade</t>
         </is>
@@ -5702,7 +5702,7 @@
           <t>Keydiy Blade Kia HY18 (Y-16#), SKU KDY-INSERT 20</t>
         </is>
       </c>
-      <c r="E63" s="7" t="inlineStr">
+      <c r="E63" s="6" t="inlineStr">
         <is>
           <t>https://car-keys-remotes.acmelocksmith.com/products/item/-/Keydiy-Blade-Kia-HY18--Y-16----KDY-INSERT-20/24006</t>
         </is>
@@ -5752,7 +5752,7 @@
           <t>HY-19P3 = EZ HY18RP</t>
         </is>
       </c>
-      <c r="E65" s="7" t="inlineStr">
+      <c r="E65" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/hy-19p3/5834/</t>
         </is>
@@ -5779,7 +5779,7 @@
           <t>TP00HY-19P1 = ILCO HYN17RBTE, SILCA HYN17RBTE</t>
         </is>
       </c>
-      <c r="E66" s="7" t="inlineStr">
+      <c r="E66" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/tp00hy-19p1/11544/</t>
         </is>
@@ -5806,7 +5806,7 @@
           <t>KEYDIY - HY18R - Flip Key Blade - #130 - For Xhorse / Keydiy Universal Remote Flip Keys</t>
         </is>
       </c>
-      <c r="E67" s="7" t="inlineStr">
+      <c r="E67" s="6" t="inlineStr">
         <is>
           <t>https://www.uhs-hardware.com/products/keydiy-hy18r-flip-key-blade-130-for-xhorse-keydiy-universal-remote-flip-keys</t>
         </is>
@@ -5833,7 +5833,7 @@
           <t>HYN17R - #130 - UB10024 (Hyundai / Kia)</t>
         </is>
       </c>
-      <c r="E68" s="7" t="inlineStr">
+      <c r="E68" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -5860,7 +5860,7 @@
           <t>Silca HYN17R(상품명 "HY17R") = JMA HY-19, 상품 코드 HYN#130</t>
         </is>
       </c>
-      <c r="E69" s="7" t="inlineStr">
+      <c r="E69" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2178&amp;controller=product</t>
         </is>
@@ -5887,7 +5887,7 @@
           <t>KD Blank Key Blade Suitable For HYN17R, 키날에 130 각인</t>
         </is>
       </c>
-      <c r="E70" s="7" t="inlineStr">
+      <c r="E70" s="6" t="inlineStr">
         <is>
           <t>https://www.remotepro.com.au/products/kd-blank-key-blade-suitable-for-hyn17r</t>
         </is>
@@ -5937,7 +5937,7 @@
           <t>HY-21P3 = ILCO KK12P</t>
         </is>
       </c>
-      <c r="E72" s="7" t="inlineStr">
+      <c r="E72" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/hy-21p3/5840/</t>
         </is>
@@ -5964,7 +5964,7 @@
           <t>TP00HY-20P1 = ERREBI T00HYN14P, SILCA KIA9TE</t>
         </is>
       </c>
-      <c r="E73" s="7" t="inlineStr">
+      <c r="E73" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/tp00hy-20p1/11545/</t>
         </is>
@@ -5991,7 +5991,7 @@
           <t>KK12 - #156 Y-75 - UB10043 (Hyundai / Kia)</t>
         </is>
       </c>
-      <c r="E74" s="7" t="inlineStr">
+      <c r="E74" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -6018,7 +6018,7 @@
           <t>Keydiy / Xhorse Kia / Hyundai KK12 Flip Key Blade #156</t>
         </is>
       </c>
-      <c r="E75" s="7" t="inlineStr">
+      <c r="E75" s="6" t="inlineStr">
         <is>
           <t>https://www.mykeysupply.com/product/keydiy-xhorse-kk12-flip-key-blade-156/</t>
         </is>
@@ -6045,7 +6045,7 @@
           <t>KEYDIY - KK12 - Flip Key Blade - #Y75 - For Xhorse / Keydiy Universal Remote Flip Keys</t>
         </is>
       </c>
-      <c r="E76" s="7" t="inlineStr">
+      <c r="E76" s="6" t="inlineStr">
         <is>
           <t>https://www.uhs-hardware.com/products/keydiy-kk12-flip-key-blade-y75-for-xhorse-keydiy-universal-remote-flip-keys</t>
         </is>
@@ -6072,7 +6072,7 @@
           <t>Silca KIA9TE = JMA HY-20, 키날에 156 각인</t>
         </is>
       </c>
-      <c r="E77" s="7" t="inlineStr">
+      <c r="E77" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2174&amp;controller=product</t>
         </is>
@@ -6099,7 +6099,7 @@
           <t>KEYDIY - KK12 Key Blade #Y75 for Xhorse / Keydiy Universal Key Fob</t>
         </is>
       </c>
-      <c r="E78" s="7" t="inlineStr">
+      <c r="E78" s="6" t="inlineStr">
         <is>
           <t>https://www.locksmithkeyless.com/products/keydiy-kk12-key-blade-y75-for-xhorse-keydiy-universal-key-fob</t>
         </is>
@@ -6126,7 +6126,7 @@
           <t>KEYDIY Key Blade — Kia / Hyundai KK12 #156 (KD-HY-156)</t>
         </is>
       </c>
-      <c r="E79" s="7" t="inlineStr">
+      <c r="E79" s="6" t="inlineStr">
         <is>
           <t>https://keydirect.ca/product/keydiy-key-blade-kia-kk12-156-kd-hy-156/</t>
         </is>
@@ -6153,7 +6153,7 @@
           <t>Keydiy / Xhorse Kia / Hyundai KK12 Flip Key Blade #156</t>
         </is>
       </c>
-      <c r="E80" s="7" t="inlineStr">
+      <c r="E80" s="6" t="inlineStr">
         <is>
           <t>https://www.mykeysupply.com/product/keydiy-xhorse-kk12-flip-key-blade-156/</t>
         </is>
@@ -6203,7 +6203,7 @@
           <t>HY-10 = ERREBI HYN11, EZ HY14, ILCO X236, SILCA HYN11 / 차종: HYUNDAI ® | VARIOUS MODELS | -</t>
         </is>
       </c>
-      <c r="E82" s="7" t="inlineStr">
+      <c r="E82" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/hy-10/5809/</t>
         </is>
@@ -6230,7 +6230,7 @@
           <t>KEYDIY - HY14 - Flip Key Blade - #15 - For Xhorse / Keydiy Universal Remote Flip Keys</t>
         </is>
       </c>
-      <c r="E83" s="7" t="inlineStr">
+      <c r="E83" s="6" t="inlineStr">
         <is>
           <t>https://www.uhs-hardware.com/products/keydiy-hy14-flip-key-blade-15-for-xhorse-keydiy-universal-remote-flip-keys</t>
         </is>
@@ -6257,7 +6257,7 @@
           <t>HYN11 Xhorse KeyDIY Flip Key Blade Replacement #15</t>
         </is>
       </c>
-      <c r="E84" s="7" t="inlineStr">
+      <c r="E84" s="6" t="inlineStr">
         <is>
           <t>https://www.bestkeysupply.com/products/hyn11-xhorse-keydiy-universal-flipkey-insert-26-b149bks</t>
         </is>
@@ -6284,7 +6284,7 @@
           <t>HY-4P2 = ERREBI HYN11P129, EZ HY14-P, SILCA HYN11CP / 차종: HYUNDAI ® | ELANTRA | 1991-1996 | HYUNDAI ® | LANTRA | 1991-</t>
         </is>
       </c>
-      <c r="E85" s="7" t="inlineStr">
+      <c r="E85" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/hy-4p2/5863/</t>
         </is>
@@ -6311,7 +6311,7 @@
           <t>Blank reference: Hyundai HY14/ HY11/HYN6, Blade number 15 (한 상품)</t>
         </is>
       </c>
-      <c r="E86" s="7" t="inlineStr">
+      <c r="E86" s="6" t="inlineStr">
         <is>
           <t>https://accessfobs.co.uk/products/blade-for-keydiy-and-xhorse-remote-hy14</t>
         </is>
@@ -6361,7 +6361,7 @@
           <t>HY-4 = ERREBI HYN1, EZ HY6, ILCO X216, SILCA HYN6 / 차종: HYUNDAI ® | ELANTRA | 1991-1996 | HYUNDAI ® | LANTRA | 1991-</t>
         </is>
       </c>
-      <c r="E88" s="7" t="inlineStr">
+      <c r="E88" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/hy-4/5858/</t>
         </is>
@@ -6388,7 +6388,7 @@
           <t>HYN6 - #15 - UB10005 (Hyundai / Kia)</t>
         </is>
       </c>
-      <c r="E89" s="7" t="inlineStr">
+      <c r="E89" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -6415,7 +6415,7 @@
           <t>Silca HYN6 = JMA HY-4, 상품 코드 HYN#15</t>
         </is>
       </c>
-      <c r="E90" s="7" t="inlineStr">
+      <c r="E90" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2142&amp;controller=product</t>
         </is>
@@ -6442,7 +6442,7 @@
           <t>Cross Reference: HYN6, HY-9</t>
         </is>
       </c>
-      <c r="E91" s="7" t="inlineStr">
+      <c r="E91" s="6" t="inlineStr">
         <is>
           <t>https://www.key4.com/hyundai-kia-flip-key-blade-hyn6-hy-9</t>
         </is>
@@ -6469,7 +6469,7 @@
           <t>HY-4P2 = ERREBI HYN11P129, EZ HY14-P, SILCA HYN11CP / 차종: HYUNDAI ® | ELANTRA | 1991-1996 | HYUNDAI ® | LANTRA | 1991-</t>
         </is>
       </c>
-      <c r="E92" s="7" t="inlineStr">
+      <c r="E92" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/hy-4p2/5863/</t>
         </is>
@@ -6496,7 +6496,7 @@
           <t>Blank reference: Hyundai HY14/ HY11/HYN6, Blade number 15 (한 상품)</t>
         </is>
       </c>
-      <c r="E93" s="7" t="inlineStr">
+      <c r="E93" s="6" t="inlineStr">
         <is>
           <t>https://accessfobs.co.uk/products/blade-for-keydiy-and-xhorse-remote-hy14</t>
         </is>
@@ -6546,7 +6546,7 @@
           <t xml:space="preserve">HY-6D = ERREBI HYN10R, HYN4R, EZ HY12, HY12, ILCO X232, X232, SILCA HYN8R, HYN7R / 차종: HYUNDAI ® | SONATA (USA) | 1993-1995 | HYUNDAI ® | SONICA | </t>
         </is>
       </c>
-      <c r="E95" s="7" t="inlineStr">
+      <c r="E95" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/hy-6d/5871/</t>
         </is>
@@ -6573,7 +6573,7 @@
           <t>HYN7R Xhorse KeyDIY Flip Key Blade Replacement #29</t>
         </is>
       </c>
-      <c r="E96" s="7" t="inlineStr">
+      <c r="E96" s="6" t="inlineStr">
         <is>
           <t>https://www.bestkeysupply.com/products/hyn7r-xhorse-keydiy-universal-flipkey-insert-29-b150bks</t>
         </is>
@@ -6600,7 +6600,7 @@
           <t>Xhorse – Keydiy Kia HY12 / HYN7R Key Blade #29</t>
         </is>
       </c>
-      <c r="E97" s="7" t="inlineStr">
+      <c r="E97" s="6" t="inlineStr">
         <is>
           <t>https://www.mykeysupply.com/product/xhorse-keydiy-kia-hy12-hyn7r-key-blade-29/</t>
         </is>
@@ -6627,7 +6627,7 @@
           <t>Flip Remote Key Blade For Hyundai Ssang Yong HYN10R</t>
         </is>
       </c>
-      <c r="E98" s="7" t="inlineStr">
+      <c r="E98" s="6" t="inlineStr">
         <is>
           <t>https://www.key4.com/hyundai-ssang-yong-flip-key-blade-hyn10r</t>
         </is>
@@ -6650,7 +6650,7 @@
           <t>KI-3D = EZ KK3, KK3, ILCO X253, X253, SILCA KIA3R</t>
         </is>
       </c>
-      <c r="E99" s="7" t="inlineStr">
+      <c r="E99" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/ki-3d/6874/</t>
         </is>
@@ -6673,7 +6673,7 @@
           <t>Silca KIA3R = Ilco X253 (KK3)</t>
         </is>
       </c>
-      <c r="E100" s="7" t="inlineStr">
+      <c r="E100" s="6" t="inlineStr">
         <is>
           <t>https://www.key4.com/uploads/files/products/metal_keys/AC-ILC-KEYDIR13/Key_Blank_Directory_-_Edition_13.pdf</t>
         </is>
@@ -6696,7 +6696,7 @@
           <t>Silca KIA3R = JMA KI-2D, 상품 코드 HYN#131</t>
         </is>
       </c>
-      <c r="E101" s="7" t="inlineStr">
+      <c r="E101" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2173&amp;controller=product</t>
         </is>
@@ -6723,7 +6723,7 @@
           <t>HY-9P2 = ERREBI HYN12P129, SILCA HYN12CP / 차종: HYUNDAI ® | STAREX | 1998-</t>
         </is>
       </c>
-      <c r="E102" s="7" t="inlineStr">
+      <c r="E102" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/hy-9p2/5879/</t>
         </is>
@@ -6750,7 +6750,7 @@
           <t>Cross Reference: HYN12, TP00HY-9.P1</t>
         </is>
       </c>
-      <c r="E103" s="7" t="inlineStr">
+      <c r="E103" s="6" t="inlineStr">
         <is>
           <t>https://www.key4.com/flip-remote-key-blade-for-hyundai-hyn12</t>
         </is>
@@ -6777,7 +6777,7 @@
           <t>Key4 HYN12 키날 사진, 각인 30</t>
         </is>
       </c>
-      <c r="E104" s="7" t="inlineStr">
+      <c r="E104" s="6" t="inlineStr">
         <is>
           <t>https://www.key4.com/uploads/files/products/xhorse_keydiy_key_blades/KB-UNV-HYN12/KB-UNV-HYN12-1.jpg</t>
         </is>
@@ -6842,7 +6842,7 @@
           <t>Cross Reference: HYN6R</t>
         </is>
       </c>
-      <c r="E107" s="7" t="inlineStr">
+      <c r="E107" s="6" t="inlineStr">
         <is>
           <t>https://www.key4.com/flip-remote-key-blade-for-hyundai-hyn6r</t>
         </is>
@@ -6865,7 +6865,7 @@
           <t>Key4 HYN6R 키날 사진, 각인 08 (다른 판매처 번호와 다름)</t>
         </is>
       </c>
-      <c r="E108" s="7" t="inlineStr">
+      <c r="E108" s="6" t="inlineStr">
         <is>
           <t>https://www.key4.com/uploads/files/products/xhorse_keydiy_key_blades/KB-UNV-HYN6R/KB-UNV-HYN6R-1.jpg</t>
         </is>
@@ -6888,7 +6888,7 @@
           <t>[KDHY131ES01] BLADE HYUNDAI, KIA FOR KEYDIY HYN6R, XHORSE #131</t>
         </is>
       </c>
-      <c r="E109" s="7" t="inlineStr">
+      <c r="E109" s="6" t="inlineStr">
         <is>
           <t>https://www.key-code.com/en/shop/kdhy131es01-blade-hyundai-kia-for-keydiy-hyn6r-xhorse-131-8706</t>
         </is>
@@ -6938,7 +6938,7 @@
           <t>HY-5 = ERREBI HYN6, EZ HY13, ILCO X235, SILCA HYN10 / 차종: HYUNDAI ® | ACCENT | 1994-1996 | HYUNDAI ® | EXCEL | 1994-19</t>
         </is>
       </c>
-      <c r="E111" s="7" t="inlineStr">
+      <c r="E111" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/hy-5/5866/</t>
         </is>
@@ -6965,7 +6965,7 @@
           <t>Silca HYN10 = JMA HY-5, 상품 코드 HYN#TS-58</t>
         </is>
       </c>
-      <c r="E112" s="7" t="inlineStr">
+      <c r="E112" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2176&amp;controller=product</t>
         </is>
@@ -6992,7 +6992,7 @@
           <t>HYN10, Blade number 92#, For Ssangyong</t>
         </is>
       </c>
-      <c r="E113" s="7" t="inlineStr">
+      <c r="E113" s="6" t="inlineStr">
         <is>
           <t>https://accessfobs.co.uk/products/blade-for-keydiy-and-xhorse-remote-hyn10</t>
         </is>
@@ -7019,7 +7019,7 @@
           <t>Keydiy / Xhorse HYN10 #92 Flip Key Blade (검색 결과)</t>
         </is>
       </c>
-      <c r="E114" s="7" t="inlineStr">
+      <c r="E114" s="6" t="inlineStr">
         <is>
           <t>https://keystation.co.uk/keydiy-xhorse-hyn10-92-flip-key-blade</t>
         </is>
@@ -7046,7 +7046,7 @@
           <t>Hyundai/SsangYong Keydiy HYN10 Flip Keyblade - Blade28 (사진 각인 28)</t>
         </is>
       </c>
-      <c r="E115" s="7" t="inlineStr">
+      <c r="E115" s="6" t="inlineStr">
         <is>
           <t>https://remkeys.com/product/hyundai-ssangyong-keydiy-hyn10-flip-keyblade-blade28-hykb13-remkeys/</t>
         </is>
@@ -7073,7 +7073,7 @@
           <t>KEYDIY Remote Flip Key Blade for Ssangyong (92#)</t>
         </is>
       </c>
-      <c r="E116" s="7" t="inlineStr">
+      <c r="E116" s="6" t="inlineStr">
         <is>
           <t>https://www.locksmithkeyless.com/products/keydiy-remote-flip-key-blade-for-ssangyong-92</t>
         </is>
@@ -7100,7 +7100,7 @@
           <t>KeyDiy KD #92 Metal Blank Uncut Flip Key Remote Blade for Ssangyong</t>
         </is>
       </c>
-      <c r="E117" s="7" t="inlineStr">
+      <c r="E117" s="6" t="inlineStr">
         <is>
           <t>https://www.tlkeys.com/products/KeyDiy-KD-92-Metal-Blank-Uncut-Flip-Key-Remote-Blade-for-Ss-33117</t>
         </is>
@@ -7127,7 +7127,7 @@
           <t>3D Group DIYB45 (검색 결과: HYN10 92#)</t>
         </is>
       </c>
-      <c r="E118" s="7" t="inlineStr">
+      <c r="E118" s="6" t="inlineStr">
         <is>
           <t>https://3dgroupuk.com/product/view/DIYB45</t>
         </is>
@@ -7177,7 +7177,7 @@
           <t>Xhorse VVDI KeyDiy KD Remote Key Blade Hyundai Ssangyong, Blade Profile HYN10R, P/N 137</t>
         </is>
       </c>
-      <c r="E120" s="7" t="inlineStr">
+      <c r="E120" s="6" t="inlineStr">
         <is>
           <t>https://www.tlkeys.com/products/Keydiy-137-Hyundai-Ssangyong-Key-Blade-33282</t>
         </is>
@@ -7204,7 +7204,7 @@
           <t>SsangYong Keydiy Flip Keyblade - Blade137 (사진 각인 137)</t>
         </is>
       </c>
-      <c r="E121" s="7" t="inlineStr">
+      <c r="E121" s="6" t="inlineStr">
         <is>
           <t>https://remkeys.com/product/ssangyong-keydiy-flip-keyblade-blade137-sykb01-remkeys/</t>
         </is>
@@ -7231,7 +7231,7 @@
           <t>Uncut Universal Flip Remote Key Blade Hyundai Ssang Yong Type HYN10R (번호 미표기)</t>
         </is>
       </c>
-      <c r="E122" s="7" t="inlineStr">
+      <c r="E122" s="6" t="inlineStr">
         <is>
           <t>https://www.key4.com/hyundai-ssang-yong-flip-key-blade-hyn10r</t>
         </is>
@@ -7273,7 +7273,7 @@
           <t>HY-17 = ERREBI HYN9, EZ HY4, ILCO X187, SILCA HYN4</t>
         </is>
       </c>
-      <c r="E124" s="7" t="inlineStr">
+      <c r="E124" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/hy-17/5829/</t>
         </is>
@@ -7296,7 +7296,7 @@
           <t>HY-3P2 = ERREBI HYN9P107, SSA1P107, EZ HY4-P, HY4P, ILCO HY4P, SILCA HYN4P, SSY2AP / 차종: HYUNDAI ® | SONATA | 1989-1990 | SSANGYONG ® | MUSSO | 1995-</t>
         </is>
       </c>
-      <c r="E125" s="7" t="inlineStr">
+      <c r="E125" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/hy-3p2/5852/</t>
         </is>
@@ -7346,7 +7346,7 @@
           <t>SSA-1P1 = ERREBI SSA2P107, SILCA SSY3* / 차종: SSANGYONG ® | VARIOUS MODELS | -</t>
         </is>
       </c>
-      <c r="E127" s="7" t="inlineStr">
+      <c r="E127" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/ssa-1p1/10705/</t>
         </is>
@@ -7373,7 +7373,7 @@
           <t>SSY3 - #92 - UB10063 (SsangYong)</t>
         </is>
       </c>
-      <c r="E128" s="7" t="inlineStr">
+      <c r="E128" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -7400,7 +7400,7 @@
           <t>Keydiy / Xhorse SSY3 #58 Flip Key Blade</t>
         </is>
       </c>
-      <c r="E129" s="7" t="inlineStr">
+      <c r="E129" s="6" t="inlineStr">
         <is>
           <t>https://keystation.co.uk/keydiy-xhorse-ssy3-58-flip-key-blade</t>
         </is>
@@ -7427,7 +7427,7 @@
           <t>Silca SSY3 = JMA SSA-1, 상품 코드 SSA#120</t>
         </is>
       </c>
-      <c r="E130" s="7" t="inlineStr">
+      <c r="E130" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2180&amp;controller=product</t>
         </is>
@@ -7454,7 +7454,7 @@
           <t>KeyDIY Ssangyong Universal Flip Key Blade (#120)</t>
         </is>
       </c>
-      <c r="E131" s="7" t="inlineStr">
+      <c r="E131" s="6" t="inlineStr">
         <is>
           <t>https://keyinnovations.com/keydiy-blade-ssangyong-120/</t>
         </is>
@@ -7481,7 +7481,7 @@
           <t>Flip Key Blade - SSANGYONG (Like: SSA-1 / SSY3) - Double Sided, Art ID SSA#120</t>
         </is>
       </c>
-      <c r="E132" s="7" t="inlineStr">
+      <c r="E132" s="6" t="inlineStr">
         <is>
           <t>https://www.sglocks.com.au/product/15636-flip-key-blade-ssangyong-like-ssa-1-ssy3-double-sided</t>
         </is>
@@ -7508,7 +7508,7 @@
           <t>Keydiy Ssangyong 120 blade</t>
         </is>
       </c>
-      <c r="E133" s="7" t="inlineStr">
+      <c r="E133" s="6" t="inlineStr">
         <is>
           <t>https://topkey.lt/new-products/5757-Keydiy-Ssangyong-120-blade.html</t>
         </is>
@@ -7535,7 +7535,7 @@
           <t xml:space="preserve">TOYO-15 = ERREBI TY37R, TY38R, EZ TR47, TR47, ILCO X217, X217, SILCA TOY43, TOY44 / 차종: GM (CHEVROLET) ® | COLORADO | 2004- | TOYOTA ® | 4 RUNNER | </t>
         </is>
       </c>
-      <c r="E134" s="7" t="inlineStr">
+      <c r="E134" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/toyo-15/11357/</t>
         </is>
@@ -7562,7 +7562,7 @@
           <t>KEYDIY - TR47 - Flip Key Blade - #02 - For Xhorse / Keydiy Universal Remote Flip Keys</t>
         </is>
       </c>
-      <c r="E135" s="7" t="inlineStr">
+      <c r="E135" s="6" t="inlineStr">
         <is>
           <t>https://www.uhs-hardware.com/products/keydiy-tr47-flip-key-blade-02-for-xhorse-keydiy-universal-remote-flip-keys</t>
         </is>
@@ -7589,7 +7589,7 @@
           <t>TOY43 - #02 - UB10001 (Toyota / Scion)</t>
         </is>
       </c>
-      <c r="E136" s="7" t="inlineStr">
+      <c r="E136" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -7616,7 +7616,7 @@
           <t>Silca TOY43 = JMA TOYO-15, 키날에 02 각인</t>
         </is>
       </c>
-      <c r="E137" s="7" t="inlineStr">
+      <c r="E137" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2152&amp;controller=product</t>
         </is>
@@ -7643,7 +7643,7 @@
           <t>Silca TOY43 = Ilco X217 (TR47)</t>
         </is>
       </c>
-      <c r="E138" s="7" t="inlineStr">
+      <c r="E138" s="6" t="inlineStr">
         <is>
           <t>https://www.key4.com/uploads/files/products/metal_keys/AC-ILC-KEYDIR13/Key_Blank_Directory_-_Edition_13.pdf</t>
         </is>
@@ -7670,7 +7670,7 @@
           <t>TOYO-19P = ERREBI TY45P79, SILCA TOY47BP / 차종: TOYOTA ® | CARINA | 1994-</t>
         </is>
       </c>
-      <c r="E139" s="7" t="inlineStr">
+      <c r="E139" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/toyo-19p/11382/</t>
         </is>
@@ -7697,7 +7697,7 @@
           <t>TOY47 - #177 Y-22 - UB10035 (Toyota)</t>
         </is>
       </c>
-      <c r="E140" s="7" t="inlineStr">
+      <c r="E140" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -7724,7 +7724,7 @@
           <t>KEYDIY - TOY47 - Flip Key Blade - #Y-22 - For Xhorse / Keydiy Universal Remote Flip Keys</t>
         </is>
       </c>
-      <c r="E141" s="7" t="inlineStr">
+      <c r="E141" s="6" t="inlineStr">
         <is>
           <t>https://www.uhs-hardware.com/products/keydiy-toy47-flip-key-blade-y-22-for-xhorse-keydiy-universal-remote-flip-keys</t>
         </is>
@@ -7751,7 +7751,7 @@
           <t>TOY47 TOYO-19, Blank number 177#. Y-22# 버전은 홈 모양은 같고 뒤쪽 결합부가 다름</t>
         </is>
       </c>
-      <c r="E142" s="7" t="inlineStr">
+      <c r="E142" s="6" t="inlineStr">
         <is>
           <t>https://accessfobs.co.uk/products/blade-for-keydiy-and-xhorse-remote-toy47-177</t>
         </is>
@@ -7778,7 +7778,7 @@
           <t>TOY47 TOYO-19, Blank number Y-22. 177# 버전과 홈 모양은 같고 뒤쪽 결합부가 다름</t>
         </is>
       </c>
-      <c r="E143" s="7" t="inlineStr">
+      <c r="E143" s="6" t="inlineStr">
         <is>
           <t>https://accessfobs.co.uk/products/blade-for-keydiy-and-xhorse-remote-toy47-y-22</t>
         </is>
@@ -7805,7 +7805,7 @@
           <t>TOYO-20D = ERREBI TY35R, EZ TR40, ILCO X174, SILCA TOY38R / 차종: TOYOTA ® | 4 RUNNER | 1990-1991 | TOYOTA ® | CARINA | 1990-1</t>
         </is>
       </c>
-      <c r="E144" s="7" t="inlineStr">
+      <c r="E144" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/toyo-20d/11388/</t>
         </is>
@@ -7832,7 +7832,7 @@
           <t>TOYO-9 = ERREBI TY35R, ILCO X174, SILCA TOY38R / 차종: TOYOTA ® | 4 RUNNER | 1990-1991 | TOYOTA ® | CARINA | 1990-1</t>
         </is>
       </c>
-      <c r="E145" s="7" t="inlineStr">
+      <c r="E145" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/toyo-9/11443/</t>
         </is>
@@ -7859,7 +7859,7 @@
           <t>TOY38R Xhorse KeyDIY Flip Key Blade Replacement #08</t>
         </is>
       </c>
-      <c r="E146" s="7" t="inlineStr">
+      <c r="E146" s="6" t="inlineStr">
         <is>
           <t>https://www.bestkeysupply.com/products/toy38r-xhorse-keydiy-universal-flipkey-insert-08-b153bks</t>
         </is>
@@ -7886,7 +7886,7 @@
           <t>TOY38R Kia Daihatsu, Blank number 08#</t>
         </is>
       </c>
-      <c r="E147" s="7" t="inlineStr">
+      <c r="E147" s="6" t="inlineStr">
         <is>
           <t>https://accessfobs.co.uk/products/blade-for-keydiy-xhorse-remote-for-toy38r-kia-daihatsu</t>
         </is>
@@ -7913,7 +7913,7 @@
           <t>Flip Remote Key Blade TOY38R 08# Metal Uncut Blank For Daihatsu FIAT PALIO Jinbei Haise KIA Carnival (검색 결과)</t>
         </is>
       </c>
-      <c r="E148" s="7" t="inlineStr">
+      <c r="E148" s="6" t="inlineStr">
         <is>
           <t>https://xienstore.com/collections/keydiy-blade</t>
         </is>
@@ -7936,7 +7936,7 @@
           <t>TOYO-10P1 = ERREBI TY42P79, SILCA TOY42P / 차종: TOYOTA ® | CELICA | 1990-1995 | TOYOTA ® | CELICA 4WD | 1990</t>
         </is>
       </c>
-      <c r="E149" s="7" t="inlineStr">
+      <c r="E149" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/toyo-10p1/11325/</t>
         </is>
@@ -7959,7 +7959,7 @@
           <t>Silca TOY42 = Ilco X212 (TR46)</t>
         </is>
       </c>
-      <c r="E150" s="7" t="inlineStr">
+      <c r="E150" s="6" t="inlineStr">
         <is>
           <t>https://www.key4.com/uploads/files/products/metal_keys/AC-ILC-KEYDIR13/Key_Blank_Directory_-_Edition_13.pdf</t>
         </is>
@@ -7982,7 +7982,7 @@
           <t>KeyDiy Xhorse Remote Key Blade For Toyota TOY42</t>
         </is>
       </c>
-      <c r="E151" s="7" t="inlineStr">
+      <c r="E151" s="6" t="inlineStr">
         <is>
           <t>https://abkeys.com/products/toyota-flip-remote-key-blade-toy42-for-kd-xhorse-remote-blade-2142</t>
         </is>
@@ -8009,7 +8009,7 @@
           <t>TOYO-33D = ERREBI TY40R, EZ TR44, ILCO X211, SILCA TOY41R</t>
         </is>
       </c>
-      <c r="E152" s="7" t="inlineStr">
+      <c r="E152" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/toyo-33d/11416/</t>
         </is>
@@ -8036,7 +8036,7 @@
           <t>TOY41R - #21 Y-21 - UB10034 (Toyota / Daihatsu)</t>
         </is>
       </c>
-      <c r="E153" s="7" t="inlineStr">
+      <c r="E153" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -8063,7 +8063,7 @@
           <t>Toyota TOY41 DH04 (TR41) Blade Y-21#</t>
         </is>
       </c>
-      <c r="E154" s="7" t="inlineStr">
+      <c r="E154" s="6" t="inlineStr">
         <is>
           <t>https://keyinnovations.com/products/keyless2go-toyota-toy41-dh04-tr41-blade-y-21</t>
         </is>
@@ -8090,7 +8090,7 @@
           <t>Keydiy Xhorse Universal Flip Remote key Blade Toy41R / DH4R (#21) Toyota</t>
         </is>
       </c>
-      <c r="E155" s="7" t="inlineStr">
+      <c r="E155" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/keydiy-xhorse-universal-flip-remote-key-blade-hummer-isuzu-toy43r-1</t>
         </is>
@@ -8117,7 +8117,7 @@
           <t>Silca TOY41R = Ilco X211 (TR44)</t>
         </is>
       </c>
-      <c r="E156" s="7" t="inlineStr">
+      <c r="E156" s="6" t="inlineStr">
         <is>
           <t>https://www.key4.com/uploads/files/products/metal_keys/AC-ILC-KEYDIR13/Key_Blank_Directory_-_Edition_13.pdf</t>
         </is>
@@ -8144,7 +8144,7 @@
           <t>Xhorse VVDI Universal Flip Remote key Blade Toy41R Toyota (21 toy41 key blade)</t>
         </is>
       </c>
-      <c r="E157" s="7" t="inlineStr">
+      <c r="E157" s="6" t="inlineStr">
         <is>
           <t>https://www.nistech.nz/product-page/21-toy41-key-blade-for-toyota</t>
         </is>
@@ -8171,7 +8171,7 @@
           <t>KDIY key Blade 21# TOY41 for Toyota</t>
         </is>
       </c>
-      <c r="E158" s="7" t="inlineStr">
+      <c r="E158" s="6" t="inlineStr">
         <is>
           <t>https://chipkeysupply.com/products/kdiy-key-blade-21-toy41-for-toyota</t>
         </is>
@@ -8198,7 +8198,7 @@
           <t>Keydiy / Xhorse TOY41R #Y21 Flip key Blade</t>
         </is>
       </c>
-      <c r="E159" s="7" t="inlineStr">
+      <c r="E159" s="6" t="inlineStr">
         <is>
           <t>https://keystation.co.uk/keydiy-xhorse-toy41r-y21-flip-key-blade</t>
         </is>
@@ -8225,7 +8225,7 @@
           <t>Keyless2Go Toyota TOY41 DH04 (TR41) Blade Y-21#</t>
         </is>
       </c>
-      <c r="E160" s="7" t="inlineStr">
+      <c r="E160" s="6" t="inlineStr">
         <is>
           <t>https://keyinnovations.com/products/keyless2go-toyota-toy41-dh04-tr41-blade-y-21</t>
         </is>
@@ -8252,7 +8252,7 @@
           <t>TOYO-40D = EZ B110, ILCO P1114, SILCA TOY43R / 차종: GM (CHEVROLET) ® | VARIOUS MODELS | - | TOYOTA ® | VARIOUS M</t>
         </is>
       </c>
-      <c r="E161" s="7" t="inlineStr">
+      <c r="E161" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/toyo-40d/11425/</t>
         </is>
@@ -8279,7 +8279,7 @@
           <t>GM-38 = EZ B110, ILCO P1114</t>
         </is>
       </c>
-      <c r="E162" s="7" t="inlineStr">
+      <c r="E162" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/gm-38/5090/</t>
         </is>
@@ -8306,7 +8306,7 @@
           <t>ISU-3D = SILCA TOY43R / 차종: ISUZU ® | D-MAX | 2002-2006 | ISUZU ® | I-290 | 2007- | ISUZ</t>
         </is>
       </c>
-      <c r="E163" s="7" t="inlineStr">
+      <c r="E163" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/isu-3d/6091/</t>
         </is>
@@ -8333,7 +8333,7 @@
           <t>KEYDIY - B110 - Flip Key Blade - #69 - For Xhorse / Keydiy Universal Remote Flip Keys</t>
         </is>
       </c>
-      <c r="E164" s="7" t="inlineStr">
+      <c r="E164" s="6" t="inlineStr">
         <is>
           <t>https://www.uhs-hardware.com/products/keydiy-b110-flip-key-blade-69-for-xhorse-keydiy-universal-remote-flip-keys</t>
         </is>
@@ -8360,7 +8360,7 @@
           <t>TOY43R - #69 - UB10019 (Subaru / GM / Isuzu)</t>
         </is>
       </c>
-      <c r="E165" s="7" t="inlineStr">
+      <c r="E165" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -8387,7 +8387,7 @@
           <t>Silca TOY43R = JMA ISU-3D, 상품 코드 ISU#69</t>
         </is>
       </c>
-      <c r="E166" s="7" t="inlineStr">
+      <c r="E166" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2163&amp;controller=product</t>
         </is>
@@ -8437,7 +8437,7 @@
           <t>DAT-15 = ERREBI NS8, EZ DA35, ILCO X238, SILCA NSN14 / 차종: NISSAN ® | CEDRIC | 1995-1997 | NISSAN ® | GLORIA | 1995-199</t>
         </is>
       </c>
-      <c r="E168" s="7" t="inlineStr">
+      <c r="E168" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/dat-15/3358/</t>
         </is>
@@ -8464,7 +8464,7 @@
           <t>DAT-16 = ERREBI NS11, EZ DA34, ILCO X237 / 차종: CHEVROLET ® | VARIOUS MODELS | - | INFINITI (NISSAN) ® | VAR</t>
         </is>
       </c>
-      <c r="E169" s="7" t="inlineStr">
+      <c r="E169" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/dat-16/3367/</t>
         </is>
@@ -8491,7 +8491,7 @@
           <t>KEYDIY - DA34 / NSN14 - Flip Key Blade - #22 - For Xhorse / Keydiy Universal Remote Flip Keys</t>
         </is>
       </c>
-      <c r="E170" s="7" t="inlineStr">
+      <c r="E170" s="6" t="inlineStr">
         <is>
           <t>https://www.uhs-hardware.com/products/keydiy-da34-nsn14-flip-key-blade-22-for-xhorse-keydiy-universal-remote-flip-keys</t>
         </is>
@@ -8518,7 +8518,7 @@
           <t>NSN14 - #22 - UB10008 (Nissan / Infiniti)</t>
         </is>
       </c>
-      <c r="E171" s="7" t="inlineStr">
+      <c r="E171" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -8545,7 +8545,7 @@
           <t>Silca NSN14 = JMA DAT-15, 상품 코드 DAT#22</t>
         </is>
       </c>
-      <c r="E172" s="7" t="inlineStr">
+      <c r="E172" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2136&amp;controller=product</t>
         </is>
@@ -8595,7 +8595,7 @@
           <t>DAT-10 = ERREBI NS5, EZ DA38, ILCO X243, SILCA NSN11 / 차종: INFINITI (NISSAN) ® | G 20 | 1992- | INFINITI (NISSAN) ® | M</t>
         </is>
       </c>
-      <c r="E174" s="7" t="inlineStr">
+      <c r="E174" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/dat-10/3335/</t>
         </is>
@@ -8622,7 +8622,7 @@
           <t>DAT-22 = ERREBI NS5, EZ DA31, ILCO X210, SILCA NSN11</t>
         </is>
       </c>
-      <c r="E175" s="7" t="inlineStr">
+      <c r="E175" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/dat-22/3394/</t>
         </is>
@@ -8649,7 +8649,7 @@
           <t>NSN11 Xhorse KeyDIY Flip Key Blade Replacement #06</t>
         </is>
       </c>
-      <c r="E176" s="7" t="inlineStr">
+      <c r="E176" s="6" t="inlineStr">
         <is>
           <t>https://www.bestkeysupply.com/products/nsn11-xhorse-keydiy-universal-flipkey-insert-06-b156bks</t>
         </is>
@@ -8676,7 +8676,7 @@
           <t>NSN11 For older Nissan Subaru Ford LDV 1995-2003, Blank number 06#</t>
         </is>
       </c>
-      <c r="E177" s="7" t="inlineStr">
+      <c r="E177" s="6" t="inlineStr">
         <is>
           <t>https://accessfobs.co.uk/products/blade-for-keydiy-and-xhorse-remote-for-nsn11-nissan-subaru</t>
         </is>
@@ -8703,7 +8703,7 @@
           <t>SUB-2P = ERREBI SUB1P175, SILCA DAT17* / 차종: SUBARU ® | VARIOUS MODELS | -</t>
         </is>
       </c>
-      <c r="E178" s="7" t="inlineStr">
+      <c r="E178" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/sub-2p/10867/</t>
         </is>
@@ -8730,7 +8730,7 @@
           <t>KEYDIY - DAT17 - Flip Key Blade - #65 - For Xhorse / Keydiy Universal Remote Flip Keys</t>
         </is>
       </c>
-      <c r="E179" s="7" t="inlineStr">
+      <c r="E179" s="6" t="inlineStr">
         <is>
           <t>https://www.uhs-hardware.com/products/keydiy-dat17-flip-key-blade-65-for-xhorse-keydiy-universal-remote-flip-keys</t>
         </is>
@@ -8757,7 +8757,7 @@
           <t>DAT17 - #65 - UB10017 (Subaru)</t>
         </is>
       </c>
-      <c r="E180" s="7" t="inlineStr">
+      <c r="E180" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -8784,7 +8784,7 @@
           <t>Silca DAT17 = JMA SUB-2, 상품 코드 SUB#65</t>
         </is>
       </c>
-      <c r="E181" s="7" t="inlineStr">
+      <c r="E181" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2150&amp;controller=product</t>
         </is>
@@ -8811,7 +8811,7 @@
           <t>SUB-1 = EZ SUB1, ILCO X251, SILCA NSN19</t>
         </is>
       </c>
-      <c r="E182" s="7" t="inlineStr">
+      <c r="E182" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/sub-1/10865/</t>
         </is>
@@ -8838,7 +8838,7 @@
           <t>Subaru NSN19 - Flip Key Blade w/Roll Pins for Xhorse Remotes (5 Pack)</t>
         </is>
       </c>
-      <c r="E183" s="7" t="inlineStr">
+      <c r="E183" s="6" t="inlineStr">
         <is>
           <t>https://autorescuetools.com/products/subaru-nsn19-flip-key-blade-w-roll-pins-for-xhorse-remotes-gtl-5-pack</t>
         </is>
@@ -8865,7 +8865,7 @@
           <t>10x Flip Remote Key Blades Xhorse and Keydiy Subaru Type NSN19 SUB1</t>
         </is>
       </c>
-      <c r="E184" s="7" t="inlineStr">
+      <c r="E184" s="6" t="inlineStr">
         <is>
           <t>https://www.ebay.com/itm/313605698988</t>
         </is>
@@ -8892,7 +8892,7 @@
           <t>Subaru RK-KD-186, ILCO SUB1, JMA SUB-1</t>
         </is>
       </c>
-      <c r="E185" s="7" t="inlineStr">
+      <c r="E185" s="6" t="inlineStr">
         <is>
           <t>https://www.americankeysupply.com/product/10098</t>
         </is>
@@ -8919,7 +8919,7 @@
           <t>Key4 NSN19 키날 사진, 각인 186</t>
         </is>
       </c>
-      <c r="E186" s="7" t="inlineStr">
+      <c r="E186" s="6" t="inlineStr">
         <is>
           <t>https://www.key4.com/uploads/files/products/xhorse_keydiy_key_blades/KB-UNV-NSN19/KB-UNV-NSN19-1.jpg</t>
         </is>
@@ -8946,7 +8946,7 @@
           <t>VVDI Key Tool/KeyDIY Blade SUB4 #186 - 5 Pack</t>
         </is>
       </c>
-      <c r="E187" s="7" t="inlineStr">
+      <c r="E187" s="6" t="inlineStr">
         <is>
           <t>https://keyinnovations.com/vvdi-key-tool-keydiy-blade-sub4-186-5-pack/</t>
         </is>
@@ -8973,7 +8973,7 @@
           <t>Ilco 스바루 면: X251 / SUB1 / SUB1-P / SUB4-PT 순서로 실림. SUB4FB, SUB4-GTK, EB3-P-SUB4도 있음</t>
         </is>
       </c>
-      <c r="E188" s="7" t="inlineStr">
+      <c r="E188" s="6" t="inlineStr">
         <is>
           <t>https://www.key4.com/uploads/files/products/metal_keys/AC-ILC-KEYDIR13/Key_Blank_Directory_-_Edition_13.pdf</t>
         </is>
@@ -9000,7 +9000,7 @@
           <t>HOND-31 = 등가 코드 없음</t>
         </is>
       </c>
-      <c r="E189" s="7" t="inlineStr">
+      <c r="E189" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/hond-31/5631/</t>
         </is>
@@ -9027,7 +9027,7 @@
           <t>KEYDIY - HO01 - Flip Key Blade - #25 - For Xhorse / Keydiy Universal Remote Flip Keys</t>
         </is>
       </c>
-      <c r="E190" s="7" t="inlineStr">
+      <c r="E190" s="6" t="inlineStr">
         <is>
           <t>https://www.uhs-hardware.com/products/keydiy-ho01-flip-key-blade-25-for-xhorse-keydiy-universal-remote-flip-keys</t>
         </is>
@@ -9054,7 +9054,7 @@
           <t>HON66 - #25 - UB10009 (Honda / Acura)</t>
         </is>
       </c>
-      <c r="E191" s="7" t="inlineStr">
+      <c r="E191" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -9081,7 +9081,7 @@
           <t>Cross Reference: HO01, HOND-31, HON66</t>
         </is>
       </c>
-      <c r="E192" s="7" t="inlineStr">
+      <c r="E192" s="6" t="inlineStr">
         <is>
           <t>https://www.key4.com/honda-flip-key-blade-ho01</t>
         </is>
@@ -9108,7 +9108,7 @@
           <t>HOND-16D = ERREBI HD43R, EZ HD103, HD104, ILCO X214, X215, SILCA HON58R / 차종: ACURA (HONDA) ® | CL | 1995-1998 | ACURA (HONDA) ® | NSX | 1</t>
         </is>
       </c>
-      <c r="E193" s="7" t="inlineStr">
+      <c r="E193" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/hond-16d/5559/</t>
         </is>
@@ -9135,7 +9135,7 @@
           <t>TP00HOND-21P = ERREBI T00HD43RP, ILCO HD106-PT, HD111-PT, SILCA HON58RT0</t>
         </is>
       </c>
-      <c r="E194" s="7" t="inlineStr">
+      <c r="E194" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/tp00hond-21p/11519/</t>
         </is>
@@ -9162,7 +9162,7 @@
           <t>KEYDIY - HD103 - Flip Key Blade - #03 - For Xhorse / Keydiy Universal Remote Flip Keys</t>
         </is>
       </c>
-      <c r="E195" s="7" t="inlineStr">
+      <c r="E195" s="6" t="inlineStr">
         <is>
           <t>https://www.uhs-hardware.com/products/keydiy-hd103-flip-key-blade-03-for-xhorse-keydiy-universal-remote-flip-keys</t>
         </is>
@@ -9189,7 +9189,7 @@
           <t>HD106 - #03 - UB10002 (Honda)</t>
         </is>
       </c>
-      <c r="E196" s="7" t="inlineStr">
+      <c r="E196" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -9216,7 +9216,7 @@
           <t>Silca HON58R = JMA HOND-21, 상품 코드 HON#03</t>
         </is>
       </c>
-      <c r="E197" s="7" t="inlineStr">
+      <c r="E197" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2140&amp;controller=product</t>
         </is>
@@ -9243,7 +9243,7 @@
           <t>MAZ-11D = ERREBI MZ23R, EZ MZ31, ILCO X249, SILCA MAZ25R / 차종: MAZDA ® | VARIOUS MODELS | 1998-</t>
         </is>
       </c>
-      <c r="E198" s="7" t="inlineStr">
+      <c r="E198" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/maz-11d/7772/</t>
         </is>
@@ -9270,7 +9270,7 @@
           <t>MAZ-11DP1 = ERREBI MZ23RP88, SILCA MAZ24REP / 차종: MAZDA ® | VARIOUS MODELS | 1998-</t>
         </is>
       </c>
-      <c r="E199" s="7" t="inlineStr">
+      <c r="E199" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/maz-11dp1/7774/</t>
         </is>
@@ -9297,7 +9297,7 @@
           <t>KEYDIY - MZ34 - Flip Key Blade - #27 - For Xhorse / Keydiy Universal Remote Flip Keys</t>
         </is>
       </c>
-      <c r="E200" s="7" t="inlineStr">
+      <c r="E200" s="6" t="inlineStr">
         <is>
           <t>https://www.uhs-hardware.com/products/keydiy-mz34-flip-key-blade-27-for-xhorse-keydiy-universal-remote-flip-keys</t>
         </is>
@@ -9324,7 +9324,7 @@
           <t>MAZ24 - #27 - UB10011 (Mazda)</t>
         </is>
       </c>
-      <c r="E201" s="7" t="inlineStr">
+      <c r="E201" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -9351,7 +9351,7 @@
           <t>Silca MAZ24R = JMA MAZ-11D, 상품 코드 MAZ#27-1</t>
         </is>
       </c>
-      <c r="E202" s="7" t="inlineStr">
+      <c r="E202" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2145&amp;controller=product</t>
         </is>
@@ -9378,7 +9378,7 @@
           <t>MAZ-17D = ERREBI MZ12R, EZ MZ19, ILCO X201, SILCA MAZ13</t>
         </is>
       </c>
-      <c r="E203" s="7" t="inlineStr">
+      <c r="E203" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/maz-17d/7790/</t>
         </is>
@@ -9405,7 +9405,7 @@
           <t>Keydiy MAZ13 Flip Keyblade - Blade09</t>
         </is>
       </c>
-      <c r="E204" s="7" t="inlineStr">
+      <c r="E204" s="6" t="inlineStr">
         <is>
           <t>https://www.remkeys.com/keydiy-maz13-flip-keyblade-blade09-mazda-makb04</t>
         </is>
@@ -9432,7 +9432,7 @@
           <t>KD Mazda Flip Remote Key Blade MAZ13, Manufacturer Part Number 09 (검색 결과)</t>
         </is>
       </c>
-      <c r="E205" s="7" t="inlineStr">
+      <c r="E205" s="6" t="inlineStr">
         <is>
           <t>https://www.mk3.com/kd-mazda-flip-remote-key-blade-maz13</t>
         </is>
@@ -9459,7 +9459,7 @@
           <t>KeyDiy Xhorse Remote Key Blade For Mazda MAZ13</t>
         </is>
       </c>
-      <c r="E206" s="7" t="inlineStr">
+      <c r="E206" s="6" t="inlineStr">
         <is>
           <t>https://abkeys.com/products/mazda-flip-remote-key-blade-maz13-for-kd-xhorse-remote-blade-14</t>
         </is>
@@ -9486,7 +9486,7 @@
           <t>Xhorse VVDI Keydiy KD Universal Flip Remote key Blade Mazda MAZ13, Part Number: 09 (VD9560)</t>
         </is>
       </c>
-      <c r="E207" s="7" t="inlineStr">
+      <c r="E207" s="6" t="inlineStr">
         <is>
           <t>https://www.ww.vvdi.com/kd900-blade-for-mazda-flip-remote-key-maz13</t>
         </is>
@@ -9513,7 +9513,7 @@
           <t>MIT-14D = ERREBI MIT8R, EZ MIT3, ILCO X224, SILCA MIT11R / 차종: DODGE ® | COLT | 1993- | DODGE ® | VISTA | 1993- | EAGLE ® |</t>
         </is>
       </c>
-      <c r="E208" s="7" t="inlineStr">
+      <c r="E208" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/mit-14d/8145/</t>
         </is>
@@ -9540,7 +9540,7 @@
           <t>MIT-8DP = ERREBI MIT8RP77, SILCA MIT11RAP / 차종: CHRYSLER ® | COLT | 1993- | CHRYSLER ® | VISTA | 1993- | DOD</t>
         </is>
       </c>
-      <c r="E209" s="7" t="inlineStr">
+      <c r="E209" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/mit-8dp/8196/</t>
         </is>
@@ -9567,7 +9567,7 @@
           <t>KEYDIY - MIT3 - Flip Key Blade - #07 - For Xhorse / Keydiy Universal Remote Flip Keys</t>
         </is>
       </c>
-      <c r="E210" s="7" t="inlineStr">
+      <c r="E210" s="6" t="inlineStr">
         <is>
           <t>https://www.uhs-hardware.com/products/keydiy-mit3-flip-key-blade-07-for-xhorse-keydiy-universal-remote-flip-keys</t>
         </is>
@@ -9594,7 +9594,7 @@
           <t>MIT11R - #07 - UB10003 (Mitsubishi)</t>
         </is>
       </c>
-      <c r="E211" s="7" t="inlineStr">
+      <c r="E211" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -9621,7 +9621,7 @@
           <t>Silca MIT11R = JMA MIT-8D, 상품 코드 MIT#07</t>
         </is>
       </c>
-      <c r="E212" s="7" t="inlineStr">
+      <c r="E212" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2146&amp;controller=product</t>
         </is>
@@ -9648,7 +9648,7 @@
           <t>MIT-16 = EZ MIT1, ILCO X176</t>
         </is>
       </c>
-      <c r="E213" s="7" t="inlineStr">
+      <c r="E213" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/mit-16/8150/</t>
         </is>
@@ -9675,7 +9675,7 @@
           <t>MIT-7 = ERREBI MIT7, EZ MIT4, ILCO X245, SILCA MIT8 / 차종: BERTONE ® | FREECLIMBER | -19- | BERTONE ® | SL-CABRIO | -19</t>
         </is>
       </c>
-      <c r="E214" s="7" t="inlineStr">
+      <c r="E214" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/mit-7/8189/</t>
         </is>
@@ -9702,7 +9702,7 @@
           <t>Silca MIT8 = Ilco X176, Silca MIT8P = MIT1-P, Silca MIT8AP = MIT4-P</t>
         </is>
       </c>
-      <c r="E215" s="7" t="inlineStr">
+      <c r="E215" s="6" t="inlineStr">
         <is>
           <t>https://www.key4.com/uploads/files/products/metal_keys/AC-ILC-KEYDIR13/Key_Blank_Directory_-_Edition_13.pdf</t>
         </is>
@@ -9729,7 +9729,7 @@
           <t>Mitsubishi RK-KD-062, ILCO MIT1, JMA MIT-16</t>
         </is>
       </c>
-      <c r="E216" s="7" t="inlineStr">
+      <c r="E216" s="6" t="inlineStr">
         <is>
           <t>https://www.americankeysupply.com/product/10098</t>
         </is>
@@ -9756,7 +9756,7 @@
           <t>Key4 MIT1 키날 사진, 각인 62</t>
         </is>
       </c>
-      <c r="E217" s="7" t="inlineStr">
+      <c r="E217" s="6" t="inlineStr">
         <is>
           <t>https://www.key4.com/uploads/files/products/universal_key_blade/KB-UNV-MIT1/KB-UNV-MIT1-6.jpg</t>
         </is>
@@ -9783,7 +9783,7 @@
           <t>Uncut key blank Mitsubishi X176 MIT1 (교차 번호: ESP MIT1, ILCO X176, SILCA MIT8, JMA MIT-16)</t>
         </is>
       </c>
-      <c r="E218" s="7" t="inlineStr">
+      <c r="E218" s="6" t="inlineStr">
         <is>
           <t>https://www.clksupplies.com/products/uncut-key-blank-mitsubishi-x176-mit1</t>
         </is>
@@ -9810,7 +9810,7 @@
           <t>KEYDIY - MIT1 - Flip Key Blade - #62 - For Xhorse / Keydiy Universal Remote Flip Keys</t>
         </is>
       </c>
-      <c r="E219" s="7" t="inlineStr">
+      <c r="E219" s="6" t="inlineStr">
         <is>
           <t>https://www.uhs-hardware.com/products/keydiy-mit1-flip-key-blade-62-for-xhorse-keydiy-universal-remote-flip-keys</t>
         </is>
@@ -9837,7 +9837,7 @@
           <t>Mitsubishi MIT4R, MIT1 - Y-13#, 62# - Key Blade for Xhorse &amp; KeyDIY Universal Remotes (Pack of 10)</t>
         </is>
       </c>
-      <c r="E220" s="7" t="inlineStr">
+      <c r="E220" s="6" t="inlineStr">
         <is>
           <t>https://autorescuetools.com/products/y-13-62-mit4r-mit1-mitsubishi-key-blade-for-xhorse-keydiy-universal-remotes-pack-of-10x</t>
         </is>
@@ -9864,7 +9864,7 @@
           <t>Mitsubishi MIT1 Blade Y-13# for Xhorse &amp; KEYDIY Universal Remotes</t>
         </is>
       </c>
-      <c r="E221" s="7" t="inlineStr">
+      <c r="E221" s="6" t="inlineStr">
         <is>
           <t>https://keyinnovations.com/keyless2go-mitsubishi-mit1-blade-y-13-for-xhorse-keydiy-universal-remotes-25-pack/</t>
         </is>
@@ -9891,7 +9891,7 @@
           <t>MIT08 - #15 Y-13 - UB10029 (Mitsubishi)</t>
         </is>
       </c>
-      <c r="E222" s="7" t="inlineStr">
+      <c r="E222" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -9918,7 +9918,7 @@
           <t>Silca MIT8 = JMA MIT-12, 상품 코드 MIT#Y-13</t>
         </is>
       </c>
-      <c r="E223" s="7" t="inlineStr">
+      <c r="E223" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2147&amp;controller=product</t>
         </is>
@@ -9945,7 +9945,7 @@
           <t>MIT8 MIT-12, Blade number Y-13, For Mitsubishi</t>
         </is>
       </c>
-      <c r="E224" s="7" t="inlineStr">
+      <c r="E224" s="6" t="inlineStr">
         <is>
           <t>https://accessfobs.co.uk/products/blade-for-keydiy-and-xhorse-remote-mit8</t>
         </is>
@@ -9972,7 +9972,7 @@
           <t>Keydiy / Xhorse MIT8 #62 Flip Key Blade (검색 결과)</t>
         </is>
       </c>
-      <c r="E225" s="7" t="inlineStr">
+      <c r="E225" s="6" t="inlineStr">
         <is>
           <t>https://keystation.co.uk/keydiy-xhorse-mit8-62-flip-key-blade</t>
         </is>
@@ -9999,7 +9999,7 @@
           <t>KEYDIY Remote Flip Key Blade MIT8 for Mitsubishi (Y-13) (같은 판매처에 MIT8 Y21 상품도 있음)</t>
         </is>
       </c>
-      <c r="E226" s="7" t="inlineStr">
+      <c r="E226" s="6" t="inlineStr">
         <is>
           <t>https://www.locksmithkeyless.com/products/keydiy-remote-flip-key-blade-mit8-for-mitsubishi-y-13</t>
         </is>
@@ -10026,7 +10026,7 @@
           <t>KEYDIY - MIT8 - Flip Key Blade - #Y21 - For Xhorse / Keydiy Universal Remote Flip Keys</t>
         </is>
       </c>
-      <c r="E227" s="7" t="inlineStr">
+      <c r="E227" s="6" t="inlineStr">
         <is>
           <t>https://www.uhs-hardware.com/products/keydiy-mit8-flip-key-blade-y21-for-xhorse-keydiy-universal-remote-flip-keys</t>
         </is>
@@ -10049,7 +10049,7 @@
           <t>MIT-13D = ERREBI MIT12R, EZ MIT5, ILCO X229, SILCA MIT12R / 차종: DODGE ® | COLT | 1993- | DODGE ® | VISTA | 1993- | EAGLE ® |</t>
         </is>
       </c>
-      <c r="E228" s="7" t="inlineStr">
+      <c r="E228" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/mit-13d/8143/</t>
         </is>
@@ -10072,7 +10072,7 @@
           <t>KEYDIY - MIT5 / X229 - Flip Key Blade - #Y21 - For Xhorse / Keydiy Universal Remote Flip Keys</t>
         </is>
       </c>
-      <c r="E229" s="7" t="inlineStr">
+      <c r="E229" s="6" t="inlineStr">
         <is>
           <t>https://www.uhs-hardware.com/products/keydiy-mit5-x229-flip-key-blade-y21-for-xhorse-keydiy-universal-remote-flip-keys</t>
         </is>
@@ -10095,7 +10095,7 @@
           <t>MIT-18 = EZ MIT6, ILCO X263</t>
         </is>
       </c>
-      <c r="E230" s="7" t="inlineStr">
+      <c r="E230" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/mit-18/8154/</t>
         </is>
@@ -10118,7 +10118,7 @@
           <t>VVDI Key Tool/KeyDIY Blade MIT6 - 5 Pack</t>
         </is>
       </c>
-      <c r="E231" s="7" t="inlineStr">
+      <c r="E231" s="6" t="inlineStr">
         <is>
           <t>https://keyinnovations.com/vvdi-key-tool-keydiy-blade-mit6-5-pack/</t>
         </is>
@@ -10141,7 +10141,7 @@
           <t>Mitsubishi RK-KD-187, ILCO MIT6, JMA MIT-18</t>
         </is>
       </c>
-      <c r="E232" s="7" t="inlineStr">
+      <c r="E232" s="6" t="inlineStr">
         <is>
           <t>https://www.americankeysupply.com/product/10098</t>
         </is>
@@ -10168,7 +10168,7 @@
           <t>MIT-2D = ERREBI MIT2R, ILCO TR33, SILCA MIT2 / 차종: MITSUBISHI ® | VARIOUS MODELS | - | TOYOTA ® | VARIOUS MODEL</t>
         </is>
       </c>
-      <c r="E233" s="7" t="inlineStr">
+      <c r="E233" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/mit-2d/8168/</t>
         </is>
@@ -10195,7 +10195,7 @@
           <t>Silca MIT2 = Ilco TR33</t>
         </is>
       </c>
-      <c r="E234" s="7" t="inlineStr">
+      <c r="E234" s="6" t="inlineStr">
         <is>
           <t>https://www.key4.com/uploads/files/products/metal_keys/AC-ILC-KEYDIR13/Key_Blank_Directory_-_Edition_13.pdf</t>
         </is>
@@ -10222,7 +10222,7 @@
           <t>Mitsubishi Keydiy MIT2 Flip Keyblade - Blade16 (사진 각인 16)</t>
         </is>
       </c>
-      <c r="E235" s="7" t="inlineStr">
+      <c r="E235" s="6" t="inlineStr">
         <is>
           <t>https://remkeys.com/product/mitsubishi-keydiy-mit2-flip-keyblade-blade16-mikb02-remkeys/</t>
         </is>
@@ -10249,7 +10249,7 @@
           <t>Xhorse KeyDiy KD Remote Key Blade, Blade Profile MIT2, P/N 16 (검색 결과)</t>
         </is>
       </c>
-      <c r="E236" s="7" t="inlineStr">
+      <c r="E236" s="6" t="inlineStr">
         <is>
           <t>https://www.tlkeys.com/products/Keydiy-KD-Metal-Blank-Uncut-Flip-Key-Blade-33942</t>
         </is>
@@ -10276,7 +10276,7 @@
           <t>Uncut Universal Flip Remote Key Blade Mitsubishi Type MIT2 (번호 미표기)</t>
         </is>
       </c>
-      <c r="E237" s="7" t="inlineStr">
+      <c r="E237" s="6" t="inlineStr">
         <is>
           <t>https://www.key4.com/mitsubishi-flip-key-blade-mit2</t>
         </is>
@@ -10303,7 +10303,7 @@
           <t>Keydiy KD Xhorse VVDI Universal Flip Remote Blade Mitsubishi MIT2, part number 16 (검색 결과)</t>
         </is>
       </c>
-      <c r="E238" s="7" t="inlineStr">
+      <c r="E238" s="6" t="inlineStr">
         <is>
           <t>https://www.mk3.com/es/MK19559</t>
         </is>
@@ -10326,7 +10326,7 @@
           <t>MIT-2I = ERREBI MIT2, EZ DC3, ILCO X121, SILCA MIT2R / 차종: CHRYSLER ® | CHALLENGER | -19- | CHRYSLER ® | CONQUEST | -19</t>
         </is>
       </c>
-      <c r="E239" s="7" t="inlineStr">
+      <c r="E239" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/mit-2i/8172/</t>
         </is>
@@ -10349,7 +10349,7 @@
           <t>Silca MIT2R = Ilco X121, DC3</t>
         </is>
       </c>
-      <c r="E240" s="7" t="inlineStr">
+      <c r="E240" s="6" t="inlineStr">
         <is>
           <t>https://www.key4.com/uploads/files/products/metal_keys/AC-ILC-KEYDIR13/Key_Blank_Directory_-_Edition_13.pdf</t>
         </is>
@@ -10372,7 +10372,7 @@
           <t>Mitsubishi Keydiy MIT2R Flip Keyblade - Blade23 (사진 각인 23)</t>
         </is>
       </c>
-      <c r="E241" s="7" t="inlineStr">
+      <c r="E241" s="6" t="inlineStr">
         <is>
           <t>https://remkeys.com/product/mitsubishi-keydiy-mit2r-flip-keyblade-blade23-mikb03-remkeys/</t>
         </is>
@@ -10399,7 +10399,7 @@
           <t>SUZU-8 = ERREBI SZ10R, EZ SUZ17, ILCO X186, SILCA SZ11R / 차종: SUZUKI ® | ALTO | 1996- | SUZUKI ® | CARRY VAN | 1989-1991 |</t>
         </is>
       </c>
-      <c r="E242" s="7" t="inlineStr">
+      <c r="E242" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/suzu-8/10938/</t>
         </is>
@@ -10426,7 +10426,7 @@
           <t>Mitsubishi, Suzuki MIT11R, MIT3, SZ11R - 07# - Key Blade for Xhorse &amp; KeyDIY Universal Remotes (Pack of 10)</t>
         </is>
       </c>
-      <c r="E243" s="7" t="inlineStr">
+      <c r="E243" s="6" t="inlineStr">
         <is>
           <t>https://autorescuetools.com/products/07-mit11r-mit3-mitsubishi-suzuki-key-blade-for-xhorse-keydiy-universal-remotes-pack-of-10x</t>
         </is>
@@ -10453,7 +10453,7 @@
           <t>KeyDiy Xhorse Remote Key Blade For Suzuki SZ11R (ABK-46), 사진 각인 35</t>
         </is>
       </c>
-      <c r="E244" s="7" t="inlineStr">
+      <c r="E244" s="6" t="inlineStr">
         <is>
           <t>https://abkeys.com/products/suzuki-sz11r-keydiy-xhorse-remote-key-blade-46</t>
         </is>
@@ -10480,7 +10480,7 @@
           <t>10pcs 35# KD Car Key Blank Uncut SZ11R Remote Blade Flip Key Blank for Suzuki Alto</t>
         </is>
       </c>
-      <c r="E245" s="7" t="inlineStr">
+      <c r="E245" s="6" t="inlineStr">
         <is>
           <t>https://www.aliexpress.us/item/3256806486913008.html</t>
         </is>
@@ -10507,7 +10507,7 @@
           <t>10PCS VVDI KD 35# Key Blank Uncut Universal SZ11R Car Key Blade for Suzuki Alto</t>
         </is>
       </c>
-      <c r="E246" s="7" t="inlineStr">
+      <c r="E246" s="6" t="inlineStr">
         <is>
           <t>https://www.aliexpress.us/item/3256804878274635.html</t>
         </is>
@@ -10534,7 +10534,7 @@
           <t>SUZU-8I = SILCA SZ11 / 차종: SUZUKI ® | VARIOUS MODELS | -</t>
         </is>
       </c>
-      <c r="E247" s="7" t="inlineStr">
+      <c r="E247" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/suzu-8i/10940/</t>
         </is>
@@ -10561,7 +10561,7 @@
           <t>Silca SZ11 = JMA SUZU-8I, 상품 코드 SUZ#36</t>
         </is>
       </c>
-      <c r="E248" s="7" t="inlineStr">
+      <c r="E248" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2168&amp;controller=product</t>
         </is>
@@ -10588,7 +10588,7 @@
           <t>Keydiy KD Xhorse VVDI Universal Flip Remote Key Uncut Blade #85 Suzuki Type SZ11</t>
         </is>
       </c>
-      <c r="E249" s="7" t="inlineStr">
+      <c r="E249" s="6" t="inlineStr">
         <is>
           <t>https://gskeyae.com/product/keydiy-flip-key-blade-suzuki-sz11/</t>
         </is>
@@ -10638,7 +10638,7 @@
           <t>Keydiy / Xhorse SZ11 #36 Flip Key Blade (검색 결과)</t>
         </is>
       </c>
-      <c r="E251" s="7" t="inlineStr">
+      <c r="E251" s="6" t="inlineStr">
         <is>
           <t>https://keystation.co.uk/vehicle-makes/suzuki-car-keys-parts/suzuki-car-key-blades</t>
         </is>
@@ -10665,7 +10665,7 @@
           <t>SZ11 SZ11MH SZ11FH For Suzuki Alto 2002-2008, Key number #36</t>
         </is>
       </c>
-      <c r="E252" s="7" t="inlineStr">
+      <c r="E252" s="6" t="inlineStr">
         <is>
           <t>https://accessfobs.co.uk/products/blade-for-keydiy-and-xhorse-remote-sx11-suzuki</t>
         </is>
@@ -10692,7 +10692,7 @@
           <t>Key4 SZ11 키날 사진, 각인 40</t>
         </is>
       </c>
-      <c r="E253" s="7" t="inlineStr">
+      <c r="E253" s="6" t="inlineStr">
         <is>
           <t>https://www.key4.com/uploads/files/products/key_blades/KB-KDY-SZ11/KB-KDY-SZ11_photo.jpg</t>
         </is>
@@ -10719,7 +10719,7 @@
           <t>TP00SUZU-14P2 = ERREBI T00SZ15P, SILCA HU133RTE / 차종: SUZUKI ® | VARIOUS MODELS | -</t>
         </is>
       </c>
-      <c r="E254" s="7" t="inlineStr">
+      <c r="E254" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/tp00suzu-14p2/11616/</t>
         </is>
@@ -10746,7 +10746,7 @@
           <t>HU133 - #52 - UB10016 (Suzuki)</t>
         </is>
       </c>
-      <c r="E255" s="7" t="inlineStr">
+      <c r="E255" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -10773,7 +10773,7 @@
           <t>KeyDIY Suzuki Universal Flip Key Blade, SUZ20 (#52)</t>
         </is>
       </c>
-      <c r="E256" s="7" t="inlineStr">
+      <c r="E256" s="6" t="inlineStr">
         <is>
           <t>https://keyinnovations.com/keydiy-blade-suz20-165153/</t>
         </is>
@@ -10800,7 +10800,7 @@
           <t>1999-2013 Suzuki SUZ20-P / Plastic Head Mechanical Key (JMA-SUZU-19.D.P) (SUZU-14-P2)</t>
         </is>
       </c>
-      <c r="E257" s="7" t="inlineStr">
+      <c r="E257" s="6" t="inlineStr">
         <is>
           <t>https://www.uhs-hardware.com/products/1999-2013-suzuki-suz20-p-plastic-head-mechanical-key-jma-suzu-19-d-p-suzu-14-p2</t>
         </is>
@@ -10827,7 +10827,7 @@
           <t>Silca HU133R = JMA SUZU-14, 상품 코드 SUZ#52</t>
         </is>
       </c>
-      <c r="E258" s="7" t="inlineStr">
+      <c r="E258" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2151&amp;controller=product</t>
         </is>
@@ -10854,7 +10854,7 @@
           <t>TP00OP-10P = ERREBI T00HF60P, SILCA HU87RT0</t>
         </is>
       </c>
-      <c r="E259" s="7" t="inlineStr">
+      <c r="E259" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/tp00op-10p/11588/</t>
         </is>
@@ -10881,7 +10881,7 @@
           <t>Silca HU87R = JMA OP-10, 상품 코드 SUZ#Y-19</t>
         </is>
       </c>
-      <c r="E260" s="7" t="inlineStr">
+      <c r="E260" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2182&amp;controller=product</t>
         </is>
@@ -10908,7 +10908,7 @@
           <t>HU87 Xhorse KeyDIY Flip Key Blade Replacement #52</t>
         </is>
       </c>
-      <c r="E261" s="7" t="inlineStr">
+      <c r="E261" s="6" t="inlineStr">
         <is>
           <t>https://www.bestkeysupply.com/products/hu87-xhorse-keydiy-universal-flipkey-insert-52-b139bks</t>
         </is>
@@ -10935,7 +10935,7 @@
           <t>Keydiy KD Xhorse VVDI Universal Flip Remote Key Blade HU133 HU87R Suzuki Swift Type #52</t>
         </is>
       </c>
-      <c r="E262" s="7" t="inlineStr">
+      <c r="E262" s="6" t="inlineStr">
         <is>
           <t>https://gskeyae.com/product/keydiy-flip-key-blade-suzuki-hu133/</t>
         </is>
@@ -10962,7 +10962,7 @@
           <t>HU87R / HU133R OP-10 / SUZU-14, Blade number 52 (한 상품)</t>
         </is>
       </c>
-      <c r="E263" s="7" t="inlineStr">
+      <c r="E263" s="6" t="inlineStr">
         <is>
           <t>https://accessfobs.co.uk/products/blade-for-keydiy-and-xhorse-remote-hu87r-hu133r</t>
         </is>
@@ -10989,7 +10989,7 @@
           <t>HU87R 검색 결과는 트랜스폰더 품번(TP00OP-10P = Silca HU87RT0 등)뿐이고 Ilco 이름 없음</t>
         </is>
       </c>
-      <c r="E264" s="7" t="inlineStr">
+      <c r="E264" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/tp00op-10p/11588/</t>
         </is>
@@ -11012,7 +11012,7 @@
           <t xml:space="preserve">SUZU-10 = ERREBI SZ11, EZ SUZ15, ILCO X185, SILCA SZ12 / 차종: HOLDEN ® | BARINA | 1991-1993 | SUZUKI ® | BALENO | 1995- | </t>
         </is>
       </c>
-      <c r="E265" s="7" t="inlineStr">
+      <c r="E265" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/suzu-10/10871/</t>
         </is>
@@ -11035,7 +11035,7 @@
           <t>KeyDiy Xhorse Remote Key Blade For Suzuki SZ12</t>
         </is>
       </c>
-      <c r="E266" s="7" t="inlineStr">
+      <c r="E266" s="6" t="inlineStr">
         <is>
           <t>https://abkeys.com/products/keydiy-xhorse-universal-remote-key-blade-for-suzuki-sz12-75</t>
         </is>
@@ -11062,7 +11062,7 @@
           <t>GM-39 = EZ B102, ILCO P1113</t>
         </is>
       </c>
-      <c r="E267" s="7" t="inlineStr">
+      <c r="E267" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/gm-39/5092/</t>
         </is>
@@ -11089,7 +11089,7 @@
           <t>KEYDIY - B102 - Flip Key Blade - #26 - For Xhorse / Keydiy Universal Remote Flip Keys</t>
         </is>
       </c>
-      <c r="E268" s="7" t="inlineStr">
+      <c r="E268" s="6" t="inlineStr">
         <is>
           <t>https://www.uhs-hardware.com/products/keydiy-b102-flip-key-blade-26-for-xhorse-keydiy-universal-remote-flip-keys</t>
         </is>
@@ -11116,7 +11116,7 @@
           <t>B86 - #26 - UB10010 (Chevrolet / Buick)</t>
         </is>
       </c>
-      <c r="E269" s="7" t="inlineStr">
+      <c r="E269" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -11143,7 +11143,7 @@
           <t>Cross Reference: B102, GM-39, B99</t>
         </is>
       </c>
-      <c r="E270" s="7" t="inlineStr">
+      <c r="E270" s="6" t="inlineStr">
         <is>
           <t>https://www.key4.com/gm-flip-key-blade-b102</t>
         </is>
@@ -11193,7 +11193,7 @@
           <t>GM-37 = EZ B106, ILCO P1115, B111</t>
         </is>
       </c>
-      <c r="E272" s="7" t="inlineStr">
+      <c r="E272" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/gm-37/5088/</t>
         </is>
@@ -11220,7 +11220,7 @@
           <t>B106/111 - #87 Y-66 - UB10042 (GM / Saab / Suzuki)</t>
         </is>
       </c>
-      <c r="E273" s="7" t="inlineStr">
+      <c r="E273" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -11247,7 +11247,7 @@
           <t>KEYDIY - B106 - Flip Key Blade - #Y66 - For Xhorse / Keydiy Universal Remote Flip Keys</t>
         </is>
       </c>
-      <c r="E274" s="7" t="inlineStr">
+      <c r="E274" s="6" t="inlineStr">
         <is>
           <t>https://www.uhs-hardware.com/products/keydiy-b106-flip-key-blade-y66-for-xhorse-keydiy-universal-remote-flip-keys</t>
         </is>
@@ -11274,7 +11274,7 @@
           <t>GM B111 #87 Flip Blade For Xhorse KEYDIY Remotes | Aftermarket</t>
         </is>
       </c>
-      <c r="E275" s="7" t="inlineStr">
+      <c r="E275" s="6" t="inlineStr">
         <is>
           <t>https://www.bestkeysupply.com/products/gm-b111-87-xhorse-kdiy-remotes-aftermarket-b276</t>
         </is>
@@ -11301,7 +11301,7 @@
           <t>KEYDIY - B106 Key Blade #Y66 for Xhorse / Keydiy Universal Key Fob</t>
         </is>
       </c>
-      <c r="E276" s="7" t="inlineStr">
+      <c r="E276" s="6" t="inlineStr">
         <is>
           <t>https://www.locksmithkeyless.com/products/keydiy-b106-key-blade-y66-for-xhorse-keydiy-universal-key-fob</t>
         </is>
@@ -11328,7 +11328,7 @@
           <t>GM B111 #87 Flip Blade For Xhorse KEYDIY Remotes</t>
         </is>
       </c>
-      <c r="E277" s="7" t="inlineStr">
+      <c r="E277" s="6" t="inlineStr">
         <is>
           <t>https://www.bestkeysupply.com/products/gm-b111-87-xhorse-kdiy-remotes-aftermarket-b276</t>
         </is>
@@ -11355,7 +11355,7 @@
           <t>KEYDIY Xhorse Flip Remote Key Blade #87 B111 GM Chevrolet</t>
         </is>
       </c>
-      <c r="E278" s="7" t="inlineStr">
+      <c r="E278" s="6" t="inlineStr">
         <is>
           <t>https://gskeyae.com/product/keydiy-flip-key-blade-buick-b111/</t>
         </is>
@@ -11405,7 +11405,7 @@
           <t>OP-11C1 = ERREBI HF66C1, SILCA HU100T / 차종: BUICK ® | VARIOUS MODELS | 2009-2019 | CADILLAC ® | SRX | 20</t>
         </is>
       </c>
-      <c r="E280" s="7" t="inlineStr">
+      <c r="E280" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/op-11c1/8871/</t>
         </is>
@@ -11432,7 +11432,7 @@
           <t>TP00OP-11P5 = ERREBI T00HF66PE, EZ B119, B120, SILCA HU100TE</t>
         </is>
       </c>
-      <c r="E281" s="7" t="inlineStr">
+      <c r="E281" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/tp00op-11p5/11591/</t>
         </is>
@@ -11459,7 +11459,7 @@
           <t>KEYDIY - HU100 - Flip Key Blade - #71 - For Xhorse / Keydiy Universal Remote Flip Keys</t>
         </is>
       </c>
-      <c r="E282" s="7" t="inlineStr">
+      <c r="E282" s="6" t="inlineStr">
         <is>
           <t>https://www.uhs-hardware.com/products/keydiy-hu100-flip-key-blade-71-for-xhorse-keydiy-universal-remote-flip-keys</t>
         </is>
@@ -11486,7 +11486,7 @@
           <t>HU100 - #71 - UB10020 (GM / Opel / Vauxhall)</t>
         </is>
       </c>
-      <c r="E283" s="7" t="inlineStr">
+      <c r="E283" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -11513,7 +11513,7 @@
           <t>Silca HU100 = JMA OP-11, 상품 코드 OP#71</t>
         </is>
       </c>
-      <c r="E284" s="7" t="inlineStr">
+      <c r="E284" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2149&amp;controller=product</t>
         </is>
@@ -11540,7 +11540,7 @@
           <t>TP00GM-49DP = ERREBI T00GM37P, SILCA GM45TE</t>
         </is>
       </c>
-      <c r="E285" s="7" t="inlineStr">
+      <c r="E285" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/tp00gm-49dp/11517/</t>
         </is>
@@ -11567,7 +11567,7 @@
           <t>KEYDIY - GM45 - Flip Key Blade - #Y28 - For Xhorse / Keydiy Universal Remote Flip Keys</t>
         </is>
       </c>
-      <c r="E286" s="7" t="inlineStr">
+      <c r="E286" s="6" t="inlineStr">
         <is>
           <t>https://www.uhs-hardware.com/products/keydiy-gm45-flip-key-blade-y28-for-xhorse-keydiy-universal-remote-flip-keys</t>
         </is>
@@ -11594,7 +11594,7 @@
           <t>Silca GM45 = JMA GM-49D, 상품 코드 GM#Y-28</t>
         </is>
       </c>
-      <c r="E287" s="7" t="inlineStr">
+      <c r="E287" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2160&amp;controller=product</t>
         </is>
@@ -11621,7 +11621,7 @@
           <t>OP-S = ERREBI HF43, EZ B61, ILCO HF59, SILCA HU46 / 차종: DAEWOO ® | LE MANS | 1983-1984 | GM (CHEVROLET BRA.) ® | CHE</t>
         </is>
       </c>
-      <c r="E288" s="7" t="inlineStr">
+      <c r="E288" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/op-s/8927/</t>
         </is>
@@ -11648,7 +11648,7 @@
           <t>OP-SP = ERREBI HF43P15, ILCO B61, SILCA HU46P / 차종: DAEWOO ® | LE MANS | 1983-1984 | GM (CHEVROLET BRA.) ® | CHE</t>
         </is>
       </c>
-      <c r="E289" s="7" t="inlineStr">
+      <c r="E289" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/op-sp/8931/</t>
         </is>
@@ -11675,7 +11675,7 @@
           <t>Keydiy KD Xhorse VVDI Universal Flip Remote Key Blade #47 HU46 Opel</t>
         </is>
       </c>
-      <c r="E290" s="7" t="inlineStr">
+      <c r="E290" s="6" t="inlineStr">
         <is>
           <t>https://gskeyae.com/product/keydiy-xhorse-flip-key-remote-blade-47-hu46-opel/</t>
         </is>
@@ -11702,7 +11702,7 @@
           <t>KeyDIY Chevrolet, Opel Universal Flip Key Blade, HU46 (49#)</t>
         </is>
       </c>
-      <c r="E291" s="7" t="inlineStr">
+      <c r="E291" s="6" t="inlineStr">
         <is>
           <t>https://keyinnovations.com/chevy-opel-blade-right-sided-groove/</t>
         </is>
@@ -11729,7 +11729,7 @@
           <t>HU46 OP-S For Vauxhall, Blank number 49#</t>
         </is>
       </c>
-      <c r="E292" s="7" t="inlineStr">
+      <c r="E292" s="6" t="inlineStr">
         <is>
           <t>https://accessfobs.co.uk/products/blade-for-keydiy-and-xhorse-remote-hu46</t>
         </is>
@@ -11756,7 +11756,7 @@
           <t>KEYDIY Remote Flip Key Blade HU46 for Opel (Left Slot) (49#)</t>
         </is>
       </c>
-      <c r="E293" s="7" t="inlineStr">
+      <c r="E293" s="6" t="inlineStr">
         <is>
           <t>https://www.locksmithkeyless.com/products/keydiy-remote-flip-key-blade-hu46-for-opel-left-slot-49</t>
         </is>
@@ -11783,7 +11783,7 @@
           <t>Keydiy /Xhorse HU46 #49 Flip Key Blade For Vauxhall (Opel)</t>
         </is>
       </c>
-      <c r="E294" s="7" t="inlineStr">
+      <c r="E294" s="6" t="inlineStr">
         <is>
           <t>https://keystation.co.uk/keydiy-xhorse-hu46-49-flip-key-blade-for-vauxhall-opel</t>
         </is>
@@ -11810,7 +11810,7 @@
           <t>Opel Keydiy HU46 Flip Remote Keyblade - Blade47 (사진 각인 47)</t>
         </is>
       </c>
-      <c r="E295" s="7" t="inlineStr">
+      <c r="E295" s="6" t="inlineStr">
         <is>
           <t>https://remkeys.com/product/opel-keydiy-hu46-flip-remote-keyblade-blade47-opkb12-remkeys/</t>
         </is>
@@ -11837,7 +11837,7 @@
           <t>Keydiy KD Xhorse VVDI Universal Flip Remote Blade HU46, part number 47 (검색 결과)</t>
         </is>
       </c>
-      <c r="E296" s="7" t="inlineStr">
+      <c r="E296" s="6" t="inlineStr">
         <is>
           <t>https://www.mk3.com/es/MK19532</t>
         </is>
@@ -11864,7 +11864,7 @@
           <t>VD9532-Universal Flip Remote key Blade HU46 Opel, part number 47 (검색 결과)</t>
         </is>
       </c>
-      <c r="E297" s="7" t="inlineStr">
+      <c r="E297" s="6" t="inlineStr">
         <is>
           <t>https://www.vvdi.com/kd900-blade-for-flip-remote-key-hu46</t>
         </is>
@@ -11891,7 +11891,7 @@
           <t>OP-WHP = ERREBI HF42P15, SILCA HU43P / 차종: ASTON MARTIN ® | LAGONDA | -19- | ASTON MARTIN ® | LAGONDA L</t>
         </is>
       </c>
-      <c r="E298" s="7" t="inlineStr">
+      <c r="E298" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/op-whp/8942/</t>
         </is>
@@ -11918,7 +11918,7 @@
           <t>KeyDIY Chevrolet, Opel Universal Flip Key Blade, HU43 (Y-18#)</t>
         </is>
       </c>
-      <c r="E299" s="7" t="inlineStr">
+      <c r="E299" s="6" t="inlineStr">
         <is>
           <t>https://keyinnovations.com/chevy-opel-blade-hu43/</t>
         </is>
@@ -11945,7 +11945,7 @@
           <t>KeyDIY Opel Universal Flip Key Blade, HU43 (18#)</t>
         </is>
       </c>
-      <c r="E300" s="7" t="inlineStr">
+      <c r="E300" s="6" t="inlineStr">
         <is>
           <t>https://keyinnovations.com/keydiy-blade-hu43/</t>
         </is>
@@ -11972,7 +11972,7 @@
           <t>For Vauxhall HU43 OP-WH, Blank number Y-18</t>
         </is>
       </c>
-      <c r="E301" s="7" t="inlineStr">
+      <c r="E301" s="6" t="inlineStr">
         <is>
           <t>https://accessfobs.co.uk/products/blade-for-keydiy-and-xhorse-remote-hu43</t>
         </is>
@@ -11999,7 +11999,7 @@
           <t>Silca HU43 = Ilco HF56</t>
         </is>
       </c>
-      <c r="E302" s="7" t="inlineStr">
+      <c r="E302" s="6" t="inlineStr">
         <is>
           <t>https://www.key4.com/uploads/files/products/metal_keys/AC-ILC-KEYDIR13/Key_Blank_Directory_-_Edition_13.pdf</t>
         </is>
@@ -12026,7 +12026,7 @@
           <t>Keydiy / Xhorse HU43 #Y-18 Flip Key Blade (검색 결과)</t>
         </is>
       </c>
-      <c r="E303" s="7" t="inlineStr">
+      <c r="E303" s="6" t="inlineStr">
         <is>
           <t>https://keystation.co.uk/vehicle-makes/vauxhall-keys-parts/vauxhall-opel-car-key-blades</t>
         </is>
@@ -12053,7 +12053,7 @@
           <t>Flip Key Blade - OPEL (Like: OP-WH / HU43) - Laser Key, Art ID OP#Y-18</t>
         </is>
       </c>
-      <c r="E304" s="7" t="inlineStr">
+      <c r="E304" s="6" t="inlineStr">
         <is>
           <t>https://www.sglocks.com.au/product/15635-flip-key-blade-opel-like-op-wh-hu43-laser-key</t>
         </is>
@@ -12080,7 +12080,7 @@
           <t>KeyDiy KD Y18 for Xhorse Opel Holden Chevrolet Insert Key, Blade Profile HU43</t>
         </is>
       </c>
-      <c r="E305" s="7" t="inlineStr">
+      <c r="E305" s="6" t="inlineStr">
         <is>
           <t>https://www.tlkeys.com/products/KeyDiy-KD-Y18-for-Xhorse-Opel-Holden-Chevrolet-Insert-Key-34353</t>
         </is>
@@ -12107,7 +12107,7 @@
           <t>OP-D = ERREBI YM24, ILCO HF59R, SILCA YM28 / 차종: DAEWOO ® | LE MANS | 1983-1984 | GM (CHEVROLET BRA.) ® | CHE</t>
         </is>
       </c>
-      <c r="E306" s="7" t="inlineStr">
+      <c r="E306" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/op-d/8894/</t>
         </is>
@@ -12134,7 +12134,7 @@
           <t>Silca YM28 = Ilco HF59R</t>
         </is>
       </c>
-      <c r="E307" s="7" t="inlineStr">
+      <c r="E307" s="6" t="inlineStr">
         <is>
           <t>https://www.key4.com/uploads/files/products/metal_keys/AC-ILC-KEYDIR13/Key_Blank_Directory_-_Edition_13.pdf</t>
         </is>
@@ -12161,7 +12161,7 @@
           <t>YM28 OP-D For Vauxhall, Blade number 68</t>
         </is>
       </c>
-      <c r="E308" s="7" t="inlineStr">
+      <c r="E308" s="6" t="inlineStr">
         <is>
           <t>https://accessfobs.co.uk/products/blade-for-keydiy-and-xhorse-remote-ym28</t>
         </is>
@@ -12188,7 +12188,7 @@
           <t>Key4 YM28 키날 사진, 각인 68</t>
         </is>
       </c>
-      <c r="E309" s="7" t="inlineStr">
+      <c r="E309" s="6" t="inlineStr">
         <is>
           <t>https://www.key4.com/uploads/files/products/key_blades/KB-KDY-YM28/KB-KDY-YM28_photo.jpg</t>
         </is>
@@ -12215,7 +12215,7 @@
           <t>Keydiy / Xhorse YM28 #68 Flip Key Blade</t>
         </is>
       </c>
-      <c r="E310" s="7" t="inlineStr">
+      <c r="E310" s="6" t="inlineStr">
         <is>
           <t>https://keystation.co.uk/keydiy-xhorse-ym28-68-flip-key-blade</t>
         </is>
@@ -12242,7 +12242,7 @@
           <t>KEYDIY Remote Flip Key Blade YM28 for Opel Corsa (Right Slot) (68#)</t>
         </is>
       </c>
-      <c r="E311" s="7" t="inlineStr">
+      <c r="E311" s="6" t="inlineStr">
         <is>
           <t>https://www.locksmithkeyless.com/products/keydiy-remote-flip-key-blade-ym28-for-opel-corsa-right-slot-68</t>
         </is>
@@ -12269,7 +12269,7 @@
           <t>VD9521-Universal Flip Remote key Blade YM28 Opel, part number 68 (검색 결과)</t>
         </is>
       </c>
-      <c r="E312" s="7" t="inlineStr">
+      <c r="E312" s="6" t="inlineStr">
         <is>
           <t>https://www.vvdi.com/kd900-blade-for-opel-flip-remote-ym28</t>
         </is>
@@ -12296,7 +12296,7 @@
           <t>KEYDIY blade 68# for Opel(right slot) YM28</t>
         </is>
       </c>
-      <c r="E313" s="7" t="inlineStr">
+      <c r="E313" s="6" t="inlineStr">
         <is>
           <t>https://www.5akeys.com/keydiy-blade-68-for-opelright-slot-ym28_p0091.html</t>
         </is>
@@ -12346,7 +12346,7 @@
           <t>DAE-3D = SILCA DWO4R / 차종: DAEWOO ® | NUBIRA | 1997-2000 | DAEWOO ® | TACUMA | 2000-200</t>
         </is>
       </c>
-      <c r="E315" s="7" t="inlineStr">
+      <c r="E315" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/dae-3d/3300/</t>
         </is>
@@ -12373,7 +12373,7 @@
           <t>DAE-3DP4 = ILCO DW04RAP, SILCA DWO4REP</t>
         </is>
       </c>
-      <c r="E316" s="7" t="inlineStr">
+      <c r="E316" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/dae-3dp4/3307/</t>
         </is>
@@ -12400,7 +12400,7 @@
           <t>DWO4R - #39 Y-11 - UB10027 (GM / Subaru)</t>
         </is>
       </c>
-      <c r="E317" s="7" t="inlineStr">
+      <c r="E317" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -12427,7 +12427,7 @@
           <t>Silca DWO4R = JMA DAE-3D, 상품 코드 DAE#Y-11</t>
         </is>
       </c>
-      <c r="E318" s="7" t="inlineStr">
+      <c r="E318" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2157&amp;controller=product</t>
         </is>
@@ -12469,7 +12469,7 @@
           <t>KeyDiy Xhorse Remote Key Blade For Chevrolet DWO4 (ABK-59), 사진 각인 05, 스파크 2004-2010</t>
         </is>
       </c>
-      <c r="E320" s="7" t="inlineStr">
+      <c r="E320" s="6" t="inlineStr">
         <is>
           <t>https://abkeys.com/products/chevrolet-dwo4-keydiy-xhorse-remote-key-blade-0059</t>
         </is>
@@ -12519,7 +12519,7 @@
           <t>DAE-4P1 = ERREBI DW1P140, ILCO DW05AP, SILCA DWO5AP / 차종: DAEWOO (USA) ® | LEGANZA | 1998-2005 | DAEWOO ® | LANOS | 19</t>
         </is>
       </c>
-      <c r="E322" s="7" t="inlineStr">
+      <c r="E322" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/dae-4p1/3315/</t>
         </is>
@@ -12546,7 +12546,7 @@
           <t>DWO5 - #40 Y-17 - UB10032 (GM / Subaru)</t>
         </is>
       </c>
-      <c r="E323" s="7" t="inlineStr">
+      <c r="E323" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -12573,7 +12573,7 @@
           <t>Silca DWO5 = JMA DAE-4, 상품 코드 DAE#Y-17</t>
         </is>
       </c>
-      <c r="E324" s="7" t="inlineStr">
+      <c r="E324" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2158&amp;controller=product</t>
         </is>
@@ -12623,7 +12623,7 @@
           <t>DAE-4D = SILCA DWO5R / 차종: DAEWOO ® | LEGANZA | 1997-</t>
         </is>
       </c>
-      <c r="E326" s="7" t="inlineStr">
+      <c r="E326" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/dae-4d/3311/</t>
         </is>
@@ -12650,7 +12650,7 @@
           <t>Keydiy Xhorse Universal Flip Remote key Blade RIGHT SIDE DW05R Chevrolet (#181 / Y-12)</t>
         </is>
       </c>
-      <c r="E327" s="7" t="inlineStr">
+      <c r="E327" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/keydiy-xhorse-universal-flip-remote-key-blade-dwo5r-chevrolet-1</t>
         </is>
@@ -12677,7 +12677,7 @@
           <t>DWO5R - #13 Y-12 - UB10028 (GM / Subaru)</t>
         </is>
       </c>
-      <c r="E328" s="7" t="inlineStr">
+      <c r="E328" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -12704,7 +12704,7 @@
           <t>DWO5R DAE-4D For Chevrolet, Daewoo, Vauxhall or Suzuki, Blank number Y-12</t>
         </is>
       </c>
-      <c r="E329" s="7" t="inlineStr">
+      <c r="E329" s="6" t="inlineStr">
         <is>
           <t>https://accessfobs.co.uk/products/blade-for-keydiy-and-xhorse-remote-dwo5r</t>
         </is>
@@ -12731,7 +12731,7 @@
           <t>Chevrolet DWO5R Blade 12# for Xhorse &amp; KEYDIY Universal Remotes</t>
         </is>
       </c>
-      <c r="E330" s="7" t="inlineStr">
+      <c r="E330" s="6" t="inlineStr">
         <is>
           <t>https://keyinnovations.com/products/keyless2go-chevrolet-dwo5r-blade-12</t>
         </is>
@@ -12758,7 +12758,7 @@
           <t>Keydiy KD Xhorse VVDI Universal Flip Remote Key Blade #93 DWO5R Chevrolet</t>
         </is>
       </c>
-      <c r="E331" s="7" t="inlineStr">
+      <c r="E331" s="6" t="inlineStr">
         <is>
           <t>https://gskeyae.com/product/keydiy-xhorse-flip-key-blade-93-dwo5r-chevrolet/</t>
         </is>
@@ -12785,7 +12785,7 @@
           <t>FO-15D = ERREBI FD18R, EZ H75, H86, H72, ILCO 1196FD / 차종: FORD (AUSTRALIA) ® | EXPLORER | 1996-1997 | FORD (AUSTRALIA)</t>
         </is>
       </c>
-      <c r="E332" s="7" t="inlineStr">
+      <c r="E332" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/fo-15d/4576/</t>
         </is>
@@ -12812,7 +12812,7 @@
           <t>FO-43D = ERREBI FD18R, EZ H75, ILCO 1196FD, SILCA FO40R / 차종: FORD ® | VARIOUS BRANDS | -</t>
         </is>
       </c>
-      <c r="E333" s="7" t="inlineStr">
+      <c r="E333" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/fo-43d/4646/</t>
         </is>
@@ -12839,7 +12839,7 @@
           <t xml:space="preserve">TP00FO-15DP = ERREBI T00FD16RP, SILCA FO38RTE / 차종: FORD (ARGENTINA) ® | PICK UP | 1993-1994 | FORD (ARGENTINA) </t>
         </is>
       </c>
-      <c r="E334" s="7" t="inlineStr">
+      <c r="E334" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/tp00fo-15dp/11501/</t>
         </is>
@@ -12866,7 +12866,7 @@
           <t>KEYDIY - H75 / FO38 - Flip Key Blade - #19 - For Xhorse / Keydiy Universal Remote Flip Keys</t>
         </is>
       </c>
-      <c r="E335" s="7" t="inlineStr">
+      <c r="E335" s="6" t="inlineStr">
         <is>
           <t>https://www.uhs-hardware.com/products/keydiy-h75-fo38-flip-key-blade-19-for-xhorse-keydiy-universal-remote-flip-keys</t>
         </is>
@@ -12893,7 +12893,7 @@
           <t>H75 / FO38 - #19 - UB10007 (Ford / Mazda)</t>
         </is>
       </c>
-      <c r="E336" s="7" t="inlineStr">
+      <c r="E336" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -12920,7 +12920,7 @@
           <t>Silca FO38R = JMA FO-15D, 상품 코드 FO#19</t>
         </is>
       </c>
-      <c r="E337" s="7" t="inlineStr">
+      <c r="E337" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2137&amp;controller=product</t>
         </is>
@@ -12947,7 +12947,7 @@
           <t>FO-24C1 = ERREBI HF65C1, SILCA HU101T / 차종: FORD ® | C-MAX | 2010-2019 | FORD ® | FOCUS | 2011-2019 | FO</t>
         </is>
       </c>
-      <c r="E338" s="7" t="inlineStr">
+      <c r="E338" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/fo-24c1/4599/</t>
         </is>
@@ -12974,7 +12974,7 @@
           <t>KEYDIY - HU101 - Flip Key Blade - #38 - For Xhorse / Keydiy Universal Remote Flip Keys</t>
         </is>
       </c>
-      <c r="E339" s="7" t="inlineStr">
+      <c r="E339" s="6" t="inlineStr">
         <is>
           <t>https://www.uhs-hardware.com/products/keydiy-hu101-flip-key-blade-38-for-xhorse-keydiy-universal-remote-flip-keys</t>
         </is>
@@ -13001,7 +13001,7 @@
           <t>HU101 - #38 - UB10014 (Ford / Volvo / JLR)</t>
         </is>
       </c>
-      <c r="E340" s="7" t="inlineStr">
+      <c r="E340" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -13028,7 +13028,7 @@
           <t>Silca HU101 = JMA FO-24, 상품 코드 FO#38</t>
         </is>
       </c>
-      <c r="E341" s="7" t="inlineStr">
+      <c r="E341" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2138&amp;controller=product</t>
         </is>
@@ -13055,7 +13055,7 @@
           <t>FO-6P = ERREBI TB1P5, ILCO S30FDP, SILCA FO21P / 차종: FORD (ARGENTINA) ® | ESCORT | 1988-1995 | FORD (ARGENTINA) ®</t>
         </is>
       </c>
-      <c r="E342" s="7" t="inlineStr">
+      <c r="E342" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/fo-6p/4652/</t>
         </is>
@@ -13082,7 +13082,7 @@
           <t>FO21 - #90 Y-39 - UB10041 (Ford Mondeo / Jaguar)</t>
         </is>
       </c>
-      <c r="E343" s="7" t="inlineStr">
+      <c r="E343" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -13109,7 +13109,7 @@
           <t>KEYDIY - FO21 - Flip Key Blade - #Y39 - Unmarked - For Xhorse / Keydiy Universal Remote Flip Keys</t>
         </is>
       </c>
-      <c r="E344" s="7" t="inlineStr">
+      <c r="E344" s="6" t="inlineStr">
         <is>
           <t>https://www.uhs-hardware.com/products/keydiy-fo21-flip-key-blade-y39-unmarked-for-xhorse-keydiy-universal-remote-flip-keys</t>
         </is>
@@ -13136,7 +13136,7 @@
           <t>Silca FO21 = JMA FO-6, 상품 코드 FO#Y-39</t>
         </is>
       </c>
-      <c r="E345" s="7" t="inlineStr">
+      <c r="E345" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2139&amp;controller=product</t>
         </is>
@@ -13163,7 +13163,7 @@
           <t>NE-52P = ERREBI NE77P91, EZ RV4P, ILCO RV4P, SILCA NE75EP / 차종: LAND-RANGE ROVER ® | DISCOVERY | 1994-1997 | ROVER ® | 820 |</t>
         </is>
       </c>
-      <c r="E346" s="7" t="inlineStr">
+      <c r="E346" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/ne-52p/8686/</t>
         </is>
@@ -13190,7 +13190,7 @@
           <t>NE-35 = ERREBI NE74, ILCO NE71R, SILCA NE71R / 차종: HONDA ® | ACCORD 2 LS | 1993-1995 | HONDA ® | ACCORD 2 S | 1</t>
         </is>
       </c>
-      <c r="E347" s="7" t="inlineStr">
+      <c r="E347" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/ne-35/8606/</t>
         </is>
@@ -13217,7 +13217,7 @@
           <t>KeyDIY Land Rover NE75 Universal Key Blade (Y-20#)</t>
         </is>
       </c>
-      <c r="E348" s="7" t="inlineStr">
+      <c r="E348" s="6" t="inlineStr">
         <is>
           <t>https://keyinnovations.com/products/kd-y-20-5pack</t>
         </is>
@@ -13244,7 +13244,7 @@
           <t>NE71R RV3 - Y-20 - UB10033 (JLR)</t>
         </is>
       </c>
-      <c r="E349" s="7" t="inlineStr">
+      <c r="E349" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -13271,7 +13271,7 @@
           <t>KEYDIY Remote Flip Key Blade NE71R for Land Rover (RV3) (Y-20#)</t>
         </is>
       </c>
-      <c r="E350" s="7" t="inlineStr">
+      <c r="E350" s="6" t="inlineStr">
         <is>
           <t>https://www.locksmithkeyless.com/products/keydiy-remote-flip-key-blade-ne71r-for-land-rover-rv3-y-20</t>
         </is>
@@ -13298,7 +13298,7 @@
           <t>Y-20# NE71R Land Rover NE38 / Xhorse / Keydiy Blade</t>
         </is>
       </c>
-      <c r="E351" s="7" t="inlineStr">
+      <c r="E351" s="6" t="inlineStr">
         <is>
           <t>https://www.keylocksupplies.com/products/y-20-land-rover-ne38-xhorse-keydiy-blade</t>
         </is>
@@ -13325,7 +13325,7 @@
           <t>CHR-14 = ERREBI CY61, EZ Y157, ILCO P1794, SILCA CY22 / 차종: AMERICAN MOTORS ® | VARIOUS MODELS | - | CHRYSLER ® | GR. VO</t>
         </is>
       </c>
-      <c r="E352" s="7" t="inlineStr">
+      <c r="E352" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/chr-14/2495/</t>
         </is>
@@ -13352,7 +13352,7 @@
           <t xml:space="preserve">CHR-15 = ERREBI CY62, EZ Y159, ILCO P1795, Y168, Y164, SILCA CY24 / 차종: CHRYSLER ® | GR. VOYAGER | 1996-1997 | CHRYSLER ® | STRATUS </t>
         </is>
       </c>
-      <c r="E353" s="7" t="inlineStr">
+      <c r="E353" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/chr-15/2501/</t>
         </is>
@@ -13379,7 +13379,7 @@
           <t>Y159 - #04 Y-35 - UB10039 (Chrysler / Dodge / Jeep)</t>
         </is>
       </c>
-      <c r="E354" s="7" t="inlineStr">
+      <c r="E354" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -13406,7 +13406,7 @@
           <t>KEYDIY - Y157 / Y159 / CY24 - Flip Key Blade - #Y35 - For Xhorse / Keydiy Universal Remote Flip Keys</t>
         </is>
       </c>
-      <c r="E355" s="7" t="inlineStr">
+      <c r="E355" s="6" t="inlineStr">
         <is>
           <t>https://www.uhs-hardware.com/products/keydiy-y157-y159-cy24-flip-key-blade-y35-for-xhorse-keydiy-universal-remote-flip-keys</t>
         </is>
@@ -13433,7 +13433,7 @@
           <t>Silca CY24 = JMA CHR-15, 상품 코드 CHR#Y-35</t>
         </is>
       </c>
-      <c r="E356" s="7" t="inlineStr">
+      <c r="E356" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2155&amp;controller=product</t>
         </is>
@@ -13460,7 +13460,7 @@
           <t>FI-16P1 = ERREBI GB18P174, SILCA SIP22KP / 차종: ABARTH ® | 500 | 2008- | ABARTH ® | GRANDE PUNTO | 2007-2010</t>
         </is>
       </c>
-      <c r="E357" s="7" t="inlineStr">
+      <c r="E357" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/fi-16p1/4447/</t>
         </is>
@@ -13487,7 +13487,7 @@
           <t>SIP22 - #157 Y-37 - UB10040 (FCA / PSA / Ferrari / Ford)</t>
         </is>
       </c>
-      <c r="E358" s="7" t="inlineStr">
+      <c r="E358" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -13514,7 +13514,7 @@
           <t>KEYDIY - SIP22 - Flip Key Blade - #Y37 - For Xhorse / Keydiy Universal Remote Flip Keys</t>
         </is>
       </c>
-      <c r="E359" s="7" t="inlineStr">
+      <c r="E359" s="6" t="inlineStr">
         <is>
           <t>https://www.uhs-hardware.com/products/keydiy-sip22-flip-key-blade-y37-for-xhorse-keydiy-universal-remote-flip-keys</t>
         </is>
@@ -13541,7 +13541,7 @@
           <t>Silca SIP22 = JMA FI-16, 상품 코드 FI#Y-37</t>
         </is>
       </c>
-      <c r="E360" s="7" t="inlineStr">
+      <c r="E360" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2159&amp;controller=product</t>
         </is>
@@ -13568,7 +13568,7 @@
           <t>SIP22 FI-16 For Fiat, Key number #157 (Shorter blade)</t>
         </is>
       </c>
-      <c r="E361" s="7" t="inlineStr">
+      <c r="E361" s="6" t="inlineStr">
         <is>
           <t>https://accessfobs.co.uk/products/copy-of-blade-for-keydiy-and-xhorse-remote-sip22</t>
         </is>
@@ -13595,7 +13595,7 @@
           <t>SIP22 FI-16 For Fiat, Key number #Y-37 (longer blade)</t>
         </is>
       </c>
-      <c r="E362" s="7" t="inlineStr">
+      <c r="E362" s="6" t="inlineStr">
         <is>
           <t>https://accessfobs.co.uk/products/blade-for-keydiy-and-xhorse-remote-sip22</t>
         </is>
@@ -13622,7 +13622,7 @@
           <t>KEYDIY Key Blade-SIP22 #157 (Y37) For Xhorse / Keydiy Universal Remote Flip Keys</t>
         </is>
       </c>
-      <c r="E363" s="7" t="inlineStr">
+      <c r="E363" s="6" t="inlineStr">
         <is>
           <t>https://keydirect.ca/product/keydiy-key-blade-sip22-y37/</t>
         </is>
@@ -13649,7 +13649,7 @@
           <t>Keydiy 157 Flip Insert Key Blade for Fiat Iveco Alfa Romeo, Profile SIP22</t>
         </is>
       </c>
-      <c r="E364" s="7" t="inlineStr">
+      <c r="E364" s="6" t="inlineStr">
         <is>
           <t>https://www.tlkeys.com/products/Keydiy-157-Flip-Insert-Key-Blade-for-Fiat-Iveco-Alfa-Romeo-33280</t>
         </is>
@@ -13676,7 +13676,7 @@
           <t>VD9554-Universal Flip Remote key Blade Fiat (small), part number 157 (검색 결과)</t>
         </is>
       </c>
-      <c r="E365" s="7" t="inlineStr">
+      <c r="E365" s="6" t="inlineStr">
         <is>
           <t>https://www.vvdi.com/kd900-small-blade-for-fiat-flip-remote-key</t>
         </is>
@@ -13703,7 +13703,7 @@
           <t>HU-HAAP1 = ERREBI HF55P65, SILCA HU66P / 차종: VOLKSWAGEN ® | VARIOUS MODELS | -</t>
         </is>
       </c>
-      <c r="E366" s="7" t="inlineStr">
+      <c r="E366" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/hu-haap1/5778/</t>
         </is>
@@ -13730,7 +13730,7 @@
           <t>HU66 - #86 - UB10023 (VAG)</t>
         </is>
       </c>
-      <c r="E367" s="7" t="inlineStr">
+      <c r="E367" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -13757,7 +13757,7 @@
           <t>KEYDIY - HU66 - Flip Key Blade - #31 - For Xhorse / Keydiy Universal Remote Flip Keys</t>
         </is>
       </c>
-      <c r="E368" s="7" t="inlineStr">
+      <c r="E368" s="6" t="inlineStr">
         <is>
           <t>https://www.uhs-hardware.com/products/keydiy-hu66-flip-key-blade-31-for-xhorse-keydiy-universal-remote-flip-keys</t>
         </is>
@@ -13784,7 +13784,7 @@
           <t>Silca HU66 = JMA HU-HAA, 상품 코드 HU#86</t>
         </is>
       </c>
-      <c r="E369" s="7" t="inlineStr">
+      <c r="E369" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2141&amp;controller=product</t>
         </is>
@@ -13811,7 +13811,7 @@
           <t>HU66 HU-HAA, Blank number 86, length 50mm</t>
         </is>
       </c>
-      <c r="E370" s="7" t="inlineStr">
+      <c r="E370" s="6" t="inlineStr">
         <is>
           <t>https://accessfobs.co.uk/products/blade-for-keydiy-and-xhorse-remote-blade-hu66</t>
         </is>
@@ -13838,7 +13838,7 @@
           <t>HU66, Blank number #31, Length 48mm (from top to bottom)</t>
         </is>
       </c>
-      <c r="E371" s="7" t="inlineStr">
+      <c r="E371" s="6" t="inlineStr">
         <is>
           <t>https://accessfobs.co.uk/products/blade-for-keydiy-and-xhorse-remote-hu66</t>
         </is>
@@ -13865,7 +13865,7 @@
           <t>HU-4C1 = SILCA HU162T</t>
         </is>
       </c>
-      <c r="E372" s="7" t="inlineStr">
+      <c r="E372" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/hu-4c1/5738/</t>
         </is>
@@ -13892,7 +13892,7 @@
           <t>HU-7C1 = ERREBI HF74C1, SILCA HU162AT</t>
         </is>
       </c>
-      <c r="E373" s="7" t="inlineStr">
+      <c r="E373" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/hu-7c1/5739/</t>
         </is>
@@ -13919,7 +13919,7 @@
           <t>HU162 - #149 Y-09 - UB10026 (VAG)</t>
         </is>
       </c>
-      <c r="E374" s="7" t="inlineStr">
+      <c r="E374" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -13946,7 +13946,7 @@
           <t>KEYDIY - HU162 - Switch Blade - #149 - Volkswagen For Xhorse &amp; KEYDIY Universal Remotes</t>
         </is>
       </c>
-      <c r="E375" s="7" t="inlineStr">
+      <c r="E375" s="6" t="inlineStr">
         <is>
           <t>https://www.uhs-hardware.com/products/keydiy-hu162-switch-blade-149-volkswagen-for-xhorse-keydiy-universal-remotes</t>
         </is>
@@ -13973,7 +13973,7 @@
           <t>Blade KEYDIY/XHORSE #Y-09 HU162T</t>
         </is>
       </c>
-      <c r="E376" s="7" t="inlineStr">
+      <c r="E376" s="6" t="inlineStr">
         <is>
           <t>https://a-d-e.pl/blades-blade-keydiy/xhorse-y-09-hu162t,c146,p3983,o1001,s1001,en.html</t>
         </is>
@@ -14000,7 +14000,7 @@
           <t>(Pack of 30) KEYDIY Key Blade-VW HU162T / #149 (KD-VW-149)</t>
         </is>
       </c>
-      <c r="E377" s="7" t="inlineStr">
+      <c r="E377" s="6" t="inlineStr">
         <is>
           <t>https://keydirect.ca/product/pack-of-30-keydiy-key-blade-vw-hu162t-149-kd-vw-149-for-xhorse-keydiy-universal-remote-flip-keys/</t>
         </is>
@@ -14027,7 +14027,7 @@
           <t>VO-2 = ERREBI HF44T, ILCO V37, SILCA HU49 / 차종: ABT ® | GOLF 3 | 1991- | AUDI ® | 100 | 1985- | AUDI ® | 200</t>
         </is>
       </c>
-      <c r="E378" s="7" t="inlineStr">
+      <c r="E378" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/vo-2/13537/</t>
         </is>
@@ -14054,7 +14054,7 @@
           <t>AU-AH = ERREBI HF44N, HF44T, ILCO V35, SILCA HU49 / 차종: ABT ® | GOLF 3 | 1991- | AUDI ® | 100 | 1985- | AUDI ® | 200</t>
         </is>
       </c>
-      <c r="E379" s="7" t="inlineStr">
+      <c r="E379" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/au-ah/1342/</t>
         </is>
@@ -14081,7 +14081,7 @@
           <t>HU49 - #01 - UB10062 (Double-Sided VAG)</t>
         </is>
       </c>
-      <c r="E380" s="7" t="inlineStr">
+      <c r="E380" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -14108,7 +14108,7 @@
           <t>HU49 Xhorse KeyDIY Flip Key Blade Replacement #01</t>
         </is>
       </c>
-      <c r="E381" s="7" t="inlineStr">
+      <c r="E381" s="6" t="inlineStr">
         <is>
           <t>https://www.bestkeysupply.com/products/hu49-xhorse-keydiy-universal-flipkey-insert-01-b159bks</t>
         </is>
@@ -14158,7 +14158,7 @@
           <t xml:space="preserve">BM-6P = ERREBI HF70P171, SILCA HU92RP / 차종: BMW (USA) ® | VARIOUS MODELS | - | BMW ® | VARIOUS MODELS | </t>
         </is>
       </c>
-      <c r="E383" s="7" t="inlineStr">
+      <c r="E383" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/bm-6p/1742/</t>
         </is>
@@ -14185,7 +14185,7 @@
           <t>KEYDIY - HU92 - Flip Key Blade - #67 - For Xhorse / Keydiy Universal Remote Flip Keys</t>
         </is>
       </c>
-      <c r="E384" s="7" t="inlineStr">
+      <c r="E384" s="6" t="inlineStr">
         <is>
           <t>https://www.uhs-hardware.com/products/keydiy-hu92-flip-key-blade-67-for-xhorse-keydiy-universal-remote-flip-keys</t>
         </is>
@@ -14212,7 +14212,7 @@
           <t>HU92 - #67 - UB10018 (BMW / Mini)</t>
         </is>
       </c>
-      <c r="E385" s="7" t="inlineStr">
+      <c r="E385" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -14239,7 +14239,7 @@
           <t>Silca HU92 = JMA BM-6, 상품 코드 BMW#67</t>
         </is>
       </c>
-      <c r="E386" s="7" t="inlineStr">
+      <c r="E386" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2154&amp;controller=product</t>
         </is>
@@ -14289,7 +14289,7 @@
           <t xml:space="preserve">BM-5P = ERREBI HF48P8, ILCO S7BWP, SILCA HU58AP / 차종: BMW ® | SERIE 3 | 1990-1995 | BMW ® | SERIE 5 | 1988-1995 | </t>
         </is>
       </c>
-      <c r="E388" s="7" t="inlineStr">
+      <c r="E388" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/bm-5p/1739/</t>
         </is>
@@ -14316,7 +14316,7 @@
           <t>KEYDIY - HU58 - Flip Key Blade - #18 - For Xhorse / Keydiy Universal Remote Flip Keys</t>
         </is>
       </c>
-      <c r="E389" s="7" t="inlineStr">
+      <c r="E389" s="6" t="inlineStr">
         <is>
           <t>https://www.uhs-hardware.com/products/keydiy-hu58-flip-key-blade-18-for-xhorse-keydiy-universal-remote-flip-keys</t>
         </is>
@@ -14343,7 +14343,7 @@
           <t>HU58 - #18 - UB10006 (BMW / Mini)</t>
         </is>
       </c>
-      <c r="E390" s="7" t="inlineStr">
+      <c r="E390" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -14389,7 +14389,7 @@
           <t>ME-7P = ERREBI HF51P17, ILCO S34YSP, SILCA HU64P / 차종: MERCEDES ® | 180C | 1993- | MERCEDES ® | 200C | 1993- | MERC</t>
         </is>
       </c>
-      <c r="E392" s="7" t="inlineStr">
+      <c r="E392" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/me-7p/7981/</t>
         </is>
@@ -14416,7 +14416,7 @@
           <t>HU64 - Y-65 - UB10044 (Mercedes-Benz)</t>
         </is>
       </c>
-      <c r="E393" s="7" t="inlineStr">
+      <c r="E393" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -14443,7 +14443,7 @@
           <t>Mercedes-Benz HU64 - 20# - Key Blade for Xhorse &amp; KeyDIY Universal Remotes (Pack of 10)</t>
         </is>
       </c>
-      <c r="E394" s="7" t="inlineStr">
+      <c r="E394" s="6" t="inlineStr">
         <is>
           <t>https://autorescuetools.com/products/20-hu64-mercedes-benz-key-blade-for-xhorse-keydiy-universal-remotes-pack-of-10x</t>
         </is>
@@ -14470,7 +14470,7 @@
           <t>Silca HU64 = JMA ME-7, 상품 코드 Y65</t>
         </is>
       </c>
-      <c r="E395" s="7" t="inlineStr">
+      <c r="E395" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2854&amp;controller=product</t>
         </is>
@@ -14497,7 +14497,7 @@
           <t>ME-2P = ERREBI HF39P17, ILCO S48HFP, SILCA HU39P / 차종: MERCEDES ® | 1000 | 1984- | MERCEDES ® | 190 | 1984-1986 | M</t>
         </is>
       </c>
-      <c r="E396" s="7" t="inlineStr">
+      <c r="E396" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/me-2p/7968/</t>
         </is>
@@ -14524,7 +14524,7 @@
           <t>Mercedes Keydiy HU39 Flip Keyblade - Blade11</t>
         </is>
       </c>
-      <c r="E397" s="7" t="inlineStr">
+      <c r="E397" s="6" t="inlineStr">
         <is>
           <t>https://remkeys.com/product/mercedes-keydiy-hu39-flip-keyblade-blade11-mekb11-remkeys/</t>
         </is>
@@ -14551,7 +14551,7 @@
           <t>KEYDIY Xhorse Flip Remote Key Blade #11 HU39 Mercedes</t>
         </is>
       </c>
-      <c r="E398" s="7" t="inlineStr">
+      <c r="E398" s="6" t="inlineStr">
         <is>
           <t>https://gskeyae.com/product/keydiy-flip-key-remote-blade-11-mercedes-benz-hu39/</t>
         </is>
@@ -14574,7 +14574,7 @@
           <t>ME-HM = ERREBI YMNF, ILCO MB17, SILCA YM15 / 차종: MERCEDES ® | 207D | -1992 | MERCEDES ® | 207F | -1992 | MERC</t>
         </is>
       </c>
-      <c r="E399" s="7" t="inlineStr">
+      <c r="E399" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/me-hm/8007/</t>
         </is>
@@ -14597,7 +14597,7 @@
           <t>Silca YM15 = Ilco MB17</t>
         </is>
       </c>
-      <c r="E400" s="7" t="inlineStr">
+      <c r="E400" s="6" t="inlineStr">
         <is>
           <t>https://www.key4.com/uploads/files/products/metal_keys/AC-ILC-KEYDIR13/Key_Blank_Directory_-_Edition_13.pdf</t>
         </is>
@@ -14620,7 +14620,7 @@
           <t>Mercedes YM15 VA5-I, Blank number 226#, Sprinter 1997-2007 등</t>
         </is>
       </c>
-      <c r="E401" s="7" t="inlineStr">
+      <c r="E401" s="6" t="inlineStr">
         <is>
           <t>https://accessfobs.co.uk/products/blade-for-keydiy-xhorse-key-blade-ym15-for-mercedes</t>
         </is>
@@ -14647,7 +14647,7 @@
           <t xml:space="preserve">TP00HU-HCAP = ERREBI T00HF63P, SILCA HU83TE / 차종: CITROEN ® | VARIOUS MODELS | - | PEUGEOT ® | VARIOUS MODELS </t>
         </is>
       </c>
-      <c r="E402" s="7" t="inlineStr">
+      <c r="E402" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/tp00hu-hcap/11536/</t>
         </is>
@@ -14674,7 +14674,7 @@
           <t>HU83 - #54 Y-31 - UB10038 (PSA / Fiat)</t>
         </is>
       </c>
-      <c r="E403" s="7" t="inlineStr">
+      <c r="E403" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -14701,7 +14701,7 @@
           <t>Silca HU83 = JMA HU-HCA, 상품 코드 HU#Y-31</t>
         </is>
       </c>
-      <c r="E404" s="7" t="inlineStr">
+      <c r="E404" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2161&amp;controller=product</t>
         </is>
@@ -14728,7 +14728,7 @@
           <t>Keydiy 54 Flip Folding Blank Remote Car Key Blade, Blade Profile HU83</t>
         </is>
       </c>
-      <c r="E405" s="7" t="inlineStr">
+      <c r="E405" s="6" t="inlineStr">
         <is>
           <t>https://www.tlkeys.com/products/Keydiy-54-New-ArrivalL-Flip-Folding-Blank-Remote-Car-Key-Bl-33126</t>
         </is>
@@ -14755,7 +14755,7 @@
           <t>KDIY key blade 54# Y-31# HU83 flip Key Blade With Grooves For Citroen for Peugeot</t>
         </is>
       </c>
-      <c r="E406" s="7" t="inlineStr">
+      <c r="E406" s="6" t="inlineStr">
         <is>
           <t>https://chipkeysupply.com/products/kdiy-key-blade-54-hu83-flip-key-blade-with-grooves-for-citroen-for-peugeot</t>
         </is>
@@ -14782,7 +14782,7 @@
           <t>10pcs 54# HU83 Metal Uncut Blank Flip Remote Key Blade for Peugeot 407 Citroen</t>
         </is>
       </c>
-      <c r="E407" s="7" t="inlineStr">
+      <c r="E407" s="6" t="inlineStr">
         <is>
           <t>https://www.aliexpress.us/item/3256803249326222.html</t>
         </is>
@@ -14832,7 +14832,7 @@
           <t>TP00CIT-1P = ERREBI T00VA1P, SILCA VA2TE</t>
         </is>
       </c>
-      <c r="E409" s="7" t="inlineStr">
+      <c r="E409" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/tp00cit-1p/11467/</t>
         </is>
@@ -14859,7 +14859,7 @@
           <t>HT-1 = ERREBI HTV1R, ILCO VA2, SILCA HT1</t>
         </is>
       </c>
-      <c r="E410" s="7" t="inlineStr">
+      <c r="E410" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/ht-1/5729/</t>
         </is>
@@ -14886,7 +14886,7 @@
           <t>VA2 - #58 Y-29 - UB10036 (FCA / Hyundai / Kia / PSA / Renault / Dacia)</t>
         </is>
       </c>
-      <c r="E411" s="7" t="inlineStr">
+      <c r="E411" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -14913,7 +14913,7 @@
           <t>KEYDIY - VA2T - Flip Key Blade - #Y29 - For Xhorse / Keydiy Universal Remote Flip Keys</t>
         </is>
       </c>
-      <c r="E412" s="7" t="inlineStr">
+      <c r="E412" s="6" t="inlineStr">
         <is>
           <t>https://www.uhs-hardware.com/products/keydiy-va2t-flip-key-blade-y29-for-xhorse-keydiy-universal-remote-flip-keys</t>
         </is>
@@ -14940,7 +14940,7 @@
           <t>Silca VA2T = JMA CIT-1, 상품 코드 CIT#Y-29</t>
         </is>
       </c>
-      <c r="E413" s="7" t="inlineStr">
+      <c r="E413" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2156&amp;controller=product</t>
         </is>
@@ -14990,7 +14990,7 @@
           <t>Cross Reference: VA2/VA6, CIT-1</t>
         </is>
       </c>
-      <c r="E415" s="7" t="inlineStr">
+      <c r="E415" s="6" t="inlineStr">
         <is>
           <t>https://www.key4.com/flip-remote-key-blade-peugeot-citroen-va2-va6</t>
         </is>
@@ -15017,7 +15017,7 @@
           <t>Blank Reference VA2/ VA6, Blade number Y29#, For Peugeot, Toyota, Citroen</t>
         </is>
       </c>
-      <c r="E416" s="7" t="inlineStr">
+      <c r="E416" s="6" t="inlineStr">
         <is>
           <t>https://accessfobs.co.uk/products/va2-va6-flip-key-blade-xhorse-key-diy</t>
         </is>
@@ -15044,7 +15044,7 @@
           <t>Key4 VA6 키날 사진, 각인 58</t>
         </is>
       </c>
-      <c r="E417" s="7" t="inlineStr">
+      <c r="E417" s="6" t="inlineStr">
         <is>
           <t>https://www.key4.com/uploads/files/products/xhorse_keydiy_key_blades/KB-UNV-VA6/KB-UNV-VA6-1.jpg</t>
         </is>
@@ -15071,7 +15071,7 @@
           <t>Keydiy / Xhorse VA2 / VA6 #Y-29 Flip Key Blade (검색 결과)</t>
         </is>
       </c>
-      <c r="E418" s="7" t="inlineStr">
+      <c r="E418" s="6" t="inlineStr">
         <is>
           <t>https://keystation.co.uk/citroen-mercedes-peugeot-renault-va2-va6-flip-key-blade</t>
         </is>
@@ -15098,7 +15098,7 @@
           <t>KEYDIY Xhorse VA2 VA6 Flip Blade #58 Peugeot 2002-2021</t>
         </is>
       </c>
-      <c r="E419" s="7" t="inlineStr">
+      <c r="E419" s="6" t="inlineStr">
         <is>
           <t>https://www.dkey1.com/product/keydiy-xhorse-flip-key-blade-va2-va6-58-b-058-for-peugeot-b04076</t>
         </is>
@@ -15125,7 +15125,7 @@
           <t>NE-36 = ERREBI NE72, SILCA NE72 / 차종: AMERICAN MOTORS ® | VARIOUS MODELS | -19- | CITROEN ® | AX |</t>
         </is>
       </c>
-      <c r="E420" s="7" t="inlineStr">
+      <c r="E420" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/ne-36/8613/</t>
         </is>
@@ -15152,7 +15152,7 @@
           <t>Silca NE72 = JMA NE-36, 상품 코드 NE#Y-14</t>
         </is>
       </c>
-      <c r="E421" s="7" t="inlineStr">
+      <c r="E421" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2164&amp;controller=product</t>
         </is>
@@ -15179,7 +15179,7 @@
           <t>NE72 Xhorse KeyDIY Flip Key Blade Replacement #53</t>
         </is>
       </c>
-      <c r="E422" s="7" t="inlineStr">
+      <c r="E422" s="6" t="inlineStr">
         <is>
           <t>https://www.bestkeysupply.com/products/ne72-xhorse-keydiy-universal-flipkey-insert-53-b155bks</t>
         </is>
@@ -15206,7 +15206,7 @@
           <t>NE72, Blank number 53/Y14</t>
         </is>
       </c>
-      <c r="E423" s="7" t="inlineStr">
+      <c r="E423" s="6" t="inlineStr">
         <is>
           <t>https://accessfobs.co.uk/products/blade-for-keydiy-and-xhorse-remote-ne73-ne72</t>
         </is>
@@ -15233,7 +15233,7 @@
           <t>Keydiy / Xhorse NE72 Y-30 / NE73 Y-14 Flip Key Blade (반대 표기)</t>
         </is>
       </c>
-      <c r="E424" s="7" t="inlineStr">
+      <c r="E424" s="6" t="inlineStr">
         <is>
           <t>https://keystation.co.uk/keydiy-xhorse-ne72-y-30-ne73-y-14-flip-key-blade</t>
         </is>
@@ -15260,7 +15260,7 @@
           <t>53# NE72 Key Blade For Peugeot 206 207 Citroen Renault for keydiy KD xhorse VVDI JMD (검색 결과)</t>
         </is>
       </c>
-      <c r="E425" s="7" t="inlineStr">
+      <c r="E425" s="6" t="inlineStr">
         <is>
           <t>https://ledekey.com/collections/universal-key-blade</t>
         </is>
@@ -15287,7 +15287,7 @@
           <t>Keydiy 53 Uncut Metal Blank Car Key Blade, Blade Profile NE72</t>
         </is>
       </c>
-      <c r="E426" s="7" t="inlineStr">
+      <c r="E426" s="6" t="inlineStr">
         <is>
           <t>https://www.tlkeys.com/products/Keydiy-53-Uncut-Metal-Scale-Blank-Car-Key-Blade-Mini-KD90-33125</t>
         </is>
@@ -15314,7 +15314,7 @@
           <t>KEYDIY Remote Flip Key Blade NE72 for Renault (Y-14#)</t>
         </is>
       </c>
-      <c r="E427" s="7" t="inlineStr">
+      <c r="E427" s="6" t="inlineStr">
         <is>
           <t>https://www.locksmithkeyless.com/products/keydiy-remote-flip-key-blade-ne72-for-renault-y-14</t>
         </is>
@@ -15341,7 +15341,7 @@
           <t>Xhorse KeyDIY NE72 Long Blade - AUTKB180 (검색 결과, 번호 미표기)</t>
         </is>
       </c>
-      <c r="E428" s="7" t="inlineStr">
+      <c r="E428" s="6" t="inlineStr">
         <is>
           <t>https://autowave.co.uk/</t>
         </is>
@@ -15368,7 +15368,7 @@
           <t>Grot KEYDIY/XHORSE #Y-30 NE73 - Y-14보다 짧음 (검색 결과)</t>
         </is>
       </c>
-      <c r="E429" s="7" t="inlineStr">
+      <c r="E429" s="6" t="inlineStr">
         <is>
           <t>https://a-d-e.pl/blades-grot-keydiy/xhorse-y-30-ne73,c146,p3970,o1001,s1001,en.html</t>
         </is>
@@ -15380,7 +15380,11 @@
           <t>NE73 (없음)</t>
         </is>
       </c>
-      <c r="B430" s="3" t="inlineStr"/>
+      <c r="B430" s="3" t="inlineStr">
+        <is>
+          <t>Y-30</t>
+        </is>
+      </c>
       <c r="C430" s="3" t="inlineStr">
         <is>
           <t>JMA 공식 전자 카탈로그 등가표</t>
@@ -15391,7 +15395,7 @@
           <t>NE-38 = ERREBI NE79, SILCA NE73 / 차종: RENAULT ® | R 21 | 1992- | RENAULT ® | R 25 | 1992- | RENAUL</t>
         </is>
       </c>
-      <c r="E430" s="7" t="inlineStr">
+      <c r="E430" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/ne-38/8624/</t>
         </is>
@@ -15403,7 +15407,11 @@
           <t>NE73 (없음)</t>
         </is>
       </c>
-      <c r="B431" s="3" t="inlineStr"/>
+      <c r="B431" s="3" t="inlineStr">
+        <is>
+          <t>Y-30</t>
+        </is>
+      </c>
       <c r="C431" s="3" t="inlineStr">
         <is>
           <t>Keyshop Online 50종 키날 묶음 목록</t>
@@ -15414,7 +15422,7 @@
           <t>NE73 - #53 Y-30 - UB10037 (Renault / Dacia)</t>
         </is>
       </c>
-      <c r="E431" s="7" t="inlineStr">
+      <c r="E431" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -15426,7 +15434,11 @@
           <t>NE73 (없음)</t>
         </is>
       </c>
-      <c r="B432" s="3" t="inlineStr"/>
+      <c r="B432" s="3" t="inlineStr">
+        <is>
+          <t>Y-30</t>
+        </is>
+      </c>
       <c r="C432" s="3" t="inlineStr">
         <is>
           <t>Access Fobs (영국)</t>
@@ -15437,7 +15449,7 @@
           <t>NE73 NE-38, Blank number Y30#</t>
         </is>
       </c>
-      <c r="E432" s="7" t="inlineStr">
+      <c r="E432" s="6" t="inlineStr">
         <is>
           <t>https://accessfobs.co.uk/products/blade-for-keydiy-and-xhorse-remote-ne73</t>
         </is>
@@ -15449,7 +15461,11 @@
           <t>NE73 (없음)</t>
         </is>
       </c>
-      <c r="B433" s="3" t="inlineStr"/>
+      <c r="B433" s="3" t="inlineStr">
+        <is>
+          <t>Y-30</t>
+        </is>
+      </c>
       <c r="C433" s="3" t="inlineStr">
         <is>
           <t>Reid's Remotes (호주)</t>
@@ -15460,7 +15476,7 @@
           <t>Silca NE73 = JMA NE-38, 상품 코드 NE#Y-30</t>
         </is>
       </c>
-      <c r="E433" s="7" t="inlineStr">
+      <c r="E433" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2165&amp;controller=product</t>
         </is>
@@ -15472,7 +15488,11 @@
           <t>NE73 (없음)</t>
         </is>
       </c>
-      <c r="B434" s="3" t="inlineStr"/>
+      <c r="B434" s="3" t="inlineStr">
+        <is>
+          <t>Y-30</t>
+        </is>
+      </c>
       <c r="C434" s="3" t="inlineStr">
         <is>
           <t>A-D-E (폴란드)</t>
@@ -15483,7 +15503,7 @@
           <t>Grot KEYDIY/XHORSE #Y-30 NE73</t>
         </is>
       </c>
-      <c r="E434" s="7" t="inlineStr">
+      <c r="E434" s="6" t="inlineStr">
         <is>
           <t>https://a-d-e.pl/blades-grot-keydiy/xhorse-y-30-ne73,c146,p3970,o1001,s1001,en.html</t>
         </is>
@@ -15495,7 +15515,11 @@
           <t>NE73 (없음)</t>
         </is>
       </c>
-      <c r="B435" s="3" t="inlineStr"/>
+      <c r="B435" s="3" t="inlineStr">
+        <is>
+          <t>Y-30</t>
+        </is>
+      </c>
       <c r="C435" s="3" t="inlineStr">
         <is>
           <t>NW Keys</t>
@@ -15506,7 +15530,7 @@
           <t>KDNE73/NE72 KeyDIY &amp; X-Horse blade (Y30)</t>
         </is>
       </c>
-      <c r="E435" s="7" t="inlineStr">
+      <c r="E435" s="6" t="inlineStr">
         <is>
           <t>https://www.nwkeys.co.uk/Product/kdne73-ne72-keydiy-blade</t>
         </is>
@@ -15518,7 +15542,11 @@
           <t>NE73 (없음)</t>
         </is>
       </c>
-      <c r="B436" s="3" t="inlineStr"/>
+      <c r="B436" s="3" t="inlineStr">
+        <is>
+          <t>Y-30</t>
+        </is>
+      </c>
       <c r="C436" s="3" t="inlineStr">
         <is>
           <t>eBay</t>
@@ -15529,7 +15557,7 @@
           <t>10pcs/lot Type 53 NE73 Metal Blank Uncut Flip KEYDIY/VVDI/JMD Remote Key Blade (반대 근거)</t>
         </is>
       </c>
-      <c r="E436" s="7" t="inlineStr">
+      <c r="E436" s="6" t="inlineStr">
         <is>
           <t>https://www.ebay.com/itm/314097440759</t>
         </is>
@@ -15541,7 +15569,11 @@
           <t>NE73 (없음)</t>
         </is>
       </c>
-      <c r="B437" s="3" t="inlineStr"/>
+      <c r="B437" s="3" t="inlineStr">
+        <is>
+          <t>Y-30</t>
+        </is>
+      </c>
       <c r="C437" s="3" t="inlineStr">
         <is>
           <t>Keylocksupplies (Sunrise)</t>
@@ -15552,7 +15584,7 @@
           <t>Y-14# Renault NE73 / Xhorse / Keydiy Blade (반대 근거)</t>
         </is>
       </c>
-      <c r="E437" s="7" t="inlineStr">
+      <c r="E437" s="6" t="inlineStr">
         <is>
           <t>https://www.keylocksupplies.com/collections/keydiy-blade</t>
         </is>
@@ -15564,7 +15596,11 @@
           <t>NE73 (없음)</t>
         </is>
       </c>
-      <c r="B438" s="3" t="inlineStr"/>
+      <c r="B438" s="3" t="inlineStr">
+        <is>
+          <t>Y-30</t>
+        </is>
+      </c>
       <c r="C438" s="3" t="inlineStr">
         <is>
           <t>MK3</t>
@@ -15575,7 +15611,7 @@
           <t>Keydiy KD Xhorse VVDI Universal Flip Remote key Blade For REN NE72 / NE73, Part Number 53 (반대 근거)</t>
         </is>
       </c>
-      <c r="E438" s="7" t="inlineStr">
+      <c r="E438" s="6" t="inlineStr">
         <is>
           <t>https://www.mk3.com/en/kd-universal-flip-remote-key-blade-ren-ne73</t>
         </is>
@@ -15602,7 +15638,7 @@
           <t>SIX-3P = ERREBI SM7P68, SM7P68, SILCA SX11BP, SX9AP / 차종: AIXAM ® | 500-4 | -19- | AIXAM ® | COUPE | 2008- | AIXAM ® |</t>
         </is>
       </c>
-      <c r="E439" s="7" t="inlineStr">
+      <c r="E439" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/six-3p/10512/</t>
         </is>
@@ -15629,7 +15665,7 @@
           <t>SX9 - #83 - UB10022 (PSA)</t>
         </is>
       </c>
-      <c r="E440" s="7" t="inlineStr">
+      <c r="E440" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -15656,7 +15692,7 @@
           <t>Silca SX9 = JMA SIX-3, 상품 코드 CIT#84</t>
         </is>
       </c>
-      <c r="E441" s="7" t="inlineStr">
+      <c r="E441" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2172&amp;controller=product</t>
         </is>
@@ -15683,7 +15719,7 @@
           <t>SX9 For Citroen, Fiat, Lancia, Peugeot, Blank number #83</t>
         </is>
       </c>
-      <c r="E442" s="7" t="inlineStr">
+      <c r="E442" s="6" t="inlineStr">
         <is>
           <t>https://accessfobs.co.uk/products/blade-for-keydiy-and-xhorse-remote-sx9</t>
         </is>
@@ -15710,7 +15746,7 @@
           <t>SX9 (2 sides) For Citroen, Fiat &amp; Peugeot, Blank number 84#</t>
         </is>
       </c>
-      <c r="E443" s="7" t="inlineStr">
+      <c r="E443" s="6" t="inlineStr">
         <is>
           <t>https://accessfobs.co.uk/products/blade-for-keydiy-xhorse-sx9-copy</t>
         </is>
@@ -15737,7 +15773,7 @@
           <t>Keydiy / Xhorse SX9 #84 Key Blade 2 Sides</t>
         </is>
       </c>
-      <c r="E444" s="7" t="inlineStr">
+      <c r="E444" s="6" t="inlineStr">
         <is>
           <t>https://keystation.co.uk/keydiy-xhorse-sx9-84-key-blade-2-sides</t>
         </is>
@@ -15764,7 +15800,7 @@
           <t>3D Group DIYB40: SX9 #83 단면, 양면은 #84 (검색 결과)</t>
         </is>
       </c>
-      <c r="E445" s="7" t="inlineStr">
+      <c r="E445" s="6" t="inlineStr">
         <is>
           <t>https://3dgroupuk.com/product/view/DIYB40</t>
         </is>
@@ -15791,7 +15827,7 @@
           <t>Flip Key Blade - CITROEN (Like: SX9) - Double Sided (#84, 검색 결과)</t>
         </is>
       </c>
-      <c r="E446" s="7" t="inlineStr">
+      <c r="E446" s="6" t="inlineStr">
         <is>
           <t>https://www.sglocks.com.au/product/15675-flip-key-blade-citroen-like-sx9-double-sided</t>
         </is>
@@ -15818,7 +15854,7 @@
           <t>VA-34P = ERREBI VC82P49, SILCA VAC102DP / 차종: DACIA ® | DUSTER | 2010-2013 | DACIA ® | LOGAN | 2004-2012 |</t>
         </is>
       </c>
-      <c r="E447" s="7" t="inlineStr">
+      <c r="E447" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/va-34p/13333/</t>
         </is>
@@ -15845,7 +15881,7 @@
           <t>VAC102 - #152 - UB10025 (Renault / Dacia)</t>
         </is>
       </c>
-      <c r="E448" s="7" t="inlineStr">
+      <c r="E448" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -15872,7 +15908,7 @@
           <t>Silca VAC102 = JMA VA-34, 상품 코드 NE#152</t>
         </is>
       </c>
-      <c r="E449" s="7" t="inlineStr">
+      <c r="E449" s="6" t="inlineStr">
         <is>
           <t>https://www.reidsremotes.com.au/index.php?id_product=2179&amp;controller=product</t>
         </is>
@@ -15899,7 +15935,7 @@
           <t>DAC-4DC1 = ERREBI DCA4RC1, SILCA HU136TA / 차종: DACIA ® | DOKKER | 2012-2016 | DACIA ® | LODGY | 2012-2016 |</t>
         </is>
       </c>
-      <c r="E450" s="7" t="inlineStr">
+      <c r="E450" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/dac-4dc1/3275/</t>
         </is>
@@ -15926,7 +15962,7 @@
           <t>HU136 - #153 Y-54 - UB10061 (Renault / Dacia)</t>
         </is>
       </c>
-      <c r="E451" s="7" t="inlineStr">
+      <c r="E451" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -15953,7 +15989,7 @@
           <t>Renault HU136 Replacement Flip Blade 109 Stamp (검색 결과 요약)</t>
         </is>
       </c>
-      <c r="E452" s="7" t="inlineStr">
+      <c r="E452" s="6" t="inlineStr">
         <is>
           <t>https://www.americankeysupply.com/category/xhorse-keydiy-blades-488</t>
         </is>
@@ -15980,7 +16016,7 @@
           <t>KeyDiy KD 153 Blank Key Remote Blade for Lada Renault Megane, Blade Profile HU136</t>
         </is>
       </c>
-      <c r="E453" s="7" t="inlineStr">
+      <c r="E453" s="6" t="inlineStr">
         <is>
           <t>https://www.tlkeys.com/products/KeyDiy-KD-153-Blank-Key-Remote-Blade-for-Lada-Renault-Megan-33146</t>
         </is>
@@ -16007,7 +16043,7 @@
           <t>10pcs 153# 153 HU136 Metal Uncut Blank Flip Remote Key Blade For Renault Megan Dacia Clio Duster</t>
         </is>
       </c>
-      <c r="E454" s="7" t="inlineStr">
+      <c r="E454" s="6" t="inlineStr">
         <is>
           <t>https://www.aliexpress.us/item/3256803028755224.html</t>
         </is>
@@ -16034,7 +16070,7 @@
           <t>KDIY key Blade 153# HU136 for renault</t>
         </is>
       </c>
-      <c r="E455" s="7" t="inlineStr">
+      <c r="E455" s="6" t="inlineStr">
         <is>
           <t>https://chipkeysupply.com/products/153-metal-kd-jmd-vvdi-remote-car-key-blade-for-renault</t>
         </is>
@@ -16107,7 +16143,7 @@
           <t xml:space="preserve">FI-13 = ERREBI GB14R, SILCA GT15R / 차종: ALFA ROMEO ® | 155 6V | 1992-1995 | ALFA ROMEO ® | 155 T.S. </t>
         </is>
       </c>
-      <c r="E458" s="7" t="inlineStr">
+      <c r="E458" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/fi-13/4426/</t>
         </is>
@@ -16134,7 +16170,7 @@
           <t>GT15 Xhorse KeyDIY Flip Key Blade Replacement #60</t>
         </is>
       </c>
-      <c r="E459" s="7" t="inlineStr">
+      <c r="E459" s="6" t="inlineStr">
         <is>
           <t>https://www.bestkeysupply.com/products/gt15-xhorse-keydiy-universal-flipkey-insert-60-b158bks</t>
         </is>
@@ -16161,7 +16197,7 @@
           <t>KD Fiat Flip Remote Key Blade GT15R 60 (검색 결과)</t>
         </is>
       </c>
-      <c r="E460" s="7" t="inlineStr">
+      <c r="E460" s="6" t="inlineStr">
         <is>
           <t>https://www.mk3.com/en/kd-fiat-flip-remote-key-blade-gt15r-60</t>
         </is>
@@ -16188,7 +16224,7 @@
           <t>Fiat Keydiy GT15 Flip Keyblade - Blade60</t>
         </is>
       </c>
-      <c r="E461" s="7" t="inlineStr">
+      <c r="E461" s="6" t="inlineStr">
         <is>
           <t>https://remkeys.com/product/fiat-keydiy-gt15-flip-keyblade-blade60-ftkb05-remkeys/</t>
         </is>
@@ -16215,7 +16251,7 @@
           <t>VD9548-Universal Flip Remote key Blade Fiat GT15R, Part Number 60 (검색 결과)</t>
         </is>
       </c>
-      <c r="E462" s="7" t="inlineStr">
+      <c r="E462" s="6" t="inlineStr">
         <is>
           <t>https://www.vvdi.com/kd900-blade-for-fiat-flip-remote-key-gt15r</t>
         </is>
@@ -16242,7 +16278,7 @@
           <t>Fiat GT15R Flip Key Blades for Xhorse Remotes (GTL), GTL-RK-KD-060</t>
         </is>
       </c>
-      <c r="E463" s="7" t="inlineStr">
+      <c r="E463" s="6" t="inlineStr">
         <is>
           <t>https://www.americankeysupply.com/product/fiat-gt15r-flip-key-blades-for-xhorse-remotes-gtl-10562</t>
         </is>
@@ -16269,7 +16305,7 @@
           <t>NE-40 = SILCA NE66 / 차종: VOLVO ® | 760 | 1991- | VOLVO ® | 762 | 1991- | VOLVO ® | 76</t>
         </is>
       </c>
-      <c r="E464" s="7" t="inlineStr">
+      <c r="E464" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/ne-40/8642/</t>
         </is>
@@ -16296,7 +16332,7 @@
           <t>NE-40P = ERREBI NE70P70, ILCO S66NNP, SILCA NE66P / 차종: VOLVO ® | 760 | 1991- | VOLVO ® | 762 | 1991- | VOLVO ® | 76</t>
         </is>
       </c>
-      <c r="E465" s="7" t="inlineStr">
+      <c r="E465" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/ne-40p/8644/</t>
         </is>
@@ -16323,7 +16359,7 @@
           <t>NE66 Xhorse KeyDIY Flip Key Blade Replacement #24</t>
         </is>
       </c>
-      <c r="E466" s="7" t="inlineStr">
+      <c r="E466" s="6" t="inlineStr">
         <is>
           <t>https://www.bestkeysupply.com/products/ne66-xhorse-keydiy-universal-flipkey-insert-24-b145bks</t>
         </is>
@@ -16350,7 +16386,7 @@
           <t>Keyless2Go Volvo NE66 Blade 24# for Xhorse KeyDIY Universal Remotes</t>
         </is>
       </c>
-      <c r="E467" s="7" t="inlineStr">
+      <c r="E467" s="6" t="inlineStr">
         <is>
           <t>https://keyinnovations.com/products/keyless2go-volvo-ne66-blade-24-for-xhorse-keydiy-universal-remotes</t>
         </is>
@@ -16377,7 +16413,7 @@
           <t>Xhorse Keydiy Key Blade Volvo NE66 (#24) Pack Of 5</t>
         </is>
       </c>
-      <c r="E468" s="7" t="inlineStr">
+      <c r="E468" s="6" t="inlineStr">
         <is>
           <t>https://keys4less.net/product/xhorse-keydiy-key-blade-volvo-ne66-24-pack-of-5</t>
         </is>
@@ -16404,7 +16440,7 @@
           <t>NE-40 NE66 TOY49 KI-7 - KIA7, 24#</t>
         </is>
       </c>
-      <c r="E469" s="7" t="inlineStr">
+      <c r="E469" s="6" t="inlineStr">
         <is>
           <t>https://accessfobs.co.uk/products/blade-for-keydiy-xhorse-key-blade-ne66-toy49-for-volvo-hyundai-kia-toyota</t>
         </is>
@@ -16431,7 +16467,7 @@
           <t>HU-DHP = ERREBI HF49P62, ILCO S60HFP, SILCA HU56RP / 차종: VOLVO ® | 440 | 1987- | VOLVO ® | 460 | 1987- | VOLVO ® | 48</t>
         </is>
       </c>
-      <c r="E470" s="7" t="inlineStr">
+      <c r="E470" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/hu-dhp/5759/</t>
         </is>
@@ -16458,7 +16494,7 @@
           <t>HU56 - #183 Y-70 - UB10045 (Volvo)</t>
         </is>
       </c>
-      <c r="E471" s="7" t="inlineStr">
+      <c r="E471" s="6" t="inlineStr">
         <is>
           <t>https://keyshop-online.com/products/eu-labeled-blade-box-kit-keydiy-xhorse-universal-flip-blades-220-keys-44-types</t>
         </is>
@@ -16485,7 +16521,7 @@
           <t>Blade for KEYDIY and Xhorse Remote - HU56R (Y70#)</t>
         </is>
       </c>
-      <c r="E472" s="7" t="inlineStr">
+      <c r="E472" s="6" t="inlineStr">
         <is>
           <t>https://accessfobs.co.uk/products/hu56-flip-key-blade-xhorse-key-diy</t>
         </is>
@@ -16512,7 +16548,7 @@
           <t>KD HU56 HU56R Y70 Key Blade for Volvo Mitsubishi S40</t>
         </is>
       </c>
-      <c r="E473" s="7" t="inlineStr">
+      <c r="E473" s="6" t="inlineStr">
         <is>
           <t>https://www.ebay.com/itm/155502528670</t>
         </is>
@@ -16539,7 +16575,7 @@
           <t>10pcs/lot Metal Car Flip Key Blank HU56 KD Flip Key Blade 183# HU56R for Volvo</t>
         </is>
       </c>
-      <c r="E474" s="7" t="inlineStr">
+      <c r="E474" s="6" t="inlineStr">
         <is>
           <t>https://www.aliexpress.us/item/3256804526671687.html</t>
         </is>
@@ -16566,7 +16602,7 @@
           <t>HU-DNP = ERREBI HF62RP157, SILCA HU57RP / 차종: VOLVO ® | 440 | 1987- | VOLVO ® | 460 | 1987- | VOLVO ® | 48</t>
         </is>
       </c>
-      <c r="E475" s="7" t="inlineStr">
+      <c r="E475" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/hu-dnp/5763/</t>
         </is>
@@ -16593,7 +16629,7 @@
           <t>KeyDIY Volvo Universal Flip Key Blade, HU57 (56#)</t>
         </is>
       </c>
-      <c r="E476" s="7" t="inlineStr">
+      <c r="E476" s="6" t="inlineStr">
         <is>
           <t>https://keyinnovations.com/volvo-byd-blade-56-hu57/</t>
         </is>
@@ -16620,7 +16656,7 @@
           <t>Volvo Keydiy HU57 Flip Keyblade - Blade56 - BYD-R (사진 각인 56)</t>
         </is>
       </c>
-      <c r="E477" s="7" t="inlineStr">
+      <c r="E477" s="6" t="inlineStr">
         <is>
           <t>https://remkeys.com/product/volvo-keydiy-hu57-flip-keyblade-blade56-byd-r-vlkb06-remkeys/</t>
         </is>
@@ -16647,7 +16683,7 @@
           <t>Volvo Keydiy HU57L Flip Keyblade - Blade57 - BYD-L (사진 각인 57, 왼쪽 홈)</t>
         </is>
       </c>
-      <c r="E478" s="7" t="inlineStr">
+      <c r="E478" s="6" t="inlineStr">
         <is>
           <t>https://remkeys.com/product/volvo-keydiy-hu57l-flip-keyblade-blade57-byd-l-vlkb07-remkeys/</t>
         </is>
@@ -16674,7 +16710,7 @@
           <t>Keydiy/Xhorse HU57 #56 Flip Blade for Volvo (검색 결과)</t>
         </is>
       </c>
-      <c r="E479" s="7" t="inlineStr">
+      <c r="E479" s="6" t="inlineStr">
         <is>
           <t>https://keystation.co.uk/vehicle-makes/volvo-car-keys-parts/volvo-car-key-blades</t>
         </is>
@@ -16701,7 +16737,7 @@
           <t>Keydiy #56 Volvo BYD Key Blade, profile HU57</t>
         </is>
       </c>
-      <c r="E480" s="7" t="inlineStr">
+      <c r="E480" s="6" t="inlineStr">
         <is>
           <t>https://www.tlkeys.com/products/Keydiy-56-Volvo-BYD-Key-Blade-33302</t>
         </is>
@@ -16728,7 +16764,7 @@
           <t>VD9539-Universal Flip Remote key Blade BYD HU57, part number 56 (검색 결과)</t>
         </is>
       </c>
-      <c r="E481" s="7" t="inlineStr">
+      <c r="E481" s="6" t="inlineStr">
         <is>
           <t>https://www.vvdi.com/kd900-blade-for-flip-remote-key-byd-56</t>
         </is>
@@ -16755,7 +16791,7 @@
           <t xml:space="preserve">FI-11 = ERREBI GB9R, SILCA GT10 / 차종: APRILIA ® | RED ROSE 50 | 1990-1991 | AUTOBIANCHI ® | Y10 | </t>
         </is>
       </c>
-      <c r="E482" s="7" t="inlineStr">
+      <c r="E482" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/fi-11/4416/</t>
         </is>
@@ -16782,7 +16818,7 @@
           <t>Silca GT10 = Ilco NE57</t>
         </is>
       </c>
-      <c r="E483" s="7" t="inlineStr">
+      <c r="E483" s="6" t="inlineStr">
         <is>
           <t>https://www.key4.com/uploads/files/products/metal_keys/AC-ILC-KEYDIR13/Key_Blank_Directory_-_Edition_13.pdf</t>
         </is>
@@ -16809,7 +16845,7 @@
           <t>GT10 IVECO, Blank number 147#</t>
         </is>
       </c>
-      <c r="E484" s="7" t="inlineStr">
+      <c r="E484" s="6" t="inlineStr">
         <is>
           <t>https://accessfobs.co.uk/products/blade-for-keydiy-xhorse-remote-gt10-iveco</t>
         </is>
@@ -16836,7 +16872,7 @@
           <t>Keydiy / Xhorse GT10 #147 Flip key Blade For Citroen, Fiat, Iveco &amp; Peugeot (검색 결과)</t>
         </is>
       </c>
-      <c r="E485" s="7" t="inlineStr">
+      <c r="E485" s="6" t="inlineStr">
         <is>
           <t>https://keystation.co.uk/vehicle-makes/fiat-car-keys-parts/fiat-car-key-blades</t>
         </is>
@@ -16863,7 +16899,7 @@
           <t>#147 Key Blade for Iveco GT10 - Pack of 10</t>
         </is>
       </c>
-      <c r="E486" s="7" t="inlineStr">
+      <c r="E486" s="6" t="inlineStr">
         <is>
           <t>https://m.norman-keys.com/147-key-blade-for-iveco-gt10-pack-of-10</t>
         </is>
@@ -16890,7 +16926,7 @@
           <t>10pcs/lot #147 GT10 Metal Blank Uncut Flip for KD / XHORSE Remote Key Blade For IVECO</t>
         </is>
       </c>
-      <c r="E487" s="7" t="inlineStr">
+      <c r="E487" s="6" t="inlineStr">
         <is>
           <t>https://www.fvdiobd.com/147-key-blade-for-iveco-for-kd-key.html</t>
         </is>
@@ -16913,7 +16949,7 @@
           <t>ISU-5 = ERREBI ISU8, EZ B113, ILCO X275, SILCA ISU5 / 차종: GMC ® | TILTMASTER W7 | 2008-2011 | ISUZU ® | NPR | 2005-200</t>
         </is>
       </c>
-      <c r="E488" s="7" t="inlineStr">
+      <c r="E488" s="6" t="inlineStr">
         <is>
           <t>https://ecatalogo.jma.es/en/isu-5/6097/</t>
         </is>
@@ -16936,7 +16972,7 @@
           <t>KeyDiy Xhorse Remote Key Blade For Isuzu ISU5</t>
         </is>
       </c>
-      <c r="E489" s="7" t="inlineStr">
+      <c r="E489" s="6" t="inlineStr">
         <is>
           <t>https://abkeys.com/products/isuzu-remote-key-blade-isu5-47</t>
         </is>
@@ -16959,7 +16995,7 @@
           <t>KeyDiy Xhorse Remote Key Blade For Isuzu ISU5 (ABK-47), 사진 각인 79</t>
         </is>
       </c>
-      <c r="E490" s="7" t="inlineStr">
+      <c r="E490" s="6" t="inlineStr">
         <is>
           <t>https://abkeys.com/products/isuzu-remote-key-blade-isu5-47</t>
         </is>
@@ -18149,7 +18185,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>확인 = KEYDIY 번호가 판매처 3곳 이상(또는 해당 없음) / 일부 확인 = KEYDIY 번호를 3곳 이상에서 확인 못 해 비워 둠 / 확인 필요 = 키웨이 이름(ILCO·SILCA·JMA) 자체가 출처끼리 엇갈림</t>
+          <t>확인 = KEYDIY 번호가 판매처 3곳 이상(또는 해당 없음) / 일부 확인 = KEYDIY 번호를 3곳 이상에서 확인 못 해 비워 둠, 또는 판매처끼리 갈려 추정으로 적음(비고 맨 앞 [추정]) / 확인 필요 = 키웨이 이름(ILCO·SILCA·JMA) 자체가 출처끼리 엇갈림</t>
         </is>
       </c>
     </row>

</xml_diff>